<commit_message>
feat: Add remove mode improvements, menu button redesign & release plan
</commit_message>
<xml_diff>
--- a/aquasphere/Excel_File/AquaSphare.xlsx
+++ b/aquasphere/Excel_File/AquaSphare.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\43680\Desktop\Schule\SYP\Aquarium\Excel_File\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\43680\Desktop\Schule\SYP\Aquarium\aquasphere\Excel_File\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F25D955D-2FB8-4336-BFD9-48DE34521E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{470DDF49-15FE-4ABF-AF84-A7B4435C02B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
   </bookViews>
@@ -17,7 +17,8 @@
     <sheet name="Sprint1" sheetId="3" r:id="rId2"/>
     <sheet name="Sprint2" sheetId="4" r:id="rId3"/>
     <sheet name="Sprint3" sheetId="5" r:id="rId4"/>
-    <sheet name="Storys" sheetId="1" r:id="rId5"/>
+    <sheet name="Sprint4" sheetId="6" r:id="rId5"/>
+    <sheet name="Storys" sheetId="1" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="156">
   <si>
     <t>Story ID</t>
   </si>
@@ -512,6 +513,24 @@
   </si>
   <si>
     <t>Als Nutzer möchte ich Steine und Korallen platzieren. Unterschiedliche Pflanzen sollen zur auswahl steten</t>
+  </si>
+  <si>
+    <t>AQ20</t>
+  </si>
+  <si>
+    <t>Cloud/Sync</t>
+  </si>
+  <si>
+    <t>Als Nutzer möchte ich mich auf individuellen geräten einloggen und MEIN Aquarium haben und bearbeiten</t>
+  </si>
+  <si>
+    <t>Coudsync</t>
+  </si>
+  <si>
+    <t>Die Nutzeroberfläche soll Userfrendly sein, Klar, deutlich, Kurze wege</t>
+  </si>
+  <si>
+    <t>Als Nutzer möchte ich Mein Aquarium auf verschiedenen geräten sehen</t>
   </si>
 </sst>
 </file>
@@ -679,152 +698,15 @@
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="84">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF0F9ED5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
+  <dxfs count="106">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
         <name val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -833,243 +715,9 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor theme="7"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF0F9ED5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -1622,15 +1270,15 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1727,6 +1375,788 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
         <family val="2"/>
@@ -1971,26 +2401,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.89999084444715716"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="16"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -2158,25 +2568,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AAF41172-5838-4CA9-A8A2-78B1E57ACF1F}" name="Tabelle1" displayName="Tabelle1" ref="A1:H8" totalsRowShown="0" headerRowDxfId="83" dataDxfId="82">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AAF41172-5838-4CA9-A8A2-78B1E57ACF1F}" name="Tabelle1" displayName="Tabelle1" ref="A1:H8" totalsRowShown="0" headerRowDxfId="105" dataDxfId="104">
   <autoFilter ref="A1:H8" xr:uid="{AAF41172-5838-4CA9-A8A2-78B1E57ACF1F}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{8BB8E342-544E-430C-A72A-9EBF9676D447}" name="Sprint" dataDxfId="81"/>
-    <tableColumn id="9" xr3:uid="{96A939A8-DA63-4E70-B123-D31A897D4192}" name="Story ID" dataDxfId="80"/>
-    <tableColumn id="2" xr3:uid="{CB307D23-EE39-436B-9E06-9E7789362DB6}" name="Estimated Hours" dataDxfId="79">
+    <tableColumn id="1" xr3:uid="{8BB8E342-544E-430C-A72A-9EBF9676D447}" name="Sprint" dataDxfId="103"/>
+    <tableColumn id="9" xr3:uid="{96A939A8-DA63-4E70-B123-D31A897D4192}" name="Story ID" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{CB307D23-EE39-436B-9E06-9E7789362DB6}" name="Estimated Hours" dataDxfId="101">
       <calculatedColumnFormula array="1">Tabelle3[Estimated time]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{5EFC7DEC-DFDE-454B-90FC-2713EB4181D8}" name="Actual Hours" dataDxfId="78">
+    <tableColumn id="3" xr3:uid="{5EFC7DEC-DFDE-454B-90FC-2713EB4181D8}" name="Actual Hours" dataDxfId="100">
       <calculatedColumnFormula array="1">Tabelle3[Actual time]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D6FF0659-1B35-4F09-B5A7-D22FEF5F7C3F}" name="Accomplished Story Points" dataDxfId="77">
+    <tableColumn id="4" xr3:uid="{D6FF0659-1B35-4F09-B5A7-D22FEF5F7C3F}" name="Accomplished Story Points" dataDxfId="99">
       <calculatedColumnFormula array="1">Tabelle4[[Total Storypoints ]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{9CD2DBE3-2E45-4440-8D7A-2A03A0291AAD}" name="Velocity" dataDxfId="76">
+    <tableColumn id="5" xr3:uid="{9CD2DBE3-2E45-4440-8D7A-2A03A0291AAD}" name="Velocity" dataDxfId="0">
       <calculatedColumnFormula>IFERROR(Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{1977DF7A-0A05-43B5-99D3-B72159480780}" name="Total Storypoints" dataDxfId="75"/>
-    <tableColumn id="7" xr3:uid="{D8A5F5FE-B9BC-448A-A9E7-3D00888AE639}" name="Storypoints Left" dataDxfId="74">
+    <tableColumn id="6" xr3:uid="{1977DF7A-0A05-43B5-99D3-B72159480780}" name="Total Storypoints" dataDxfId="98"/>
+    <tableColumn id="7" xr3:uid="{D8A5F5FE-B9BC-448A-A9E7-3D00888AE639}" name="Storypoints Left" dataDxfId="97">
       <calculatedColumnFormula>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2185,13 +2595,13 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0134C802-458D-4153-B0D4-D8B08E02E26A}" name="Tabelle4912" displayName="Tabelle4912" ref="E16:F17" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0134C802-458D-4153-B0D4-D8B08E02E26A}" name="Tabelle4912" displayName="Tabelle4912" ref="E16:F17" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="E16:F17" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C3438C75-AD69-46E0-B1BD-0445ED469483}" name="Total Storypoints " dataDxfId="1">
+    <tableColumn id="1" xr3:uid="{C3438C75-AD69-46E0-B1BD-0445ED469483}" name="Total Storypoints " dataDxfId="33">
       <calculatedColumnFormula>SUM(Tabelle2710[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0655740B-E1AB-4BD3-B7CA-852D4C79FC17}" name="Effort/Hour" dataDxfId="0">
+    <tableColumn id="2" xr3:uid="{0655740B-E1AB-4BD3-B7CA-852D4C79FC17}" name="Effort/Hour" dataDxfId="32">
       <calculatedColumnFormula>Tabelle4912[[#This Row],[Total Storypoints ]]/Tabelle3811[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2200,51 +2610,104 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:G27" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}" name="Tabelle271013" displayName="Tabelle271013" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+  <autoFilter ref="A1:K11" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{946A4B14-799A-49AD-8E3E-31E3F4BBE559}" name="Sprint Start" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{E61A962F-4EE4-4843-AF21-C647918EECAB}" name="Sprint End" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{4EC50B40-18BD-4D00-8BE2-5596A9347BB8}" name="User" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{2A1F175E-D14E-491C-B452-39567CF84CD6}" name="ID" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{DCE5121F-D243-470B-B0AF-D0EE5264DD5A}" name="Epic" dataDxfId="16"/>
+    <tableColumn id="12" xr3:uid="{45FDCCAE-F13D-47C1-B91E-2EF3CC9A5BA0}" name="User Story /Task" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{4057DF12-8977-4284-BF2B-9ED3AAE7221F}" name="Estimated time" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{08443A2E-5832-4299-8009-1F0D489DEE15}" name="COS (Criteria of Satisfaction)" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{8777A429-C11B-4CDC-BB2F-785D0BC89DAB}" name="Story points" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{0B18443F-D8D9-4015-8EAA-7050016E43C2}" name="Time in Hours" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{5C5B5C91-6376-4597-B69B-4D162307C569}" name="Status" dataDxfId="10"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}" name="Tabelle381114" displayName="Tabelle381114" ref="A15:C16" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A15:C16" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{E71994D0-AB06-482B-8487-03AB7E3B1FF7}" name="Estimated time" dataDxfId="7">
+      <calculatedColumnFormula>SUM(Tabelle271013[Estimated time])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{E607785B-5B58-4D1E-81ED-45AAAAF488F0}" name="Actual time" dataDxfId="6">
+      <calculatedColumnFormula>SUM(Tabelle271013[Time in Hours])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{0197CFBA-597E-49C6-88E5-ABAC17763EA4}" name="Delta" dataDxfId="5">
+      <calculatedColumnFormula>Tabelle381114[[#This Row],[Estimated time]]-Tabelle381114[[#This Row],[Actual time]]</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}" name="Tabelle491215" displayName="Tabelle491215" ref="E15:F16" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="E15:F16" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{E0381C51-E5FF-4087-9146-76E105FE701A}" name="Total Storypoints " dataDxfId="2">
+      <calculatedColumnFormula>SUM(Tabelle271013[Story points])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{0971B46C-CFAA-4F13-88AB-CDC5655C1F84}" name="Effort/Hour" dataDxfId="1">
+      <calculatedColumnFormula>Tabelle491215[[#This Row],[Total Storypoints ]]/Tabelle381114[[#This Row],[Actual time]]</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:G27" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
   <autoFilter ref="A1:G27" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="50"/>
-    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="49"/>
-    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="48"/>
-    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Effort" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="46"/>
-    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="45"/>
-    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="44"/>
+    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Effort" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}" name="Tabelle2" displayName="Tabelle2" ref="A1:J9" insertRowShift="1" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}" name="Tabelle2" displayName="Tabelle2" ref="A1:J9" insertRowShift="1" totalsRowShown="0" headerRowDxfId="96" dataDxfId="95">
   <autoFilter ref="A1:J9" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{0351E8C1-0BB8-4C19-A406-233CC12328E5}" name="Sprint Start" dataDxfId="71"/>
-    <tableColumn id="2" xr3:uid="{51BD2FE0-507A-4398-BD96-E186E78BB2C7}" name="Sprint End" dataDxfId="70"/>
-    <tableColumn id="3" xr3:uid="{A3B7E86B-E01A-4D78-82AD-BA81F6AC7ADF}" name="User" dataDxfId="69"/>
-    <tableColumn id="5" xr3:uid="{CE780601-F45C-4063-B216-98ACE5588903}" name="ID" dataDxfId="68"/>
-    <tableColumn id="6" xr3:uid="{A14D049D-AC5C-49A5-A7CC-A4D5ED8A8330}" name="Epic" dataDxfId="67"/>
-    <tableColumn id="12" xr3:uid="{770F10A6-830A-41AC-B069-6267CAE00BDF}" name="User Story /Task" dataDxfId="66"/>
-    <tableColumn id="11" xr3:uid="{0D9AB552-F7B4-4231-A35B-245B57383919}" name="Estimated time" dataDxfId="65"/>
-    <tableColumn id="8" xr3:uid="{3E2E3644-9002-4AB9-B3EC-96FFF84D8900}" name="COS (Criteria of Satisfaction)" dataDxfId="64"/>
-    <tableColumn id="9" xr3:uid="{14C8E3A9-BC37-48D9-A399-32A48A46993A}" name="Story points" dataDxfId="63"/>
-    <tableColumn id="10" xr3:uid="{151786D9-5F15-42D7-932B-664A024F4131}" name="Time in Hours" dataDxfId="62"/>
+    <tableColumn id="1" xr3:uid="{0351E8C1-0BB8-4C19-A406-233CC12328E5}" name="Sprint Start" dataDxfId="94"/>
+    <tableColumn id="2" xr3:uid="{51BD2FE0-507A-4398-BD96-E186E78BB2C7}" name="Sprint End" dataDxfId="93"/>
+    <tableColumn id="3" xr3:uid="{A3B7E86B-E01A-4D78-82AD-BA81F6AC7ADF}" name="User" dataDxfId="92"/>
+    <tableColumn id="5" xr3:uid="{CE780601-F45C-4063-B216-98ACE5588903}" name="ID" dataDxfId="91"/>
+    <tableColumn id="6" xr3:uid="{A14D049D-AC5C-49A5-A7CC-A4D5ED8A8330}" name="Epic" dataDxfId="90"/>
+    <tableColumn id="12" xr3:uid="{770F10A6-830A-41AC-B069-6267CAE00BDF}" name="User Story /Task" dataDxfId="89"/>
+    <tableColumn id="11" xr3:uid="{0D9AB552-F7B4-4231-A35B-245B57383919}" name="Estimated time" dataDxfId="88"/>
+    <tableColumn id="8" xr3:uid="{3E2E3644-9002-4AB9-B3EC-96FFF84D8900}" name="COS (Criteria of Satisfaction)" dataDxfId="87"/>
+    <tableColumn id="9" xr3:uid="{14C8E3A9-BC37-48D9-A399-32A48A46993A}" name="Story points" dataDxfId="86"/>
+    <tableColumn id="10" xr3:uid="{151786D9-5F15-42D7-932B-664A024F4131}" name="Time in Hours" dataDxfId="85"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}" name="Tabelle3" displayName="Tabelle3" ref="A15:C16" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}" name="Tabelle3" displayName="Tabelle3" ref="A15:C16" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
   <autoFilter ref="A15:C16" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CD2D4D96-DD34-4EA3-92D7-B02BB9DE5647}" name="Estimated time" dataDxfId="59">
+    <tableColumn id="1" xr3:uid="{CD2D4D96-DD34-4EA3-92D7-B02BB9DE5647}" name="Estimated time" dataDxfId="82">
       <calculatedColumnFormula>SUM(Tabelle2[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0F14E190-6E0A-4AB8-8ADE-83875E98D4B5}" name="Actual time" dataDxfId="58">
+    <tableColumn id="2" xr3:uid="{0F14E190-6E0A-4AB8-8ADE-83875E98D4B5}" name="Actual time" dataDxfId="81">
       <calculatedColumnFormula>SUM(Tabelle2[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{5DE18543-F4D3-4732-9F2D-5B7F140CB974}" name="Delta" dataDxfId="57">
+    <tableColumn id="3" xr3:uid="{5DE18543-F4D3-4732-9F2D-5B7F140CB974}" name="Delta" dataDxfId="80">
       <calculatedColumnFormula>Tabelle3[[#This Row],[Estimated time]]-Tabelle3[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2253,13 +2716,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}" name="Tabelle4" displayName="Tabelle4" ref="E15:F16" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}" name="Tabelle4" displayName="Tabelle4" ref="E15:F16" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
   <autoFilter ref="E15:F16" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{2E187AEA-682F-4749-9FC8-ED3BA3DE1DA2}" name="Total Storypoints " dataDxfId="54">
+    <tableColumn id="1" xr3:uid="{2E187AEA-682F-4749-9FC8-ED3BA3DE1DA2}" name="Total Storypoints " dataDxfId="77">
       <calculatedColumnFormula>SUM(Tabelle2[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3C6DC8F5-724A-43AC-9128-7661A96380C1}" name="Efford/Hour" dataDxfId="53">
+    <tableColumn id="2" xr3:uid="{3C6DC8F5-724A-43AC-9128-7661A96380C1}" name="Efford/Hour" dataDxfId="76">
       <calculatedColumnFormula>Tabelle4[[#This Row],[Total Storypoints ]]/Tabelle3[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2268,36 +2731,36 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A211D33B-248F-4E66-AF7C-9632EAA38DAC}" name="Tabelle27" displayName="Tabelle27" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A211D33B-248F-4E66-AF7C-9632EAA38DAC}" name="Tabelle27" displayName="Tabelle27" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
   <autoFilter ref="A1:K12" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{9C36A560-9153-4D8E-BA50-0044E74E1896}" name="Sprint Start" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{4FAB3106-8621-41F1-B866-EA5558F083D8}" name="Sprint End" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{2D2022CC-B165-4671-9773-4C7DCE737FC7}" name="User" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{6D49D607-DA69-4FF5-AC26-260E9F796217}" name="ID" dataDxfId="38"/>
-    <tableColumn id="6" xr3:uid="{95077F2F-115F-484E-A38C-A34A2BCBCB78}" name="Epic" dataDxfId="37"/>
-    <tableColumn id="12" xr3:uid="{2EAFDE91-2C58-4973-A684-28E2E964F629}" name="User Story /Task" dataDxfId="36"/>
-    <tableColumn id="11" xr3:uid="{D17AAC02-918A-4F08-B037-3622F37B62F0}" name="Estimated time" dataDxfId="35"/>
-    <tableColumn id="8" xr3:uid="{4D053EE2-698A-4191-ABEB-8F0701DA4D4E}" name="COS (Criteria of Satisfaction)" dataDxfId="34"/>
-    <tableColumn id="9" xr3:uid="{73BF0134-792D-4614-95FB-754C4A317665}" name="Story points" dataDxfId="33"/>
-    <tableColumn id="10" xr3:uid="{2620A9CC-A288-4874-BF27-2BBE69671B14}" name="Time in Hours" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{9C36A560-9153-4D8E-BA50-0044E74E1896}" name="Sprint Start" dataDxfId="73"/>
+    <tableColumn id="2" xr3:uid="{4FAB3106-8621-41F1-B866-EA5558F083D8}" name="Sprint End" dataDxfId="72"/>
+    <tableColumn id="3" xr3:uid="{2D2022CC-B165-4671-9773-4C7DCE737FC7}" name="User" dataDxfId="71"/>
+    <tableColumn id="5" xr3:uid="{6D49D607-DA69-4FF5-AC26-260E9F796217}" name="ID" dataDxfId="70"/>
+    <tableColumn id="6" xr3:uid="{95077F2F-115F-484E-A38C-A34A2BCBCB78}" name="Epic" dataDxfId="69"/>
+    <tableColumn id="12" xr3:uid="{2EAFDE91-2C58-4973-A684-28E2E964F629}" name="User Story /Task" dataDxfId="68"/>
+    <tableColumn id="11" xr3:uid="{D17AAC02-918A-4F08-B037-3622F37B62F0}" name="Estimated time" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{4D053EE2-698A-4191-ABEB-8F0701DA4D4E}" name="COS (Criteria of Satisfaction)" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{73BF0134-792D-4614-95FB-754C4A317665}" name="Story points" dataDxfId="65"/>
+    <tableColumn id="10" xr3:uid="{2620A9CC-A288-4874-BF27-2BBE69671B14}" name="Time in Hours" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
   <autoFilter ref="A16:C17" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="28">
+    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="60">
       <calculatedColumnFormula>SUM(Tabelle27[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="27">
+    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="59">
       <calculatedColumnFormula>SUM(Tabelle27[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="26">
+    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="58">
       <calculatedColumnFormula>Tabelle38[[#This Row],[Estimated time]]-Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2306,13 +2769,13 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
   <autoFilter ref="E16:F17" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="23">
+    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="55">
       <calculatedColumnFormula>SUM(Tabelle27[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="22">
+    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="54">
       <calculatedColumnFormula>Tabelle49[[#This Row],[Total Storypoints ]]/Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2321,36 +2784,36 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6303AB7F-CDC2-408B-A450-96D692A68B43}" name="Tabelle2710" displayName="Tabelle2710" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6303AB7F-CDC2-408B-A450-96D692A68B43}" name="Tabelle2710" displayName="Tabelle2710" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
   <autoFilter ref="A1:K12" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{949CA967-02A0-4249-BB07-B02F4C4F69AE}" name="Sprint Start" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{A70AE104-D3DD-4C6E-8E50-E151404B19BD}" name="Sprint End" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{9168C6BE-6970-4420-9D5F-DBCF1E8E2BAE}" name="User" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{A7C4968E-9480-42FF-949B-9E41609C26A2}" name="ID" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{8564B7DD-8DB4-4E2B-BDDB-9791D9AAA0EA}" name="Epic" dataDxfId="15"/>
-    <tableColumn id="12" xr3:uid="{56FA47CB-3810-4B7F-A047-8358D5C73F6C}" name="User Story /Task" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{988CB3AF-F268-445B-887C-5163D9AE41DF}" name="Estimated time" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{14BDCFB4-F75D-4798-AFF3-3F8B177B78D6}" name="COS (Criteria of Satisfaction)" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{97C18CBF-2D3F-4A8A-B36D-6328E17F31C4}" name="Story points" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{D3E339CF-38BF-4AC1-8C80-41ECD30B6907}" name="Time in Hours" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{3BCBC0DA-7C9B-4D2B-9269-A319CBD925C5}" name="Status" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{949CA967-02A0-4249-BB07-B02F4C4F69AE}" name="Sprint Start" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{A70AE104-D3DD-4C6E-8E50-E151404B19BD}" name="Sprint End" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{9168C6BE-6970-4420-9D5F-DBCF1E8E2BAE}" name="User" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{A7C4968E-9480-42FF-949B-9E41609C26A2}" name="ID" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{8564B7DD-8DB4-4E2B-BDDB-9791D9AAA0EA}" name="Epic" dataDxfId="47"/>
+    <tableColumn id="12" xr3:uid="{56FA47CB-3810-4B7F-A047-8358D5C73F6C}" name="User Story /Task" dataDxfId="46"/>
+    <tableColumn id="11" xr3:uid="{988CB3AF-F268-445B-887C-5163D9AE41DF}" name="Estimated time" dataDxfId="45"/>
+    <tableColumn id="8" xr3:uid="{14BDCFB4-F75D-4798-AFF3-3F8B177B78D6}" name="COS (Criteria of Satisfaction)" dataDxfId="44"/>
+    <tableColumn id="9" xr3:uid="{97C18CBF-2D3F-4A8A-B36D-6328E17F31C4}" name="Story points" dataDxfId="43"/>
+    <tableColumn id="10" xr3:uid="{D3E339CF-38BF-4AC1-8C80-41ECD30B6907}" name="Time in Hours" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{3BCBC0DA-7C9B-4D2B-9269-A319CBD925C5}" name="Status" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C1E761E2-D340-4C7F-A19A-AE84A76F5971}" name="Tabelle3811" displayName="Tabelle3811" ref="A16:C17" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C1E761E2-D340-4C7F-A19A-AE84A76F5971}" name="Tabelle3811" displayName="Tabelle3811" ref="A16:C17" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
   <autoFilter ref="A16:C17" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{F045D4AD-2D00-44A7-8EA7-B5C34869B26F}" name="Estimated time" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{F045D4AD-2D00-44A7-8EA7-B5C34869B26F}" name="Estimated time" dataDxfId="38">
       <calculatedColumnFormula>SUM(Tabelle2710[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DFDFE0A8-6207-4F3B-9D05-4D3AF083E31B}" name="Actual time" dataDxfId="5">
+    <tableColumn id="2" xr3:uid="{DFDFE0A8-6207-4F3B-9D05-4D3AF083E31B}" name="Actual time" dataDxfId="37">
       <calculatedColumnFormula>SUM(Tabelle2710[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{2529739A-9C5E-4AE4-80A6-DFC080EFE2D8}" name="Delta" dataDxfId="4">
+    <tableColumn id="3" xr3:uid="{2529739A-9C5E-4AE4-80A6-DFC080EFE2D8}" name="Delta" dataDxfId="36">
       <calculatedColumnFormula>Tabelle3811[[#This Row],[Estimated time]]-Tabelle3811[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2789,42 +3252,59 @@
       </c>
       <c r="C4" s="7" cm="1">
         <f t="array" ref="C4">Tabelle3811[Estimated time]</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D4" s="7" cm="1">
         <f t="array" ref="D4">Tabelle3811[Actual time]</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E4" s="7" cm="1">
         <f t="array" ref="E4">Tabelle4912[[Total Storypoints ]]</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F4" s="7">
         <f>IFERROR(Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]],0)</f>
-        <v>0</v>
-      </c>
-      <c r="G4" s="7"/>
+        <v>1</v>
+      </c>
+      <c r="G4" s="7">
+        <f>H3</f>
+        <v>122</v>
+      </c>
       <c r="H4" s="7">
         <f>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</f>
-        <v>0</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="21" x14ac:dyDescent="0.5">
       <c r="A5" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
+      <c r="B5" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C5" s="7" cm="1">
+        <f t="array" ref="C5">Tabelle381114[Estimated time]</f>
+        <v>13</v>
+      </c>
+      <c r="D5" s="7" cm="1">
+        <f t="array" ref="D5">Tabelle381114[Actual time]</f>
+        <v>14</v>
+      </c>
+      <c r="E5" s="7" cm="1">
+        <f t="array" ref="E5">Tabelle491215[[Total Storypoints ]]</f>
+        <v>26</v>
+      </c>
       <c r="F5" s="7">
         <f>IFERROR(Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]],0)</f>
-        <v>0</v>
-      </c>
-      <c r="G5" s="7"/>
+        <v>1.8571428571428572</v>
+      </c>
+      <c r="G5" s="7">
+        <f>H4</f>
+        <v>112</v>
+      </c>
       <c r="H5" s="7">
         <f>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</f>
-        <v>0</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.5">
@@ -2895,7 +3375,7 @@
       </c>
       <c r="C13" s="5">
         <f>C12-SUM(Tabelle1[Accomplished Story Points])</f>
-        <v>122</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
@@ -2913,7 +3393,7 @@
       </c>
       <c r="C15" s="5">
         <f>AVERAGE(Tabelle1[Velocity])</f>
-        <v>0.10084033613445378</v>
+        <v>0.50900360144057621</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
@@ -2922,7 +3402,7 @@
       </c>
       <c r="C16" s="14">
         <f>(SUM(Tabelle1[Accomplished Story Points],)/G2)</f>
-        <v>0.16438356164383561</v>
+        <v>0.41095890410958902</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="23.5" x14ac:dyDescent="0.55000000000000004">
@@ -2931,11 +3411,11 @@
       </c>
       <c r="C17" s="18">
         <f>C13/C15</f>
-        <v>1209.8333333333333</v>
+        <v>168.95754716981133</v>
       </c>
       <c r="D17">
         <f>C17/3</f>
-        <v>403.27777777777777</v>
+        <v>56.319182389937112</v>
       </c>
     </row>
   </sheetData>
@@ -3801,22 +4281,46 @@
       <c r="H3" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="19"/>
+      <c r="I3" s="8">
+        <v>3</v>
+      </c>
+      <c r="J3" s="8">
+        <v>6</v>
+      </c>
+      <c r="K3" s="19" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="19"/>
+      <c r="C4" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="8">
+        <v>4</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="8">
+        <v>7</v>
+      </c>
+      <c r="J4" s="8">
+        <v>4</v>
+      </c>
+      <c r="K4" s="19" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="8"/>
@@ -3824,7 +4328,7 @@
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
+      <c r="F5" s="2"/>
       <c r="G5" s="8"/>
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
@@ -3983,24 +4487,24 @@
     <row r="17" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A17" s="12">
         <f>SUM(Tabelle2710[Estimated time])</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B17" s="12">
         <f>SUM(Tabelle2710[Time in Hours])</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C17" s="12">
         <f>Tabelle3811[[#This Row],[Estimated time]]-Tabelle3811[[#This Row],[Actual time]]</f>
-        <v>5</v>
+        <v>-1</v>
       </c>
       <c r="D17" s="8"/>
       <c r="E17" s="12">
         <f>SUM(Tabelle2710[Story points])</f>
-        <v>0</v>
-      </c>
-      <c r="F17" s="12" t="e">
+        <v>10</v>
+      </c>
+      <c r="F17" s="12">
         <f>Tabelle4912[[#This Row],[Total Storypoints ]]/Tabelle3811[[#This Row],[Actual time]]</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
@@ -4019,6 +4523,359 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11843E7F-69B2-4364-9B99-E21372FE87D3}">
+  <sheetPr>
+    <tabColor theme="0"/>
+  </sheetPr>
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="9">
+        <v>45981</v>
+      </c>
+      <c r="B2" s="9">
+        <v>45995</v>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="19"/>
+    </row>
+    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="G3" s="8">
+        <v>10</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="I3" s="8">
+        <v>8</v>
+      </c>
+      <c r="J3" s="8">
+        <v>10</v>
+      </c>
+      <c r="K3" s="19" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A4" s="8"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="8">
+        <v>1</v>
+      </c>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8">
+        <v>4</v>
+      </c>
+      <c r="J4" s="8">
+        <v>1</v>
+      </c>
+      <c r="K4" s="19" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="G5" s="8">
+        <v>1</v>
+      </c>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8">
+        <v>8</v>
+      </c>
+      <c r="J5" s="8">
+        <v>1</v>
+      </c>
+      <c r="K5" s="19" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="8">
+        <v>1</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="I6" s="8">
+        <v>6</v>
+      </c>
+      <c r="J6" s="8">
+        <v>2</v>
+      </c>
+      <c r="K6" s="19" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="19"/>
+    </row>
+    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="19"/>
+    </row>
+    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="19"/>
+    </row>
+    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="19"/>
+    </row>
+    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="19"/>
+    </row>
+    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+    </row>
+    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+    </row>
+    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A15" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D15" s="8"/>
+      <c r="E15" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+    </row>
+    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A16" s="12">
+        <f>SUM(Tabelle271013[Estimated time])</f>
+        <v>13</v>
+      </c>
+      <c r="B16" s="12">
+        <f>SUM(Tabelle271013[Time in Hours])</f>
+        <v>14</v>
+      </c>
+      <c r="C16" s="12">
+        <f>Tabelle381114[[#This Row],[Estimated time]]-Tabelle381114[[#This Row],[Actual time]]</f>
+        <v>-1</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="12">
+        <f>SUM(Tabelle271013[Story points])</f>
+        <v>26</v>
+      </c>
+      <c r="F16" s="12">
+        <f>Tabelle491215[[#This Row],[Total Storypoints ]]/Tabelle381114[[#This Row],[Actual time]]</f>
+        <v>1.8571428571428572</v>
+      </c>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <tableParts count="3">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7C2A55-0520-4EB5-86E6-237FE14873A1}">
   <sheetPr>
     <tabColor theme="6"/>
@@ -4097,12 +4954,14 @@
         <v>126</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>9</v>
+        <v>136</v>
       </c>
       <c r="F3" s="2">
         <v>8</v>
       </c>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2">
+        <v>2</v>
+      </c>
       <c r="I3" s="17"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -4124,7 +4983,9 @@
       <c r="F4" s="2">
         <v>8</v>
       </c>
-      <c r="G4" s="2"/>
+      <c r="G4" s="2">
+        <v>4</v>
+      </c>
       <c r="I4" s="17"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -4141,12 +5002,14 @@
         <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>9</v>
+        <v>136</v>
       </c>
       <c r="F5" s="2">
         <v>5</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="G5" s="2">
+        <v>3</v>
+      </c>
       <c r="I5" s="17"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -4163,12 +5026,14 @@
         <v>17</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>9</v>
+        <v>136</v>
       </c>
       <c r="F6" s="2">
         <v>4</v>
       </c>
-      <c r="G6" s="2"/>
+      <c r="G6" s="2">
+        <v>3</v>
+      </c>
       <c r="I6" s="17"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -4185,12 +5050,14 @@
         <v>20</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>9</v>
+        <v>136</v>
       </c>
       <c r="F7" s="2">
         <v>6</v>
       </c>
-      <c r="G7" s="2"/>
+      <c r="G7" s="2">
+        <v>2</v>
+      </c>
       <c r="I7" s="17"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -4229,12 +5096,14 @@
         <v>26</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>9</v>
+        <v>136</v>
       </c>
       <c r="F9" s="2">
         <v>4</v>
       </c>
-      <c r="G9" s="2"/>
+      <c r="G9" s="2">
+        <v>4</v>
+      </c>
       <c r="I9" s="17"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -4295,12 +5164,14 @@
         <v>35</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>9</v>
+        <v>136</v>
       </c>
       <c r="F12" s="2">
         <v>6</v>
       </c>
-      <c r="G12" s="2"/>
+      <c r="G12" s="2">
+        <v>4</v>
+      </c>
       <c r="I12" s="17"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
@@ -4339,12 +5210,14 @@
         <v>41</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>9</v>
+        <v>136</v>
       </c>
       <c r="F14" s="2">
         <v>7</v>
       </c>
-      <c r="G14" s="2"/>
+      <c r="G14" s="2">
+        <v>3</v>
+      </c>
       <c r="I14" s="17"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
refactored component to services and models; Added hunger and feeding system; added death to fish; changed particle behaviour
</commit_message>
<xml_diff>
--- a/aquasphere/Excel_File/AquaSphare.xlsx
+++ b/aquasphere/Excel_File/AquaSphare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\43680\Desktop\Schule\SYP\Aquarium\aquasphere\Excel_File\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielhoheneder/Desktop/Schule/syp/AquaSphere/aquasphere/Excel_File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{470DDF49-15FE-4ABF-AF84-A7B4435C02B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{814EE111-34FA-1442-A523-9E9D2A8E3C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
+    <workbookView xWindow="6800" yWindow="680" windowWidth="27760" windowHeight="20140" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Dashboard" sheetId="2" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="154">
   <si>
     <t>Story ID</t>
   </si>
@@ -131,12 +131,6 @@
     <t>AQU7</t>
   </si>
   <si>
-    <t>Gamification</t>
-  </si>
-  <si>
-    <t>Als Nutzer möchte ich neue Fischarten freischalten.</t>
-  </si>
-  <si>
     <t>AQU8</t>
   </si>
   <si>
@@ -149,12 +143,6 @@
     <t>AQU9</t>
   </si>
   <si>
-    <t>Premium</t>
-  </si>
-  <si>
-    <t>Als Nutzer möchte ich seltene Fischarten kaufen.</t>
-  </si>
-  <si>
     <t>AQU10</t>
   </si>
   <si>
@@ -176,12 +164,6 @@
     <t>AQU12</t>
   </si>
   <si>
-    <t>Sound</t>
-  </si>
-  <si>
-    <t>Als Nutzer möchte ich entspannende Hintergrundmusik hören.</t>
-  </si>
-  <si>
     <t>AQU13</t>
   </si>
   <si>
@@ -194,12 +176,6 @@
     <t>AQU14</t>
   </si>
   <si>
-    <t>Community</t>
-  </si>
-  <si>
-    <t>Als Nutzer möchte ich Screenshots meines Aquariums teilen.</t>
-  </si>
-  <si>
     <t>AQU15</t>
   </si>
   <si>
@@ -284,21 +260,6 @@
     <t>AQU24</t>
   </si>
   <si>
-    <t>Offline-Modus</t>
-  </si>
-  <si>
-    <t>Als Nutzer möchte ich die App ohne Internet nutzen.</t>
-  </si>
-  <si>
-    <t>AQU25</t>
-  </si>
-  <si>
-    <t>Mini-Spiele</t>
-  </si>
-  <si>
-    <t>Als Nutzer möchte ich kleine Spiele im Aquarium spielen.</t>
-  </si>
-  <si>
     <t>Estimated Hours</t>
   </si>
   <si>
@@ -485,9 +446,6 @@
     <t>Effort/Hour</t>
   </si>
   <si>
-    <t>Started / not done</t>
-  </si>
-  <si>
     <t>Als Nutzer möchte ich mein Aquarium geräteübergreifend synchronisieren. / Backend mit Datenbank erstellen</t>
   </si>
   <si>
@@ -515,9 +473,6 @@
     <t>Als Nutzer möchte ich Steine und Korallen platzieren. Unterschiedliche Pflanzen sollen zur auswahl steten</t>
   </si>
   <si>
-    <t>AQ20</t>
-  </si>
-  <si>
     <t>Cloud/Sync</t>
   </si>
   <si>
@@ -531,6 +486,45 @@
   </si>
   <si>
     <t>Als Nutzer möchte ich Mein Aquarium auf verschiedenen geräten sehen</t>
+  </si>
+  <si>
+    <t>FischKI</t>
+  </si>
+  <si>
+    <t>Die KI muss verschiedene Szenarien und verhaltensweisen aufweisen (Füttern, FreeRoam, Tot)</t>
+  </si>
+  <si>
+    <t>Futter-System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Als Nutzer möchte ich die Fische füttern können und müssen </t>
+  </si>
+  <si>
+    <t>Hunger-System</t>
+  </si>
+  <si>
+    <t>Fisch-Statistiken</t>
+  </si>
+  <si>
+    <t>Als Nutzer möchte ich sehen welcher Fisch was für einen Zustand hat</t>
+  </si>
+  <si>
+    <t>Als Nutzer möchte ich den Hungerzustand meiner Fische wissen und handeln können</t>
+  </si>
+  <si>
+    <t>Als Nutzer möchte ich einen Tag/Nacht Zyklus haben</t>
+  </si>
+  <si>
+    <t>Tutorial/Onboarding</t>
+  </si>
+  <si>
+    <t>Als Nutzer möchte ich wissen wie ich die App bediene und einen Überblick über die Funktionen bekommen</t>
+  </si>
+  <si>
+    <t>AQ17</t>
+  </si>
+  <si>
+    <t>Es muss ein visueller Balken oder ähnliches vorhanden sein der anzeigt wann ein Fisch Hunger hat und gefüttert gehört</t>
   </si>
 </sst>
 </file>
@@ -672,7 +666,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -693,423 +687,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="4" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Prozent" xfId="1" builtinId="5"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="106">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="16"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.89999084444715716"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF0F9ED5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF0F9ED5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2052,15 +1636,15 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2157,6 +1741,397 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
         <family val="2"/>
@@ -2401,6 +2376,26 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -2582,11 +2577,11 @@
     <tableColumn id="4" xr3:uid="{D6FF0659-1B35-4F09-B5A7-D22FEF5F7C3F}" name="Accomplished Story Points" dataDxfId="99">
       <calculatedColumnFormula array="1">Tabelle4[[Total Storypoints ]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{9CD2DBE3-2E45-4440-8D7A-2A03A0291AAD}" name="Velocity" dataDxfId="0">
+    <tableColumn id="5" xr3:uid="{9CD2DBE3-2E45-4440-8D7A-2A03A0291AAD}" name="Velocity" dataDxfId="98">
       <calculatedColumnFormula>IFERROR(Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{1977DF7A-0A05-43B5-99D3-B72159480780}" name="Total Storypoints" dataDxfId="98"/>
-    <tableColumn id="7" xr3:uid="{D8A5F5FE-B9BC-448A-A9E7-3D00888AE639}" name="Storypoints Left" dataDxfId="97">
+    <tableColumn id="6" xr3:uid="{1977DF7A-0A05-43B5-99D3-B72159480780}" name="Total Storypoints" dataDxfId="97"/>
+    <tableColumn id="7" xr3:uid="{D8A5F5FE-B9BC-448A-A9E7-3D00888AE639}" name="Storypoints Left" dataDxfId="96">
       <calculatedColumnFormula>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2595,13 +2590,13 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0134C802-458D-4153-B0D4-D8B08E02E26A}" name="Tabelle4912" displayName="Tabelle4912" ref="E16:F17" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0134C802-458D-4153-B0D4-D8B08E02E26A}" name="Tabelle4912" displayName="Tabelle4912" ref="E16:F17" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <autoFilter ref="E16:F17" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C3438C75-AD69-46E0-B1BD-0445ED469483}" name="Total Storypoints " dataDxfId="33">
+    <tableColumn id="1" xr3:uid="{C3438C75-AD69-46E0-B1BD-0445ED469483}" name="Total Storypoints " dataDxfId="32">
       <calculatedColumnFormula>SUM(Tabelle2710[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0655740B-E1AB-4BD3-B7CA-852D4C79FC17}" name="Effort/Hour" dataDxfId="32">
+    <tableColumn id="2" xr3:uid="{0655740B-E1AB-4BD3-B7CA-852D4C79FC17}" name="Effort/Hour" dataDxfId="31">
       <calculatedColumnFormula>Tabelle4912[[#This Row],[Total Storypoints ]]/Tabelle3811[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2610,36 +2605,36 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}" name="Tabelle271013" displayName="Tabelle271013" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}" name="Tabelle271013" displayName="Tabelle271013" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
   <autoFilter ref="A1:K11" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{946A4B14-799A-49AD-8E3E-31E3F4BBE559}" name="Sprint Start" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{E61A962F-4EE4-4843-AF21-C647918EECAB}" name="Sprint End" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{4EC50B40-18BD-4D00-8BE2-5596A9347BB8}" name="User" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{2A1F175E-D14E-491C-B452-39567CF84CD6}" name="ID" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{DCE5121F-D243-470B-B0AF-D0EE5264DD5A}" name="Epic" dataDxfId="16"/>
-    <tableColumn id="12" xr3:uid="{45FDCCAE-F13D-47C1-B91E-2EF3CC9A5BA0}" name="User Story /Task" dataDxfId="15"/>
-    <tableColumn id="11" xr3:uid="{4057DF12-8977-4284-BF2B-9ED3AAE7221F}" name="Estimated time" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{08443A2E-5832-4299-8009-1F0D489DEE15}" name="COS (Criteria of Satisfaction)" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{8777A429-C11B-4CDC-BB2F-785D0BC89DAB}" name="Story points" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{0B18443F-D8D9-4015-8EAA-7050016E43C2}" name="Time in Hours" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{5C5B5C91-6376-4597-B69B-4D162307C569}" name="Status" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{946A4B14-799A-49AD-8E3E-31E3F4BBE559}" name="Sprint Start" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{E61A962F-4EE4-4843-AF21-C647918EECAB}" name="Sprint End" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{4EC50B40-18BD-4D00-8BE2-5596A9347BB8}" name="User" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{2A1F175E-D14E-491C-B452-39567CF84CD6}" name="ID" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{DCE5121F-D243-470B-B0AF-D0EE5264DD5A}" name="Epic" dataDxfId="24"/>
+    <tableColumn id="12" xr3:uid="{45FDCCAE-F13D-47C1-B91E-2EF3CC9A5BA0}" name="User Story /Task" dataDxfId="23"/>
+    <tableColumn id="11" xr3:uid="{4057DF12-8977-4284-BF2B-9ED3AAE7221F}" name="Estimated time" dataDxfId="22"/>
+    <tableColumn id="8" xr3:uid="{08443A2E-5832-4299-8009-1F0D489DEE15}" name="COS (Criteria of Satisfaction)" dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{8777A429-C11B-4CDC-BB2F-785D0BC89DAB}" name="Story points" dataDxfId="20"/>
+    <tableColumn id="10" xr3:uid="{0B18443F-D8D9-4015-8EAA-7050016E43C2}" name="Time in Hours" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{5C5B5C91-6376-4597-B69B-4D162307C569}" name="Status" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}" name="Tabelle381114" displayName="Tabelle381114" ref="A15:C16" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}" name="Tabelle381114" displayName="Tabelle381114" ref="A15:C16" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="A15:C16" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{E71994D0-AB06-482B-8487-03AB7E3B1FF7}" name="Estimated time" dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{E71994D0-AB06-482B-8487-03AB7E3B1FF7}" name="Estimated time" dataDxfId="15">
       <calculatedColumnFormula>SUM(Tabelle271013[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E607785B-5B58-4D1E-81ED-45AAAAF488F0}" name="Actual time" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{E607785B-5B58-4D1E-81ED-45AAAAF488F0}" name="Actual time" dataDxfId="14">
       <calculatedColumnFormula>SUM(Tabelle271013[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{0197CFBA-597E-49C6-88E5-ABAC17763EA4}" name="Delta" dataDxfId="5">
+    <tableColumn id="3" xr3:uid="{0197CFBA-597E-49C6-88E5-ABAC17763EA4}" name="Delta" dataDxfId="13">
       <calculatedColumnFormula>Tabelle381114[[#This Row],[Estimated time]]-Tabelle381114[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2648,13 +2643,13 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}" name="Tabelle491215" displayName="Tabelle491215" ref="E15:F16" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}" name="Tabelle491215" displayName="Tabelle491215" ref="E15:F16" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="E15:F16" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{E0381C51-E5FF-4087-9146-76E105FE701A}" name="Total Storypoints " dataDxfId="2">
+    <tableColumn id="1" xr3:uid="{E0381C51-E5FF-4087-9146-76E105FE701A}" name="Total Storypoints " dataDxfId="10">
       <calculatedColumnFormula>SUM(Tabelle271013[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0971B46C-CFAA-4F13-88AB-CDC5655C1F84}" name="Effort/Hour" dataDxfId="1">
+    <tableColumn id="2" xr3:uid="{0971B46C-CFAA-4F13-88AB-CDC5655C1F84}" name="Effort/Hour" dataDxfId="9">
       <calculatedColumnFormula>Tabelle491215[[#This Row],[Total Storypoints ]]/Tabelle381114[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2663,51 +2658,51 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:G27" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
-  <autoFilter ref="A1:G27" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:G26" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:G26" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Effort" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Effort" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}" name="Tabelle2" displayName="Tabelle2" ref="A1:J9" insertRowShift="1" totalsRowShown="0" headerRowDxfId="96" dataDxfId="95">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}" name="Tabelle2" displayName="Tabelle2" ref="A1:J9" insertRowShift="1" totalsRowShown="0" headerRowDxfId="95" dataDxfId="94">
   <autoFilter ref="A1:J9" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{0351E8C1-0BB8-4C19-A406-233CC12328E5}" name="Sprint Start" dataDxfId="94"/>
-    <tableColumn id="2" xr3:uid="{51BD2FE0-507A-4398-BD96-E186E78BB2C7}" name="Sprint End" dataDxfId="93"/>
-    <tableColumn id="3" xr3:uid="{A3B7E86B-E01A-4D78-82AD-BA81F6AC7ADF}" name="User" dataDxfId="92"/>
-    <tableColumn id="5" xr3:uid="{CE780601-F45C-4063-B216-98ACE5588903}" name="ID" dataDxfId="91"/>
-    <tableColumn id="6" xr3:uid="{A14D049D-AC5C-49A5-A7CC-A4D5ED8A8330}" name="Epic" dataDxfId="90"/>
-    <tableColumn id="12" xr3:uid="{770F10A6-830A-41AC-B069-6267CAE00BDF}" name="User Story /Task" dataDxfId="89"/>
-    <tableColumn id="11" xr3:uid="{0D9AB552-F7B4-4231-A35B-245B57383919}" name="Estimated time" dataDxfId="88"/>
-    <tableColumn id="8" xr3:uid="{3E2E3644-9002-4AB9-B3EC-96FFF84D8900}" name="COS (Criteria of Satisfaction)" dataDxfId="87"/>
-    <tableColumn id="9" xr3:uid="{14C8E3A9-BC37-48D9-A399-32A48A46993A}" name="Story points" dataDxfId="86"/>
-    <tableColumn id="10" xr3:uid="{151786D9-5F15-42D7-932B-664A024F4131}" name="Time in Hours" dataDxfId="85"/>
+    <tableColumn id="1" xr3:uid="{0351E8C1-0BB8-4C19-A406-233CC12328E5}" name="Sprint Start" dataDxfId="93"/>
+    <tableColumn id="2" xr3:uid="{51BD2FE0-507A-4398-BD96-E186E78BB2C7}" name="Sprint End" dataDxfId="92"/>
+    <tableColumn id="3" xr3:uid="{A3B7E86B-E01A-4D78-82AD-BA81F6AC7ADF}" name="User" dataDxfId="91"/>
+    <tableColumn id="5" xr3:uid="{CE780601-F45C-4063-B216-98ACE5588903}" name="ID" dataDxfId="90"/>
+    <tableColumn id="6" xr3:uid="{A14D049D-AC5C-49A5-A7CC-A4D5ED8A8330}" name="Epic" dataDxfId="89"/>
+    <tableColumn id="12" xr3:uid="{770F10A6-830A-41AC-B069-6267CAE00BDF}" name="User Story /Task" dataDxfId="88"/>
+    <tableColumn id="11" xr3:uid="{0D9AB552-F7B4-4231-A35B-245B57383919}" name="Estimated time" dataDxfId="87"/>
+    <tableColumn id="8" xr3:uid="{3E2E3644-9002-4AB9-B3EC-96FFF84D8900}" name="COS (Criteria of Satisfaction)" dataDxfId="86"/>
+    <tableColumn id="9" xr3:uid="{14C8E3A9-BC37-48D9-A399-32A48A46993A}" name="Story points" dataDxfId="85"/>
+    <tableColumn id="10" xr3:uid="{151786D9-5F15-42D7-932B-664A024F4131}" name="Time in Hours" dataDxfId="84"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}" name="Tabelle3" displayName="Tabelle3" ref="A15:C16" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}" name="Tabelle3" displayName="Tabelle3" ref="A15:C16" totalsRowShown="0" headerRowDxfId="83" dataDxfId="82">
   <autoFilter ref="A15:C16" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CD2D4D96-DD34-4EA3-92D7-B02BB9DE5647}" name="Estimated time" dataDxfId="82">
+    <tableColumn id="1" xr3:uid="{CD2D4D96-DD34-4EA3-92D7-B02BB9DE5647}" name="Estimated time" dataDxfId="81">
       <calculatedColumnFormula>SUM(Tabelle2[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0F14E190-6E0A-4AB8-8ADE-83875E98D4B5}" name="Actual time" dataDxfId="81">
+    <tableColumn id="2" xr3:uid="{0F14E190-6E0A-4AB8-8ADE-83875E98D4B5}" name="Actual time" dataDxfId="80">
       <calculatedColumnFormula>SUM(Tabelle2[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{5DE18543-F4D3-4732-9F2D-5B7F140CB974}" name="Delta" dataDxfId="80">
+    <tableColumn id="3" xr3:uid="{5DE18543-F4D3-4732-9F2D-5B7F140CB974}" name="Delta" dataDxfId="79">
       <calculatedColumnFormula>Tabelle3[[#This Row],[Estimated time]]-Tabelle3[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2716,13 +2711,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}" name="Tabelle4" displayName="Tabelle4" ref="E15:F16" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}" name="Tabelle4" displayName="Tabelle4" ref="E15:F16" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
   <autoFilter ref="E15:F16" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{2E187AEA-682F-4749-9FC8-ED3BA3DE1DA2}" name="Total Storypoints " dataDxfId="77">
+    <tableColumn id="1" xr3:uid="{2E187AEA-682F-4749-9FC8-ED3BA3DE1DA2}" name="Total Storypoints " dataDxfId="76">
       <calculatedColumnFormula>SUM(Tabelle2[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3C6DC8F5-724A-43AC-9128-7661A96380C1}" name="Efford/Hour" dataDxfId="76">
+    <tableColumn id="2" xr3:uid="{3C6DC8F5-724A-43AC-9128-7661A96380C1}" name="Efford/Hour" dataDxfId="75">
       <calculatedColumnFormula>Tabelle4[[#This Row],[Total Storypoints ]]/Tabelle3[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2731,36 +2726,36 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A211D33B-248F-4E66-AF7C-9632EAA38DAC}" name="Tabelle27" displayName="Tabelle27" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A211D33B-248F-4E66-AF7C-9632EAA38DAC}" name="Tabelle27" displayName="Tabelle27" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="74" dataDxfId="73">
   <autoFilter ref="A1:K12" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{9C36A560-9153-4D8E-BA50-0044E74E1896}" name="Sprint Start" dataDxfId="73"/>
-    <tableColumn id="2" xr3:uid="{4FAB3106-8621-41F1-B866-EA5558F083D8}" name="Sprint End" dataDxfId="72"/>
-    <tableColumn id="3" xr3:uid="{2D2022CC-B165-4671-9773-4C7DCE737FC7}" name="User" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{6D49D607-DA69-4FF5-AC26-260E9F796217}" name="ID" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{95077F2F-115F-484E-A38C-A34A2BCBCB78}" name="Epic" dataDxfId="69"/>
-    <tableColumn id="12" xr3:uid="{2EAFDE91-2C58-4973-A684-28E2E964F629}" name="User Story /Task" dataDxfId="68"/>
-    <tableColumn id="11" xr3:uid="{D17AAC02-918A-4F08-B037-3622F37B62F0}" name="Estimated time" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{4D053EE2-698A-4191-ABEB-8F0701DA4D4E}" name="COS (Criteria of Satisfaction)" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{73BF0134-792D-4614-95FB-754C4A317665}" name="Story points" dataDxfId="65"/>
-    <tableColumn id="10" xr3:uid="{2620A9CC-A288-4874-BF27-2BBE69671B14}" name="Time in Hours" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{9C36A560-9153-4D8E-BA50-0044E74E1896}" name="Sprint Start" dataDxfId="72"/>
+    <tableColumn id="2" xr3:uid="{4FAB3106-8621-41F1-B866-EA5558F083D8}" name="Sprint End" dataDxfId="71"/>
+    <tableColumn id="3" xr3:uid="{2D2022CC-B165-4671-9773-4C7DCE737FC7}" name="User" dataDxfId="70"/>
+    <tableColumn id="5" xr3:uid="{6D49D607-DA69-4FF5-AC26-260E9F796217}" name="ID" dataDxfId="69"/>
+    <tableColumn id="6" xr3:uid="{95077F2F-115F-484E-A38C-A34A2BCBCB78}" name="Epic" dataDxfId="68"/>
+    <tableColumn id="12" xr3:uid="{2EAFDE91-2C58-4973-A684-28E2E964F629}" name="User Story /Task" dataDxfId="67"/>
+    <tableColumn id="11" xr3:uid="{D17AAC02-918A-4F08-B037-3622F37B62F0}" name="Estimated time" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{4D053EE2-698A-4191-ABEB-8F0701DA4D4E}" name="COS (Criteria of Satisfaction)" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{73BF0134-792D-4614-95FB-754C4A317665}" name="Story points" dataDxfId="64"/>
+    <tableColumn id="10" xr3:uid="{2620A9CC-A288-4874-BF27-2BBE69671B14}" name="Time in Hours" dataDxfId="63"/>
+    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="62"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60">
   <autoFilter ref="A16:C17" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="60">
+    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="59">
       <calculatedColumnFormula>SUM(Tabelle27[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="59">
+    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="58">
       <calculatedColumnFormula>SUM(Tabelle27[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="58">
+    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="57">
       <calculatedColumnFormula>Tabelle38[[#This Row],[Estimated time]]-Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2769,13 +2764,13 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="E16:F17" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="55">
+    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="54">
       <calculatedColumnFormula>SUM(Tabelle27[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="54">
+    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="53">
       <calculatedColumnFormula>Tabelle49[[#This Row],[Total Storypoints ]]/Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2784,36 +2779,36 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6303AB7F-CDC2-408B-A450-96D692A68B43}" name="Tabelle2710" displayName="Tabelle2710" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6303AB7F-CDC2-408B-A450-96D692A68B43}" name="Tabelle2710" displayName="Tabelle2710" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
   <autoFilter ref="A1:K12" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{949CA967-02A0-4249-BB07-B02F4C4F69AE}" name="Sprint Start" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{A70AE104-D3DD-4C6E-8E50-E151404B19BD}" name="Sprint End" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{9168C6BE-6970-4420-9D5F-DBCF1E8E2BAE}" name="User" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{A7C4968E-9480-42FF-949B-9E41609C26A2}" name="ID" dataDxfId="48"/>
-    <tableColumn id="6" xr3:uid="{8564B7DD-8DB4-4E2B-BDDB-9791D9AAA0EA}" name="Epic" dataDxfId="47"/>
-    <tableColumn id="12" xr3:uid="{56FA47CB-3810-4B7F-A047-8358D5C73F6C}" name="User Story /Task" dataDxfId="46"/>
-    <tableColumn id="11" xr3:uid="{988CB3AF-F268-445B-887C-5163D9AE41DF}" name="Estimated time" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{14BDCFB4-F75D-4798-AFF3-3F8B177B78D6}" name="COS (Criteria of Satisfaction)" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{97C18CBF-2D3F-4A8A-B36D-6328E17F31C4}" name="Story points" dataDxfId="43"/>
-    <tableColumn id="10" xr3:uid="{D3E339CF-38BF-4AC1-8C80-41ECD30B6907}" name="Time in Hours" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{3BCBC0DA-7C9B-4D2B-9269-A319CBD925C5}" name="Status" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{949CA967-02A0-4249-BB07-B02F4C4F69AE}" name="Sprint Start" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{A70AE104-D3DD-4C6E-8E50-E151404B19BD}" name="Sprint End" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{9168C6BE-6970-4420-9D5F-DBCF1E8E2BAE}" name="User" dataDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{A7C4968E-9480-42FF-949B-9E41609C26A2}" name="ID" dataDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{8564B7DD-8DB4-4E2B-BDDB-9791D9AAA0EA}" name="Epic" dataDxfId="46"/>
+    <tableColumn id="12" xr3:uid="{56FA47CB-3810-4B7F-A047-8358D5C73F6C}" name="User Story /Task" dataDxfId="45"/>
+    <tableColumn id="11" xr3:uid="{988CB3AF-F268-445B-887C-5163D9AE41DF}" name="Estimated time" dataDxfId="44"/>
+    <tableColumn id="8" xr3:uid="{14BDCFB4-F75D-4798-AFF3-3F8B177B78D6}" name="COS (Criteria of Satisfaction)" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{97C18CBF-2D3F-4A8A-B36D-6328E17F31C4}" name="Story points" dataDxfId="42"/>
+    <tableColumn id="10" xr3:uid="{D3E339CF-38BF-4AC1-8C80-41ECD30B6907}" name="Time in Hours" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{3BCBC0DA-7C9B-4D2B-9269-A319CBD925C5}" name="Status" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C1E761E2-D340-4C7F-A19A-AE84A76F5971}" name="Tabelle3811" displayName="Tabelle3811" ref="A16:C17" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C1E761E2-D340-4C7F-A19A-AE84A76F5971}" name="Tabelle3811" displayName="Tabelle3811" ref="A16:C17" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
   <autoFilter ref="A16:C17" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{F045D4AD-2D00-44A7-8EA7-B5C34869B26F}" name="Estimated time" dataDxfId="38">
+    <tableColumn id="1" xr3:uid="{F045D4AD-2D00-44A7-8EA7-B5C34869B26F}" name="Estimated time" dataDxfId="37">
       <calculatedColumnFormula>SUM(Tabelle2710[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DFDFE0A8-6207-4F3B-9D05-4D3AF083E31B}" name="Actual time" dataDxfId="37">
+    <tableColumn id="2" xr3:uid="{DFDFE0A8-6207-4F3B-9D05-4D3AF083E31B}" name="Actual time" dataDxfId="36">
       <calculatedColumnFormula>SUM(Tabelle2710[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{2529739A-9C5E-4AE4-80A6-DFC080EFE2D8}" name="Delta" dataDxfId="36">
+    <tableColumn id="3" xr3:uid="{2529739A-9C5E-4AE4-80A6-DFC080EFE2D8}" name="Delta" dataDxfId="35">
       <calculatedColumnFormula>Tabelle3811[[#This Row],[Estimated time]]-Tabelle3811[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3142,20 +3137,20 @@
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:H17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>5</v>
       </c>
@@ -3163,30 +3158,30 @@
         <v>0</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="C2" s="7" cm="1">
         <f t="array" ref="C2">Tabelle3[Estimated time]</f>
@@ -3212,12 +3207,12 @@
         <v>146</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C3" s="7" cm="1">
         <f t="array" ref="C3">Tabelle38[Estimated time]</f>
@@ -3243,9 +3238,9 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>14</v>
@@ -3275,28 +3270,28 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="C5" s="7" cm="1">
         <f t="array" ref="C5">Tabelle381114[Estimated time]</f>
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D5" s="7" cm="1">
         <f t="array" ref="D5">Tabelle381114[Actual time]</f>
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E5" s="7" cm="1">
         <f t="array" ref="E5">Tabelle491215[[Total Storypoints ]]</f>
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="F5" s="7">
         <f>IFERROR(Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]],0)</f>
-        <v>1.8571428571428572</v>
+        <v>1.625</v>
       </c>
       <c r="G5" s="7">
         <f>H4</f>
@@ -3304,12 +3299,12 @@
       </c>
       <c r="H5" s="7">
         <f>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</f>
-        <v>86</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -3325,9 +3320,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -3343,9 +3338,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -3361,61 +3356,61 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="C12" s="5">
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="C13" s="5">
         <f>C12-SUM(Tabelle1[Accomplished Story Points])</f>
-        <v>86</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="C14" s="5">
         <f>COUNTIF(Tabelle1[Sprint],"*Sprint*")</f>
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="C15" s="5">
         <f>AVERAGE(Tabelle1[Velocity])</f>
-        <v>0.50900360144057621</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>0.47584033613445381</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="C16" s="14">
         <f>(SUM(Tabelle1[Accomplished Story Points],)/G2)</f>
-        <v>0.41095890410958902</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" ht="24" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="C17" s="18">
         <f>C13/C15</f>
-        <v>168.95754716981133</v>
+        <v>153.41280353200881</v>
       </c>
       <c r="D17">
         <f>C17/3</f>
-        <v>56.319182389937112</v>
+        <v>51.137601177336272</v>
       </c>
     </row>
   </sheetData>
@@ -3433,53 +3428,53 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:J16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="95.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="95.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>111</v>
-      </c>
       <c r="G1" s="8" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45925</v>
       </c>
@@ -3487,60 +3482,60 @@
         <v>45932</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D2" s="10"/>
       <c r="E2" s="8" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="G2" s="8">
         <v>2</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="J2" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
       <c r="F3" s="8" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="G3" s="8">
         <v>4</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I3" s="8"/>
       <c r="J3" s="8">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
       <c r="F4" s="8" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
       <c r="G4" s="8">
         <v>1</v>
@@ -3551,7 +3546,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -3563,26 +3558,26 @@
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
     </row>
-    <row r="6" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="G6" s="8">
         <v>2</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="I6" s="8">
         <v>0</v>
@@ -3591,46 +3586,46 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>6</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="G7" s="8">
         <v>3</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="I7" s="8"/>
       <c r="J7" s="8">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>6</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="G8" s="8">
         <v>1</v>
@@ -3641,7 +3636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -3653,7 +3648,7 @@
       <c r="I9" s="8"/>
       <c r="J9" s="8"/>
     </row>
-    <row r="10" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -3665,7 +3660,7 @@
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
     </row>
-    <row r="11" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -3677,7 +3672,7 @@
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
     </row>
-    <row r="12" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -3689,7 +3684,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -3701,7 +3696,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -3713,29 +3708,29 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="13" t="s">
-        <v>117</v>
+        <v>104</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <f>SUM(Tabelle2[Estimated time])</f>
         <v>13</v>
@@ -3778,57 +3773,57 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>111</v>
-      </c>
       <c r="G1" s="8" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45939</v>
       </c>
@@ -3836,22 +3831,22 @@
         <v>45953</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="G2" s="8">
         <v>2</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="I2" s="10">
         <v>5</v>
@@ -3860,39 +3855,39 @@
         <v>2</v>
       </c>
       <c r="K2" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="G3" s="8">
         <v>1</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="I3" s="8"/>
       <c r="J3" s="8">
         <v>1</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -3905,11 +3900,11 @@
       <c r="J4" s="8"/>
       <c r="K4" s="19"/>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>11</v>
@@ -3918,13 +3913,13 @@
         <v>12</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="G5" s="8">
         <v>5</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="I5" s="8">
         <v>8</v>
@@ -3934,11 +3929,11 @@
       </c>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>13</v>
@@ -3947,23 +3942,23 @@
         <v>14</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="G6" s="8">
         <v>4</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="I6" s="8">
         <v>5</v>
       </c>
       <c r="J6" s="8"/>
       <c r="K6" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -3976,7 +3971,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -3989,26 +3984,26 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="G9" s="8">
         <v>10</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="I9" s="8">
         <v>3</v>
@@ -4017,29 +4012,29 @@
         <v>15</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="G10" s="8">
         <v>15</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="I10" s="8">
         <v>3</v>
@@ -4048,37 +4043,37 @@
         <v>10</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="G11" s="8">
         <v>5</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
       <c r="K11" s="19" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4091,7 +4086,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="19"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4103,7 +4098,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4115,7 +4110,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -4127,29 +4122,29 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="13" t="s">
-        <v>117</v>
+        <v>104</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <f>SUM(Tabelle27[Estimated time])</f>
         <v>42</v>
@@ -4193,57 +4188,57 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>111</v>
-      </c>
       <c r="G1" s="8" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45953</v>
       </c>
@@ -4260,14 +4255,14 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>14</v>
@@ -4279,7 +4274,7 @@
         <v>5</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="I3" s="8">
         <v>3</v>
@@ -4288,29 +4283,29 @@
         <v>6</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="G4" s="8">
         <v>4</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="I4" s="8">
         <v>7</v>
@@ -4319,10 +4314,10 @@
         <v>4</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -4335,7 +4330,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -4348,7 +4343,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="19"/>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -4361,7 +4356,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -4374,7 +4369,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -4387,7 +4382,7 @@
       <c r="J9" s="8"/>
       <c r="K9" s="19"/>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -4400,7 +4395,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -4413,7 +4408,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4426,7 +4421,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="19"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4438,7 +4433,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4450,7 +4445,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -4462,29 +4457,29 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="13" t="s">
-        <v>117</v>
+        <v>104</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <f>SUM(Tabelle2710[Estimated time])</f>
         <v>9</v>
@@ -4528,57 +4523,57 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>111</v>
-      </c>
       <c r="G1" s="8" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45981</v>
       </c>
@@ -4595,26 +4590,26 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="G3" s="8">
         <v>10</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="I3" s="8">
         <v>8</v>
@@ -4623,23 +4618,23 @@
         <v>10</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="G4" s="8">
         <v>1</v>
@@ -4652,14 +4647,14 @@
         <v>1</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>11</v>
@@ -4668,7 +4663,7 @@
         <v>12</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="G5" s="8">
         <v>1</v>
@@ -4681,29 +4676,29 @@
         <v>1</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G6" s="8">
         <v>1</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="I6" s="8">
         <v>6</v>
@@ -4712,10 +4707,10 @@
         <v>2</v>
       </c>
       <c r="K6" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -4728,33 +4723,69 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="19"/>
-    </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="C8" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" s="8">
+        <v>4</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="I8" s="8">
+        <v>9</v>
+      </c>
+      <c r="J8" s="8">
+        <v>6</v>
+      </c>
+      <c r="K8" s="19" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="19"/>
-    </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="C9" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="G9" s="8">
+        <v>5</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="I9" s="8">
+        <v>4</v>
+      </c>
+      <c r="J9" s="8">
+        <v>4</v>
+      </c>
+      <c r="K9" s="19" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -4767,7 +4798,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -4780,7 +4811,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4792,7 +4823,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4804,7 +4835,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4816,49 +4847,49 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="13" t="s">
-        <v>117</v>
+        <v>104</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <f>SUM(Tabelle271013[Estimated time])</f>
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B16" s="12">
         <f>SUM(Tabelle271013[Time in Hours])</f>
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C16" s="12">
         <f>Tabelle381114[[#This Row],[Estimated time]]-Tabelle381114[[#This Row],[Actual time]]</f>
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="12">
         <f>SUM(Tabelle271013[Story points])</f>
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="F16" s="12">
         <f>Tabelle491215[[#This Row],[Total Storypoints ]]/Tabelle381114[[#This Row],[Actual time]]</f>
-        <v>1.8571428571428572</v>
+        <v>1.625</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
@@ -4880,19 +4911,19 @@
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" customWidth="1"/>
-    <col min="4" max="4" width="61.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" customWidth="1"/>
+    <col min="4" max="4" width="81.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -4909,14 +4940,14 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
       <c r="I1" s="17"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -4930,7 +4961,7 @@
         <v>8</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="F2" s="2">
         <v>5</v>
@@ -4940,21 +4971,21 @@
       </c>
       <c r="I2" s="17"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="C3" s="2">
         <v>2</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="F3" s="2">
         <v>8</v>
@@ -4964,7 +4995,7 @@
       </c>
       <c r="I3" s="17"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -4975,10 +5006,10 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="F4" s="2">
         <v>8</v>
@@ -4988,7 +5019,7 @@
       </c>
       <c r="I4" s="17"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -5002,7 +5033,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="F5" s="2">
         <v>5</v>
@@ -5012,7 +5043,7 @@
       </c>
       <c r="I5" s="17"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -5026,7 +5057,7 @@
         <v>17</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="F6" s="2">
         <v>4</v>
@@ -5036,7 +5067,7 @@
       </c>
       <c r="I6" s="17"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -5050,7 +5081,7 @@
         <v>20</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="F7" s="2">
         <v>6</v>
@@ -5060,18 +5091,18 @@
       </c>
       <c r="I7" s="17"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C8" s="2">
         <v>6</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>23</v>
+        <v>149</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>9</v>
@@ -5082,21 +5113,21 @@
       <c r="G8" s="2"/>
       <c r="I8" s="17"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C9" s="2">
         <v>5</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="F9" s="2">
         <v>4</v>
@@ -5106,399 +5137,384 @@
       </c>
       <c r="I9" s="17"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="C10" s="2">
+        <v>7</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="C10" s="2">
-        <v>8</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F10" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G10" s="2"/>
       <c r="I10" s="17"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="C11" s="2">
+        <v>3</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="2">
-        <v>7</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="F11" s="2">
-        <v>5</v>
-      </c>
-      <c r="G11" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G11" s="2">
+        <v>4</v>
+      </c>
       <c r="I11" s="17"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>34</v>
       </c>
       <c r="C12" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>35</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="F12" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G12" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I12" s="17"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C13" s="2">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F13" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G13" s="2"/>
       <c r="I13" s="17"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C14" s="2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>136</v>
+        <v>9</v>
       </c>
       <c r="F14" s="2">
-        <v>7</v>
-      </c>
-      <c r="G14" s="2">
-        <v>3</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="G14" s="2"/>
       <c r="I14" s="17"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F15" s="2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G15" s="2"/>
       <c r="I15" s="17"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C16" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F16" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G16" s="2"/>
       <c r="I16" s="17"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C17" s="2">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F17" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G17" s="2"/>
       <c r="I17" s="17"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C18" s="2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E18" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F18" s="2">
         <v>9</v>
       </c>
-      <c r="F18" s="2">
-        <v>6</v>
-      </c>
-      <c r="G18" s="2"/>
+      <c r="G18" s="2">
+        <v>4</v>
+      </c>
       <c r="I18" s="17"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C19" s="2">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F19" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G19" s="2"/>
       <c r="I19" s="17"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C20" s="2">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E20" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F20" s="2">
         <v>9</v>
       </c>
-      <c r="F20" s="2">
-        <v>5</v>
-      </c>
-      <c r="G20" s="2"/>
+      <c r="G20" s="2">
+        <v>4</v>
+      </c>
       <c r="I20" s="17"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C21" s="2">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>140</v>
+        <v>9</v>
       </c>
       <c r="F21" s="2">
-        <v>9</v>
-      </c>
-      <c r="G21" s="2">
-        <v>2</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G21" s="2"/>
       <c r="I21" s="17"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>64</v>
+        <v>143</v>
       </c>
       <c r="C22" s="2">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>65</v>
+        <v>144</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="F22" s="2">
         <v>4</v>
       </c>
-      <c r="G22" s="2"/>
+      <c r="G22" s="2">
+        <v>4</v>
+      </c>
       <c r="I22" s="17"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>67</v>
+        <v>146</v>
       </c>
       <c r="C23" s="2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>68</v>
+        <v>147</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F23" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G23" s="2"/>
       <c r="I23" s="17"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>70</v>
+        <v>145</v>
       </c>
       <c r="C24" s="2">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>71</v>
+        <v>148</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="F24" s="2">
-        <v>6</v>
-      </c>
-      <c r="G24" s="2"/>
-      <c r="I24" s="17"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="G24" s="2">
+        <v>4</v>
+      </c>
+      <c r="I24" s="20"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>73</v>
+        <v>150</v>
       </c>
       <c r="C25" s="2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>74</v>
+        <v>151</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F25" s="2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G25" s="2"/>
-      <c r="I25" s="17"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="C26" s="2">
-        <v>16</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F26" s="2">
-        <v>7</v>
-      </c>
-      <c r="G26" s="2"/>
-      <c r="I26" s="17"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A27" s="4"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4">
-        <f>SUM(F2:F26)</f>
-        <v>146</v>
-      </c>
-      <c r="G27" s="4"/>
+      <c r="I25" s="20"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" s="4"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4">
+        <f>SUM(F2:F24)</f>
+        <v>135</v>
+      </c>
+      <c r="G26" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat: Implement points system with fish tiers and costs
</commit_message>
<xml_diff>
--- a/aquasphere/Excel_File/AquaSphare.xlsx
+++ b/aquasphere/Excel_File/AquaSphare.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\43680\Desktop\Schule\SYP\Aquarium\aquasphere\Excel_File\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3A471DF-94A1-4F7A-ADE8-E33CA4A7D327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BAC59EE-EE84-497F-9500-514D19F5BB4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="5" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="157">
   <si>
     <t>Story ID</t>
   </si>
@@ -704,417 +704,6 @@
   </cellStyles>
   <dxfs count="128">
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="16"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.89999084444715716"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF0F9ED5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF0F9ED5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -2447,6 +2036,50 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
         <family val="2"/>
@@ -2461,6 +2094,67 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2491,6 +2185,200 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
         <family val="2"/>
@@ -2505,7 +2393,11 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -2525,18 +2417,21 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -2546,6 +2441,30 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -2566,6 +2485,67 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2796,6 +2776,26 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -2977,11 +2977,11 @@
     <tableColumn id="4" xr3:uid="{D6FF0659-1B35-4F09-B5A7-D22FEF5F7C3F}" name="Accomplished Story Points" dataDxfId="121">
       <calculatedColumnFormula array="1">Tabelle4[[Total Storypoints ]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{9CD2DBE3-2E45-4440-8D7A-2A03A0291AAD}" name="Velocity" dataDxfId="0">
+    <tableColumn id="5" xr3:uid="{9CD2DBE3-2E45-4440-8D7A-2A03A0291AAD}" name="Velocity" dataDxfId="120">
       <calculatedColumnFormula>Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{1977DF7A-0A05-43B5-99D3-B72159480780}" name="Total Storypoints" dataDxfId="120"/>
-    <tableColumn id="7" xr3:uid="{D8A5F5FE-B9BC-448A-A9E7-3D00888AE639}" name="Storypoints Left" dataDxfId="119">
+    <tableColumn id="6" xr3:uid="{1977DF7A-0A05-43B5-99D3-B72159480780}" name="Total Storypoints" dataDxfId="119"/>
+    <tableColumn id="7" xr3:uid="{D8A5F5FE-B9BC-448A-A9E7-3D00888AE639}" name="Storypoints Left" dataDxfId="118">
       <calculatedColumnFormula>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2990,13 +2990,13 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0134C802-458D-4153-B0D4-D8B08E02E26A}" name="Tabelle4912" displayName="Tabelle4912" ref="E16:F17" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0134C802-458D-4153-B0D4-D8B08E02E26A}" name="Tabelle4912" displayName="Tabelle4912" ref="E16:F17" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="E16:F17" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C3438C75-AD69-46E0-B1BD-0445ED469483}" name="Total Storypoints " dataDxfId="55">
+    <tableColumn id="1" xr3:uid="{C3438C75-AD69-46E0-B1BD-0445ED469483}" name="Total Storypoints " dataDxfId="54">
       <calculatedColumnFormula>SUM(Tabelle2710[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0655740B-E1AB-4BD3-B7CA-852D4C79FC17}" name="Effort/Hour" dataDxfId="54">
+    <tableColumn id="2" xr3:uid="{0655740B-E1AB-4BD3-B7CA-852D4C79FC17}" name="Effort/Hour" dataDxfId="53">
       <calculatedColumnFormula>Tabelle4912[[#This Row],[Total Storypoints ]]/Tabelle3811[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3005,36 +3005,36 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}" name="Tabelle271013" displayName="Tabelle271013" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}" name="Tabelle271013" displayName="Tabelle271013" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
   <autoFilter ref="A1:K11" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{946A4B14-799A-49AD-8E3E-31E3F4BBE559}" name="Sprint Start" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{E61A962F-4EE4-4843-AF21-C647918EECAB}" name="Sprint End" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{4EC50B40-18BD-4D00-8BE2-5596A9347BB8}" name="User" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{2A1F175E-D14E-491C-B452-39567CF84CD6}" name="ID" dataDxfId="48"/>
-    <tableColumn id="6" xr3:uid="{DCE5121F-D243-470B-B0AF-D0EE5264DD5A}" name="Epic" dataDxfId="47"/>
-    <tableColumn id="12" xr3:uid="{45FDCCAE-F13D-47C1-B91E-2EF3CC9A5BA0}" name="User Story /Task" dataDxfId="46"/>
-    <tableColumn id="11" xr3:uid="{4057DF12-8977-4284-BF2B-9ED3AAE7221F}" name="Estimated time" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{08443A2E-5832-4299-8009-1F0D489DEE15}" name="COS (Criteria of Satisfaction)" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{8777A429-C11B-4CDC-BB2F-785D0BC89DAB}" name="Story points" dataDxfId="43"/>
-    <tableColumn id="10" xr3:uid="{0B18443F-D8D9-4015-8EAA-7050016E43C2}" name="Time in Hours" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{5C5B5C91-6376-4597-B69B-4D162307C569}" name="Status" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{946A4B14-799A-49AD-8E3E-31E3F4BBE559}" name="Sprint Start" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{E61A962F-4EE4-4843-AF21-C647918EECAB}" name="Sprint End" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{4EC50B40-18BD-4D00-8BE2-5596A9347BB8}" name="User" dataDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{2A1F175E-D14E-491C-B452-39567CF84CD6}" name="ID" dataDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{DCE5121F-D243-470B-B0AF-D0EE5264DD5A}" name="Epic" dataDxfId="46"/>
+    <tableColumn id="12" xr3:uid="{45FDCCAE-F13D-47C1-B91E-2EF3CC9A5BA0}" name="User Story /Task" dataDxfId="45"/>
+    <tableColumn id="11" xr3:uid="{4057DF12-8977-4284-BF2B-9ED3AAE7221F}" name="Estimated time" dataDxfId="44"/>
+    <tableColumn id="8" xr3:uid="{08443A2E-5832-4299-8009-1F0D489DEE15}" name="COS (Criteria of Satisfaction)" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{8777A429-C11B-4CDC-BB2F-785D0BC89DAB}" name="Story points" dataDxfId="42"/>
+    <tableColumn id="10" xr3:uid="{0B18443F-D8D9-4015-8EAA-7050016E43C2}" name="Time in Hours" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{5C5B5C91-6376-4597-B69B-4D162307C569}" name="Status" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}" name="Tabelle381114" displayName="Tabelle381114" ref="A15:C16" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}" name="Tabelle381114" displayName="Tabelle381114" ref="A15:C16" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
   <autoFilter ref="A15:C16" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{E71994D0-AB06-482B-8487-03AB7E3B1FF7}" name="Estimated time" dataDxfId="38">
+    <tableColumn id="1" xr3:uid="{E71994D0-AB06-482B-8487-03AB7E3B1FF7}" name="Estimated time" dataDxfId="37">
       <calculatedColumnFormula>SUM(Tabelle271013[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E607785B-5B58-4D1E-81ED-45AAAAF488F0}" name="Actual time" dataDxfId="37">
+    <tableColumn id="2" xr3:uid="{E607785B-5B58-4D1E-81ED-45AAAAF488F0}" name="Actual time" dataDxfId="36">
       <calculatedColumnFormula>SUM(Tabelle271013[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{0197CFBA-597E-49C6-88E5-ABAC17763EA4}" name="Delta" dataDxfId="36">
+    <tableColumn id="3" xr3:uid="{0197CFBA-597E-49C6-88E5-ABAC17763EA4}" name="Delta" dataDxfId="35">
       <calculatedColumnFormula>Tabelle381114[[#This Row],[Estimated time]]-Tabelle381114[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3043,13 +3043,13 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}" name="Tabelle491215" displayName="Tabelle491215" ref="E15:F16" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}" name="Tabelle491215" displayName="Tabelle491215" ref="E15:F16" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <autoFilter ref="E15:F16" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{E0381C51-E5FF-4087-9146-76E105FE701A}" name="Total Storypoints " dataDxfId="33">
+    <tableColumn id="1" xr3:uid="{E0381C51-E5FF-4087-9146-76E105FE701A}" name="Total Storypoints " dataDxfId="32">
       <calculatedColumnFormula>SUM(Tabelle271013[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0971B46C-CFAA-4F13-88AB-CDC5655C1F84}" name="Effort/Hour" dataDxfId="32">
+    <tableColumn id="2" xr3:uid="{0971B46C-CFAA-4F13-88AB-CDC5655C1F84}" name="Effort/Hour" dataDxfId="31">
       <calculatedColumnFormula>Tabelle491215[[#This Row],[Total Storypoints ]]/Tabelle381114[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3058,36 +3058,36 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{235F589F-8BC0-4A3D-A02E-03E630D61504}" name="Tabelle27101316" displayName="Tabelle27101316" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{235F589F-8BC0-4A3D-A02E-03E630D61504}" name="Tabelle27101316" displayName="Tabelle27101316" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
   <autoFilter ref="A1:K11" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{B7D16283-E8F5-4C03-BEC2-39D9F536B2DF}" name="Sprint Start" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{743B7730-744D-48F9-8435-134B358D299C}" name="Sprint End" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{6BB0BFF2-8337-4911-B853-52953695FFB8}" name="User" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{23B9485C-C756-4653-9A7E-4CBFBC4BDCC9}" name="ID" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{DA3B151D-2F3B-4817-810C-2B84F6D521DF}" name="Epic" dataDxfId="16"/>
-    <tableColumn id="12" xr3:uid="{0B21ADB3-F002-4AC8-8EFB-36998E0BA400}" name="User Story /Task" dataDxfId="15"/>
-    <tableColumn id="11" xr3:uid="{0AF7F7D2-16D8-4903-AFB0-E002FAFE9A7B}" name="Estimated time" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{2F945FB5-B8D6-4015-9863-4264314B3D66}" name="COS (Criteria of Satisfaction)" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{72841B6A-9C3A-4632-878E-ADBD76467B91}" name="Story points" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{99643A57-EC89-4FC7-B6E0-CEECFE14CE6B}" name="Time in Hours" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{D3F46A45-6C79-4B7E-9924-30DF1A278D97}" name="Status" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{B7D16283-E8F5-4C03-BEC2-39D9F536B2DF}" name="Sprint Start" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{743B7730-744D-48F9-8435-134B358D299C}" name="Sprint End" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{6BB0BFF2-8337-4911-B853-52953695FFB8}" name="User" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{23B9485C-C756-4653-9A7E-4CBFBC4BDCC9}" name="ID" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{DA3B151D-2F3B-4817-810C-2B84F6D521DF}" name="Epic" dataDxfId="24"/>
+    <tableColumn id="12" xr3:uid="{0B21ADB3-F002-4AC8-8EFB-36998E0BA400}" name="User Story /Task" dataDxfId="23"/>
+    <tableColumn id="11" xr3:uid="{0AF7F7D2-16D8-4903-AFB0-E002FAFE9A7B}" name="Estimated time" dataDxfId="22"/>
+    <tableColumn id="8" xr3:uid="{2F945FB5-B8D6-4015-9863-4264314B3D66}" name="COS (Criteria of Satisfaction)" dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{72841B6A-9C3A-4632-878E-ADBD76467B91}" name="Story points" dataDxfId="20"/>
+    <tableColumn id="10" xr3:uid="{99643A57-EC89-4FC7-B6E0-CEECFE14CE6B}" name="Time in Hours" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{D3F46A45-6C79-4B7E-9924-30DF1A278D97}" name="Status" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{E0805314-F662-4E1D-85A9-F2EC30EC262D}" name="Tabelle38111417" displayName="Tabelle38111417" ref="A15:C16" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{E0805314-F662-4E1D-85A9-F2EC30EC262D}" name="Tabelle38111417" displayName="Tabelle38111417" ref="A15:C16" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="A15:C16" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{1993629C-98D2-4E46-B14A-696AAE563315}" name="Estimated time" dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{1993629C-98D2-4E46-B14A-696AAE563315}" name="Estimated time" dataDxfId="15">
       <calculatedColumnFormula>SUM(Tabelle27101316[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C3F5A116-86A6-4D3A-9417-88FA122B0C81}" name="Actual time" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{C3F5A116-86A6-4D3A-9417-88FA122B0C81}" name="Actual time" dataDxfId="14">
       <calculatedColumnFormula>SUM(Tabelle27101316[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B86C31E6-5405-4B45-9B86-86A0C1DBF35C}" name="Delta" dataDxfId="5">
+    <tableColumn id="3" xr3:uid="{B86C31E6-5405-4B45-9B86-86A0C1DBF35C}" name="Delta" dataDxfId="13">
       <calculatedColumnFormula>Tabelle38111417[[#This Row],[Estimated time]]-Tabelle38111417[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3096,13 +3096,13 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{FE78B35D-B1A7-42FC-BB42-AF310800AF69}" name="Tabelle49121518" displayName="Tabelle49121518" ref="E15:F16" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{FE78B35D-B1A7-42FC-BB42-AF310800AF69}" name="Tabelle49121518" displayName="Tabelle49121518" ref="E15:F16" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="E15:F16" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{E7934959-5DF7-4D4C-858C-1FAD310B1F3B}" name="Total Storypoints " dataDxfId="2">
+    <tableColumn id="1" xr3:uid="{E7934959-5DF7-4D4C-858C-1FAD310B1F3B}" name="Total Storypoints " dataDxfId="10">
       <calculatedColumnFormula>SUM(Tabelle27101316[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D7E6F4E2-872C-4E38-9126-8A958E19087E}" name="Effort/Hour" dataDxfId="1">
+    <tableColumn id="2" xr3:uid="{D7E6F4E2-872C-4E38-9126-8A958E19087E}" name="Effort/Hour" dataDxfId="9">
       <calculatedColumnFormula>Tabelle49121518[[#This Row],[Total Storypoints ]]/Tabelle38111417[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3111,54 +3111,54 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:G26" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:G26" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <autoFilter ref="A1:G26" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G26">
     <sortCondition ref="C9:C26"/>
   </sortState>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Effort" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Effort" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}" name="Tabelle2" displayName="Tabelle2" ref="A1:J9" insertRowShift="1" totalsRowShown="0" headerRowDxfId="118" dataDxfId="117">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}" name="Tabelle2" displayName="Tabelle2" ref="A1:J9" insertRowShift="1" totalsRowShown="0" headerRowDxfId="117" dataDxfId="116">
   <autoFilter ref="A1:J9" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{0351E8C1-0BB8-4C19-A406-233CC12328E5}" name="Sprint Start" dataDxfId="116"/>
-    <tableColumn id="2" xr3:uid="{51BD2FE0-507A-4398-BD96-E186E78BB2C7}" name="Sprint End" dataDxfId="115"/>
-    <tableColumn id="3" xr3:uid="{A3B7E86B-E01A-4D78-82AD-BA81F6AC7ADF}" name="User" dataDxfId="114"/>
-    <tableColumn id="5" xr3:uid="{CE780601-F45C-4063-B216-98ACE5588903}" name="ID" dataDxfId="113"/>
-    <tableColumn id="6" xr3:uid="{A14D049D-AC5C-49A5-A7CC-A4D5ED8A8330}" name="Epic" dataDxfId="112"/>
-    <tableColumn id="12" xr3:uid="{770F10A6-830A-41AC-B069-6267CAE00BDF}" name="User Story /Task" dataDxfId="111"/>
-    <tableColumn id="11" xr3:uid="{0D9AB552-F7B4-4231-A35B-245B57383919}" name="Estimated time" dataDxfId="110"/>
-    <tableColumn id="8" xr3:uid="{3E2E3644-9002-4AB9-B3EC-96FFF84D8900}" name="COS (Criteria of Satisfaction)" dataDxfId="109"/>
-    <tableColumn id="9" xr3:uid="{14C8E3A9-BC37-48D9-A399-32A48A46993A}" name="Story points" dataDxfId="108"/>
-    <tableColumn id="10" xr3:uid="{151786D9-5F15-42D7-932B-664A024F4131}" name="Time in Hours" dataDxfId="107"/>
+    <tableColumn id="1" xr3:uid="{0351E8C1-0BB8-4C19-A406-233CC12328E5}" name="Sprint Start" dataDxfId="115"/>
+    <tableColumn id="2" xr3:uid="{51BD2FE0-507A-4398-BD96-E186E78BB2C7}" name="Sprint End" dataDxfId="114"/>
+    <tableColumn id="3" xr3:uid="{A3B7E86B-E01A-4D78-82AD-BA81F6AC7ADF}" name="User" dataDxfId="113"/>
+    <tableColumn id="5" xr3:uid="{CE780601-F45C-4063-B216-98ACE5588903}" name="ID" dataDxfId="112"/>
+    <tableColumn id="6" xr3:uid="{A14D049D-AC5C-49A5-A7CC-A4D5ED8A8330}" name="Epic" dataDxfId="111"/>
+    <tableColumn id="12" xr3:uid="{770F10A6-830A-41AC-B069-6267CAE00BDF}" name="User Story /Task" dataDxfId="110"/>
+    <tableColumn id="11" xr3:uid="{0D9AB552-F7B4-4231-A35B-245B57383919}" name="Estimated time" dataDxfId="109"/>
+    <tableColumn id="8" xr3:uid="{3E2E3644-9002-4AB9-B3EC-96FFF84D8900}" name="COS (Criteria of Satisfaction)" dataDxfId="108"/>
+    <tableColumn id="9" xr3:uid="{14C8E3A9-BC37-48D9-A399-32A48A46993A}" name="Story points" dataDxfId="107"/>
+    <tableColumn id="10" xr3:uid="{151786D9-5F15-42D7-932B-664A024F4131}" name="Time in Hours" dataDxfId="106"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}" name="Tabelle3" displayName="Tabelle3" ref="A15:C16" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}" name="Tabelle3" displayName="Tabelle3" ref="A15:C16" totalsRowShown="0" headerRowDxfId="105" dataDxfId="104">
   <autoFilter ref="A15:C16" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CD2D4D96-DD34-4EA3-92D7-B02BB9DE5647}" name="Estimated time" dataDxfId="104">
+    <tableColumn id="1" xr3:uid="{CD2D4D96-DD34-4EA3-92D7-B02BB9DE5647}" name="Estimated time" dataDxfId="103">
       <calculatedColumnFormula>SUM(Tabelle2[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0F14E190-6E0A-4AB8-8ADE-83875E98D4B5}" name="Actual time" dataDxfId="103">
+    <tableColumn id="2" xr3:uid="{0F14E190-6E0A-4AB8-8ADE-83875E98D4B5}" name="Actual time" dataDxfId="102">
       <calculatedColumnFormula>SUM(Tabelle2[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{5DE18543-F4D3-4732-9F2D-5B7F140CB974}" name="Delta" dataDxfId="102">
+    <tableColumn id="3" xr3:uid="{5DE18543-F4D3-4732-9F2D-5B7F140CB974}" name="Delta" dataDxfId="101">
       <calculatedColumnFormula>Tabelle3[[#This Row],[Estimated time]]-Tabelle3[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3167,13 +3167,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}" name="Tabelle4" displayName="Tabelle4" ref="E15:F16" totalsRowShown="0" headerRowDxfId="101" dataDxfId="100">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}" name="Tabelle4" displayName="Tabelle4" ref="E15:F16" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
   <autoFilter ref="E15:F16" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{2E187AEA-682F-4749-9FC8-ED3BA3DE1DA2}" name="Total Storypoints " dataDxfId="99">
+    <tableColumn id="1" xr3:uid="{2E187AEA-682F-4749-9FC8-ED3BA3DE1DA2}" name="Total Storypoints " dataDxfId="98">
       <calculatedColumnFormula>SUM(Tabelle2[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3C6DC8F5-724A-43AC-9128-7661A96380C1}" name="Efford/Hour" dataDxfId="98">
+    <tableColumn id="2" xr3:uid="{3C6DC8F5-724A-43AC-9128-7661A96380C1}" name="Efford/Hour" dataDxfId="97">
       <calculatedColumnFormula>Tabelle4[[#This Row],[Total Storypoints ]]/Tabelle3[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3182,36 +3182,36 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A211D33B-248F-4E66-AF7C-9632EAA38DAC}" name="Tabelle27" displayName="Tabelle27" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="97" dataDxfId="96">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A211D33B-248F-4E66-AF7C-9632EAA38DAC}" name="Tabelle27" displayName="Tabelle27" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="96" dataDxfId="95">
   <autoFilter ref="A1:K12" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{9C36A560-9153-4D8E-BA50-0044E74E1896}" name="Sprint Start" dataDxfId="95"/>
-    <tableColumn id="2" xr3:uid="{4FAB3106-8621-41F1-B866-EA5558F083D8}" name="Sprint End" dataDxfId="94"/>
-    <tableColumn id="3" xr3:uid="{2D2022CC-B165-4671-9773-4C7DCE737FC7}" name="User" dataDxfId="93"/>
-    <tableColumn id="5" xr3:uid="{6D49D607-DA69-4FF5-AC26-260E9F796217}" name="ID" dataDxfId="92"/>
-    <tableColumn id="6" xr3:uid="{95077F2F-115F-484E-A38C-A34A2BCBCB78}" name="Epic" dataDxfId="91"/>
-    <tableColumn id="12" xr3:uid="{2EAFDE91-2C58-4973-A684-28E2E964F629}" name="User Story /Task" dataDxfId="90"/>
-    <tableColumn id="11" xr3:uid="{D17AAC02-918A-4F08-B037-3622F37B62F0}" name="Estimated time" dataDxfId="89"/>
-    <tableColumn id="8" xr3:uid="{4D053EE2-698A-4191-ABEB-8F0701DA4D4E}" name="COS (Criteria of Satisfaction)" dataDxfId="88"/>
-    <tableColumn id="9" xr3:uid="{73BF0134-792D-4614-95FB-754C4A317665}" name="Story points" dataDxfId="87"/>
-    <tableColumn id="10" xr3:uid="{2620A9CC-A288-4874-BF27-2BBE69671B14}" name="Time in Hours" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="85"/>
+    <tableColumn id="1" xr3:uid="{9C36A560-9153-4D8E-BA50-0044E74E1896}" name="Sprint Start" dataDxfId="94"/>
+    <tableColumn id="2" xr3:uid="{4FAB3106-8621-41F1-B866-EA5558F083D8}" name="Sprint End" dataDxfId="93"/>
+    <tableColumn id="3" xr3:uid="{2D2022CC-B165-4671-9773-4C7DCE737FC7}" name="User" dataDxfId="92"/>
+    <tableColumn id="5" xr3:uid="{6D49D607-DA69-4FF5-AC26-260E9F796217}" name="ID" dataDxfId="91"/>
+    <tableColumn id="6" xr3:uid="{95077F2F-115F-484E-A38C-A34A2BCBCB78}" name="Epic" dataDxfId="90"/>
+    <tableColumn id="12" xr3:uid="{2EAFDE91-2C58-4973-A684-28E2E964F629}" name="User Story /Task" dataDxfId="89"/>
+    <tableColumn id="11" xr3:uid="{D17AAC02-918A-4F08-B037-3622F37B62F0}" name="Estimated time" dataDxfId="88"/>
+    <tableColumn id="8" xr3:uid="{4D053EE2-698A-4191-ABEB-8F0701DA4D4E}" name="COS (Criteria of Satisfaction)" dataDxfId="87"/>
+    <tableColumn id="9" xr3:uid="{73BF0134-792D-4614-95FB-754C4A317665}" name="Story points" dataDxfId="86"/>
+    <tableColumn id="10" xr3:uid="{2620A9CC-A288-4874-BF27-2BBE69671B14}" name="Time in Hours" dataDxfId="85"/>
+    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="84"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="83" dataDxfId="82">
   <autoFilter ref="A16:C17" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="82">
+    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="81">
       <calculatedColumnFormula>SUM(Tabelle27[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="81">
+    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="80">
       <calculatedColumnFormula>SUM(Tabelle27[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="80">
+    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="79">
       <calculatedColumnFormula>Tabelle38[[#This Row],[Estimated time]]-Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3220,13 +3220,13 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
   <autoFilter ref="E16:F17" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="77">
+    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="76">
       <calculatedColumnFormula>SUM(Tabelle27[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="76">
+    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="75">
       <calculatedColumnFormula>Tabelle49[[#This Row],[Total Storypoints ]]/Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3235,36 +3235,36 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6303AB7F-CDC2-408B-A450-96D692A68B43}" name="Tabelle2710" displayName="Tabelle2710" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6303AB7F-CDC2-408B-A450-96D692A68B43}" name="Tabelle2710" displayName="Tabelle2710" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="74" dataDxfId="73">
   <autoFilter ref="A1:K12" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{949CA967-02A0-4249-BB07-B02F4C4F69AE}" name="Sprint Start" dataDxfId="73"/>
-    <tableColumn id="2" xr3:uid="{A70AE104-D3DD-4C6E-8E50-E151404B19BD}" name="Sprint End" dataDxfId="72"/>
-    <tableColumn id="3" xr3:uid="{9168C6BE-6970-4420-9D5F-DBCF1E8E2BAE}" name="User" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{A7C4968E-9480-42FF-949B-9E41609C26A2}" name="ID" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{8564B7DD-8DB4-4E2B-BDDB-9791D9AAA0EA}" name="Epic" dataDxfId="69"/>
-    <tableColumn id="12" xr3:uid="{56FA47CB-3810-4B7F-A047-8358D5C73F6C}" name="User Story /Task" dataDxfId="68"/>
-    <tableColumn id="11" xr3:uid="{988CB3AF-F268-445B-887C-5163D9AE41DF}" name="Estimated time" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{14BDCFB4-F75D-4798-AFF3-3F8B177B78D6}" name="COS (Criteria of Satisfaction)" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{97C18CBF-2D3F-4A8A-B36D-6328E17F31C4}" name="Story points" dataDxfId="65"/>
-    <tableColumn id="10" xr3:uid="{D3E339CF-38BF-4AC1-8C80-41ECD30B6907}" name="Time in Hours" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{3BCBC0DA-7C9B-4D2B-9269-A319CBD925C5}" name="Status" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{949CA967-02A0-4249-BB07-B02F4C4F69AE}" name="Sprint Start" dataDxfId="72"/>
+    <tableColumn id="2" xr3:uid="{A70AE104-D3DD-4C6E-8E50-E151404B19BD}" name="Sprint End" dataDxfId="71"/>
+    <tableColumn id="3" xr3:uid="{9168C6BE-6970-4420-9D5F-DBCF1E8E2BAE}" name="User" dataDxfId="70"/>
+    <tableColumn id="5" xr3:uid="{A7C4968E-9480-42FF-949B-9E41609C26A2}" name="ID" dataDxfId="69"/>
+    <tableColumn id="6" xr3:uid="{8564B7DD-8DB4-4E2B-BDDB-9791D9AAA0EA}" name="Epic" dataDxfId="68"/>
+    <tableColumn id="12" xr3:uid="{56FA47CB-3810-4B7F-A047-8358D5C73F6C}" name="User Story /Task" dataDxfId="67"/>
+    <tableColumn id="11" xr3:uid="{988CB3AF-F268-445B-887C-5163D9AE41DF}" name="Estimated time" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{14BDCFB4-F75D-4798-AFF3-3F8B177B78D6}" name="COS (Criteria of Satisfaction)" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{97C18CBF-2D3F-4A8A-B36D-6328E17F31C4}" name="Story points" dataDxfId="64"/>
+    <tableColumn id="10" xr3:uid="{D3E339CF-38BF-4AC1-8C80-41ECD30B6907}" name="Time in Hours" dataDxfId="63"/>
+    <tableColumn id="4" xr3:uid="{3BCBC0DA-7C9B-4D2B-9269-A319CBD925C5}" name="Status" dataDxfId="62"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C1E761E2-D340-4C7F-A19A-AE84A76F5971}" name="Tabelle3811" displayName="Tabelle3811" ref="A16:C17" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C1E761E2-D340-4C7F-A19A-AE84A76F5971}" name="Tabelle3811" displayName="Tabelle3811" ref="A16:C17" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60">
   <autoFilter ref="A16:C17" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{F045D4AD-2D00-44A7-8EA7-B5C34869B26F}" name="Estimated time" dataDxfId="60">
+    <tableColumn id="1" xr3:uid="{F045D4AD-2D00-44A7-8EA7-B5C34869B26F}" name="Estimated time" dataDxfId="59">
       <calculatedColumnFormula>SUM(Tabelle2710[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DFDFE0A8-6207-4F3B-9D05-4D3AF083E31B}" name="Actual time" dataDxfId="59">
+    <tableColumn id="2" xr3:uid="{DFDFE0A8-6207-4F3B-9D05-4D3AF083E31B}" name="Actual time" dataDxfId="58">
       <calculatedColumnFormula>SUM(Tabelle2710[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{2529739A-9C5E-4AE4-80A6-DFC080EFE2D8}" name="Delta" dataDxfId="58">
+    <tableColumn id="3" xr3:uid="{2529739A-9C5E-4AE4-80A6-DFC080EFE2D8}" name="Delta" dataDxfId="57">
       <calculatedColumnFormula>Tabelle3811[[#This Row],[Estimated time]]-Tabelle3811[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3771,15 +3771,15 @@
       </c>
       <c r="D6" s="7" cm="1">
         <f t="array" ref="D6">Tabelle38111417[Actual time]</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E6" s="7" cm="1">
         <f t="array" ref="E6">Tabelle49121518[[Total Storypoints ]]</f>
         <v>8</v>
       </c>
-      <c r="F6" s="7" t="e">
+      <c r="F6" s="7">
         <f>Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]]</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="G6" s="7">
         <f>H5</f>
@@ -3844,9 +3844,9 @@
       <c r="B15" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C15" s="5" t="e">
+      <c r="C15" s="5">
         <f>AVERAGE(Tabelle1[Velocity])</f>
-        <v>#DIV/0!</v>
+        <v>0.86617647058823533</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
@@ -3862,13 +3862,13 @@
       <c r="B17" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="18" t="e">
+      <c r="C17" s="18">
         <f>C13/C15</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D17" t="e">
+        <v>75.042444821731749</v>
+      </c>
+      <c r="D17">
         <f>C17/4</f>
-        <v>#DIV/0!</v>
+        <v>18.760611205432937</v>
       </c>
     </row>
   </sheetData>
@@ -5461,8 +5461,12 @@
       <c r="I3" s="8">
         <v>8</v>
       </c>
-      <c r="J3" s="8"/>
-      <c r="K3" s="19"/>
+      <c r="J3" s="8">
+        <v>8</v>
+      </c>
+      <c r="K3" s="19" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="8"/>
@@ -5633,20 +5637,20 @@
       </c>
       <c r="B16" s="12">
         <f>SUM(Tabelle27101316[Time in Hours])</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C16" s="12">
         <f>Tabelle38111417[[#This Row],[Estimated time]]-Tabelle38111417[[#This Row],[Actual time]]</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="12">
         <f>SUM(Tabelle27101316[Story points])</f>
         <v>8</v>
       </c>
-      <c r="F16" s="12" t="e">
+      <c r="F16" s="12">
         <f>Tabelle49121518[[#This Row],[Total Storypoints ]]/Tabelle38111417[[#This Row],[Actual time]]</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
@@ -5655,10 +5659,11 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="3">
-    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
edited excel, added dirt and cleaning
</commit_message>
<xml_diff>
--- a/aquasphere/Excel_File/AquaSphare.xlsx
+++ b/aquasphere/Excel_File/AquaSphare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\43680\Desktop\Schule\SYP\Aquarium\aquasphere\Excel_File\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielhoheneder/Desktop/Schule/syp/AquaSphere/aquasphere/Excel_File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BAC59EE-EE84-497F-9500-514D19F5BB4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA7D020-B382-A94A-A63B-681770F8748B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="5" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="25820" windowHeight="15500" activeTab="5" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Dashboard" sheetId="2" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="159">
   <si>
     <t>Story ID</t>
   </si>
@@ -534,7 +534,13 @@
     <t>Punktesystem</t>
   </si>
   <si>
-    <t>Ein Punktesystem ist implementiert, Preise und "einkommen" sind deviniert</t>
+    <t>Ein Punktesystem ist implementiert, Preise und "einkommen" sind definiert</t>
+  </si>
+  <si>
+    <t>AQ22</t>
+  </si>
+  <si>
+    <t>Schmutz muss entstehen und sichtbar sein. User kann über reinigen button oder mit einem Brush tool das Aquarium reinigen</t>
   </si>
 </sst>
 </file>
@@ -699,8 +705,8 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Prozent" xfId="1" builtinId="5"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="128">
     <dxf>
@@ -3593,20 +3599,20 @@
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:H17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>5</v>
       </c>
@@ -3632,7 +3638,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>70</v>
       </c>
@@ -3663,7 +3669,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>71</v>
       </c>
@@ -3694,7 +3700,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>72</v>
       </c>
@@ -3726,7 +3732,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>73</v>
       </c>
@@ -3758,7 +3764,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>74</v>
       </c>
@@ -3767,15 +3773,15 @@
       </c>
       <c r="C6" s="7" cm="1">
         <f t="array" ref="C6">Tabelle38111417[Estimated time]</f>
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D6" s="7" cm="1">
         <f t="array" ref="D6">Tabelle38111417[Actual time]</f>
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E6" s="7" cm="1">
         <f t="array" ref="E6">Tabelle49121518[[Total Storypoints ]]</f>
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F6" s="7">
         <f>Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]]</f>
@@ -3787,10 +3793,10 @@
       </c>
       <c r="H6" s="7">
         <f>C13</f>
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>75</v>
       </c>
@@ -3802,7 +3808,7 @@
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>76</v>
       </c>
@@ -3814,7 +3820,7 @@
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
     </row>
-    <row r="12" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>77</v>
       </c>
@@ -3822,16 +3828,16 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>118</v>
       </c>
       <c r="C13" s="5">
         <f>C12-SUM(Tabelle1[Accomplished Story Points])</f>
-        <v>65</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>81</v>
       </c>
@@ -3840,7 +3846,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>78</v>
       </c>
@@ -3849,26 +3855,26 @@
         <v>0.86617647058823533</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>79</v>
       </c>
       <c r="C16" s="14">
         <f>(SUM(Tabelle1[Accomplished Story Points],)/G2)</f>
-        <v>0.5547945205479452</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>0.58904109589041098</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" ht="24" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>69</v>
       </c>
       <c r="C17" s="18">
         <f>C13/C15</f>
-        <v>75.042444821731749</v>
+        <v>69.269949066213925</v>
       </c>
       <c r="D17">
         <f>C17/4</f>
-        <v>18.760611205432937</v>
+        <v>17.317487266553481</v>
       </c>
     </row>
   </sheetData>
@@ -3886,21 +3892,21 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:J16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="95.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="95.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>83</v>
       </c>
@@ -3932,7 +3938,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45925</v>
       </c>
@@ -3962,7 +3968,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -3984,7 +3990,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -4004,7 +4010,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -4016,7 +4022,7 @@
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
     </row>
-    <row r="6" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -4044,7 +4050,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
@@ -4070,7 +4076,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
@@ -4094,7 +4100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -4106,7 +4112,7 @@
       <c r="I9" s="8"/>
       <c r="J9" s="8"/>
     </row>
-    <row r="10" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -4118,7 +4124,7 @@
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
     </row>
-    <row r="11" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -4130,7 +4136,7 @@
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
     </row>
-    <row r="12" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4142,7 +4148,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4154,7 +4160,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4166,7 +4172,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>93</v>
       </c>
@@ -4188,7 +4194,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <f>SUM(Tabelle2[Estimated time])</f>
         <v>13</v>
@@ -4231,22 +4237,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>83</v>
       </c>
@@ -4281,7 +4287,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45939</v>
       </c>
@@ -4316,7 +4322,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -4345,7 +4351,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -4358,7 +4364,7 @@
       <c r="J4" s="8"/>
       <c r="K4" s="19"/>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
@@ -4387,7 +4393,7 @@
       </c>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -4416,7 +4422,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -4429,7 +4435,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -4442,7 +4448,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
@@ -4473,7 +4479,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8" t="s">
@@ -4504,7 +4510,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8" t="s">
@@ -4531,7 +4537,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4544,7 +4550,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="19"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4556,7 +4562,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4568,7 +4574,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -4580,7 +4586,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>93</v>
       </c>
@@ -4602,7 +4608,7 @@
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <f>SUM(Tabelle27[Estimated time])</f>
         <v>42</v>
@@ -4646,22 +4652,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>83</v>
       </c>
@@ -4696,7 +4702,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45953</v>
       </c>
@@ -4713,7 +4719,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -4744,7 +4750,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -4775,7 +4781,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -4788,7 +4794,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -4801,7 +4807,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="19"/>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -4814,7 +4820,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -4827,7 +4833,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -4840,7 +4846,7 @@
       <c r="J9" s="8"/>
       <c r="K9" s="19"/>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -4853,7 +4859,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -4866,7 +4872,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4879,7 +4885,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="19"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4891,7 +4897,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4903,7 +4909,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -4915,7 +4921,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>93</v>
       </c>
@@ -4937,7 +4943,7 @@
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <f>SUM(Tabelle2710[Estimated time])</f>
         <v>9</v>
@@ -4981,22 +4987,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>83</v>
       </c>
@@ -5031,7 +5037,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45981</v>
       </c>
@@ -5048,7 +5054,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -5079,7 +5085,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -5108,7 +5114,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
@@ -5137,7 +5143,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -5168,7 +5174,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -5181,7 +5187,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
@@ -5212,7 +5218,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
@@ -5243,7 +5249,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -5256,7 +5262,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -5269,7 +5275,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -5281,7 +5287,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -5293,7 +5299,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -5305,7 +5311,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>93</v>
       </c>
@@ -5327,7 +5333,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <f>SUM(Tabelle271013[Estimated time])</f>
         <v>22</v>
@@ -5370,22 +5376,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>83</v>
       </c>
@@ -5420,7 +5426,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45623</v>
       </c>
@@ -5437,7 +5443,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -5468,7 +5474,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -5481,7 +5487,7 @@
       <c r="J4" s="8"/>
       <c r="K4" s="19"/>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -5494,7 +5500,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -5507,20 +5513,38 @@
       <c r="J6" s="8"/>
       <c r="K6" s="19"/>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="19"/>
-    </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="C7" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="8">
+        <v>6</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="I7" s="8">
+        <v>5</v>
+      </c>
+      <c r="J7" s="8">
+        <v>5</v>
+      </c>
+      <c r="K7" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -5533,7 +5557,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -5546,7 +5570,7 @@
       <c r="J9" s="8"/>
       <c r="K9" s="19"/>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -5559,7 +5583,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -5572,7 +5596,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -5584,7 +5608,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -5596,7 +5620,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -5608,7 +5632,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>93</v>
       </c>
@@ -5630,23 +5654,23 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <f>SUM(Tabelle27101316[Estimated time])</f>
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B16" s="12">
         <f>SUM(Tabelle27101316[Time in Hours])</f>
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C16" s="12">
         <f>Tabelle38111417[[#This Row],[Estimated time]]-Tabelle38111417[[#This Row],[Actual time]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="12">
         <f>SUM(Tabelle27101316[Story points])</f>
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F16" s="12">
         <f>Tabelle49121518[[#This Row],[Total Storypoints ]]/Tabelle38111417[[#This Row],[Actual time]]</f>
@@ -5674,18 +5698,18 @@
     <tabColor theme="6"/>
   </sheetPr>
   <dimension ref="A1:I26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="86.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="86.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -5709,7 +5733,7 @@
       </c>
       <c r="I1" s="17"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -5733,9 +5757,9 @@
       </c>
       <c r="I2" s="17"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>12</v>
@@ -5757,9 +5781,9 @@
       </c>
       <c r="I3" s="17"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>45</v>
@@ -5779,9 +5803,9 @@
       <c r="G4" s="2"/>
       <c r="I4" s="17"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>110</v>
@@ -5803,9 +5827,9 @@
       </c>
       <c r="I5" s="17"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>19</v>
@@ -5827,9 +5851,9 @@
       </c>
       <c r="I6" s="17"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>152</v>
@@ -5851,9 +5875,9 @@
       </c>
       <c r="I7" s="17"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>14</v>
@@ -5875,9 +5899,9 @@
       </c>
       <c r="I8" s="17"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>30</v>
@@ -5899,9 +5923,9 @@
       </c>
       <c r="I9" s="17"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>148</v>
@@ -5921,9 +5945,9 @@
       <c r="G10" s="2"/>
       <c r="I10" s="17"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>14</v>
@@ -5945,7 +5969,7 @@
       </c>
       <c r="I11" s="17"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>29</v>
       </c>
@@ -5969,9 +5993,9 @@
       </c>
       <c r="I12" s="17"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>23</v>
@@ -5993,9 +6017,9 @@
       </c>
       <c r="I13" s="17"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>57</v>
@@ -6017,9 +6041,9 @@
       </c>
       <c r="I14" s="17"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>30</v>
@@ -6039,9 +6063,9 @@
       <c r="G15" s="2"/>
       <c r="I15" s="17"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>27</v>
@@ -6061,9 +6085,9 @@
       <c r="G16" s="2"/>
       <c r="I16" s="17"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>141</v>
@@ -6085,9 +6109,9 @@
       </c>
       <c r="I17" s="17"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>144</v>
@@ -6107,9 +6131,9 @@
       <c r="G18" s="2"/>
       <c r="I18" s="17"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>143</v>
@@ -6131,9 +6155,9 @@
       </c>
       <c r="I19" s="17"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>51</v>
@@ -6155,9 +6179,9 @@
       </c>
       <c r="I20" s="17"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>38</v>
@@ -6177,9 +6201,9 @@
       <c r="G21" s="2"/>
       <c r="I21" s="17"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>42</v>
@@ -6199,9 +6223,9 @@
       <c r="G22" s="2"/>
       <c r="I22" s="17"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>48</v>
@@ -6221,9 +6245,9 @@
       <c r="G23" s="2"/>
       <c r="I23" s="17"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>54</v>
@@ -6243,9 +6267,9 @@
       <c r="G24" s="2"/>
       <c r="I24" s="17"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>60</v>
@@ -6264,7 +6288,7 @@
       </c>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="4"/>
       <c r="B26" s="16"/>
       <c r="C26" s="4"/>

</xml_diff>

<commit_message>
deleted old excelFile; Tweaked UX; added FishInfo;
</commit_message>
<xml_diff>
--- a/aquasphere/Excel_File/AquaSphare.xlsx
+++ b/aquasphere/Excel_File/AquaSphare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\43680\Desktop\Schule\SYP\Aquarium\aquasphere\Excel_File\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielhoheneder/Desktop/Schule/syp/AquaSphere/aquasphere/Excel_File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{070799D5-BC06-4827-A752-D685CB8BEA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BD7AFB5-4F57-4E47-A701-097F71B3D360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="25820" windowHeight="15500" activeTab="5" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Dashboard" sheetId="2" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="162">
   <si>
     <t>Story ID</t>
   </si>
@@ -541,6 +541,15 @@
   </si>
   <si>
     <t>Schmutz muss entstehen und sichtbar sein. User kann über reinigen button oder mit einem Brush tool das Aquarium reinigen</t>
+  </si>
+  <si>
+    <t>Schmutz spawn optimiert.</t>
+  </si>
+  <si>
+    <t>Es müssen Daten über den ausgewählten Fisch preisgegeben werden können und vernünftig sowie für den User klar verständlich präsentiert werden.</t>
+  </si>
+  <si>
+    <t>Punktesystem/UX Tweaks</t>
   </si>
 </sst>
 </file>
@@ -705,8 +714,8 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Prozent" xfId="1" builtinId="5"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="128">
     <dxf>
@@ -3599,20 +3608,20 @@
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:H17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>5</v>
       </c>
@@ -3638,7 +3647,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>70</v>
       </c>
@@ -3669,7 +3678,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>71</v>
       </c>
@@ -3700,7 +3709,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>72</v>
       </c>
@@ -3732,7 +3741,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>73</v>
       </c>
@@ -3764,28 +3773,28 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>74</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C6" s="7" cm="1">
         <f t="array" ref="C6">Tabelle38111417[Estimated time]</f>
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D6" s="7" cm="1">
         <f t="array" ref="D6">Tabelle38111417[Actual time]</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E6" s="7" cm="1">
         <f t="array" ref="E6">Tabelle49121518[[Total Storypoints ]]</f>
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F6" s="7">
         <f>Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]]</f>
-        <v>1</v>
+        <v>1.3125</v>
       </c>
       <c r="G6" s="7">
         <f>H5</f>
@@ -3793,10 +3802,10 @@
       </c>
       <c r="H6" s="7">
         <f>C13</f>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>75</v>
       </c>
@@ -3808,7 +3817,7 @@
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>76</v>
       </c>
@@ -3820,7 +3829,7 @@
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
     </row>
-    <row r="12" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>77</v>
       </c>
@@ -3828,16 +3837,16 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>118</v>
       </c>
       <c r="C13" s="5">
         <f>C12-SUM(Tabelle1[Accomplished Story Points])</f>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>81</v>
       </c>
@@ -3846,35 +3855,35 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C15" s="5">
         <f>AVERAGE(Tabelle1[Velocity])</f>
-        <v>0.86617647058823533</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>0.92867647058823533</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>79</v>
       </c>
       <c r="C16" s="14">
         <f>(SUM(Tabelle1[Accomplished Story Points],)/G2)</f>
-        <v>0.58904109589041098</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+        <v>0.64383561643835618</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" ht="24" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>69</v>
       </c>
       <c r="C17" s="18">
         <f>C13/C15</f>
-        <v>69.269949066213925</v>
+        <v>55.993665874901026</v>
       </c>
       <c r="D17">
         <f>C17/4</f>
-        <v>17.317487266553481</v>
+        <v>13.998416468725257</v>
       </c>
     </row>
   </sheetData>
@@ -3892,21 +3901,21 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:J16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="95.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="95.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>83</v>
       </c>
@@ -3938,7 +3947,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45925</v>
       </c>
@@ -3968,7 +3977,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -3990,7 +3999,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -4010,7 +4019,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -4022,7 +4031,7 @@
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
     </row>
-    <row r="6" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -4050,7 +4059,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
@@ -4076,7 +4085,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
@@ -4100,7 +4109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -4112,7 +4121,7 @@
       <c r="I9" s="8"/>
       <c r="J9" s="8"/>
     </row>
-    <row r="10" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -4124,7 +4133,7 @@
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
     </row>
-    <row r="11" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -4136,7 +4145,7 @@
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
     </row>
-    <row r="12" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4148,7 +4157,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4160,7 +4169,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4172,7 +4181,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>93</v>
       </c>
@@ -4194,7 +4203,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <f>SUM(Tabelle2[Estimated time])</f>
         <v>13</v>
@@ -4237,22 +4246,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>83</v>
       </c>
@@ -4287,7 +4296,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45939</v>
       </c>
@@ -4322,7 +4331,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -4351,7 +4360,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -4364,7 +4373,7 @@
       <c r="J4" s="8"/>
       <c r="K4" s="19"/>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
@@ -4393,7 +4402,7 @@
       </c>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -4422,7 +4431,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -4435,7 +4444,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -4448,7 +4457,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
@@ -4479,7 +4488,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8" t="s">
@@ -4510,7 +4519,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8" t="s">
@@ -4537,7 +4546,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4550,7 +4559,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="19"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4562,7 +4571,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4574,7 +4583,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -4586,7 +4595,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>93</v>
       </c>
@@ -4608,7 +4617,7 @@
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <f>SUM(Tabelle27[Estimated time])</f>
         <v>42</v>
@@ -4652,22 +4661,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>83</v>
       </c>
@@ -4702,7 +4711,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45953</v>
       </c>
@@ -4719,7 +4728,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -4750,7 +4759,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -4781,7 +4790,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -4794,7 +4803,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -4807,7 +4816,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="19"/>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -4820,7 +4829,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -4833,7 +4842,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -4846,7 +4855,7 @@
       <c r="J9" s="8"/>
       <c r="K9" s="19"/>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -4859,7 +4868,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -4872,7 +4881,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4885,7 +4894,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="19"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4897,7 +4906,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4909,7 +4918,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -4921,7 +4930,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>93</v>
       </c>
@@ -4943,7 +4952,7 @@
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <f>SUM(Tabelle2710[Estimated time])</f>
         <v>9</v>
@@ -4987,22 +4996,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>83</v>
       </c>
@@ -5037,7 +5046,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45981</v>
       </c>
@@ -5054,7 +5063,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -5085,7 +5094,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -5114,7 +5123,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
@@ -5143,7 +5152,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -5174,7 +5183,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -5187,7 +5196,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
@@ -5218,7 +5227,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
@@ -5249,7 +5258,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -5262,7 +5271,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -5275,7 +5284,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -5287,7 +5296,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -5299,7 +5308,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -5311,7 +5320,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>93</v>
       </c>
@@ -5333,7 +5342,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <f>SUM(Tabelle271013[Estimated time])</f>
         <v>22</v>
@@ -5376,22 +5385,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>83</v>
       </c>
@@ -5426,7 +5435,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45623</v>
       </c>
@@ -5443,7 +5452,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -5474,7 +5483,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -5487,7 +5496,7 @@
       <c r="J4" s="8"/>
       <c r="K4" s="19"/>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -5500,7 +5509,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -5513,7 +5522,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="19"/>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
@@ -5544,33 +5553,55 @@
         <v>121</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
+      <c r="C8" s="8" t="s">
+        <v>123</v>
+      </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
+      <c r="H8" s="8" t="s">
+        <v>159</v>
+      </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="19"/>
-    </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="C9" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="G9" s="8">
+        <v>3</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="I9" s="8">
+        <v>8</v>
+      </c>
+      <c r="J9" s="8">
+        <v>3</v>
+      </c>
+      <c r="K9" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -5583,7 +5614,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -5596,7 +5627,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -5608,7 +5639,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -5620,7 +5651,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -5632,7 +5663,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>93</v>
       </c>
@@ -5654,14 +5685,14 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <f>SUM(Tabelle27101316[Estimated time])</f>
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B16" s="12">
         <f>SUM(Tabelle27101316[Time in Hours])</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C16" s="12">
         <f>Tabelle38111417[[#This Row],[Estimated time]]-Tabelle38111417[[#This Row],[Actual time]]</f>
@@ -5670,11 +5701,11 @@
       <c r="D16" s="8"/>
       <c r="E16" s="12">
         <f>SUM(Tabelle27101316[Story points])</f>
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F16" s="12">
         <f>Tabelle49121518[[#This Row],[Total Storypoints ]]/Tabelle38111417[[#This Row],[Actual time]]</f>
-        <v>1</v>
+        <v>1.3125</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
@@ -5698,18 +5729,18 @@
     <tabColor theme="6"/>
   </sheetPr>
   <dimension ref="A1:I26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="86.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="86.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -5733,7 +5764,7 @@
       </c>
       <c r="I1" s="17"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -5757,7 +5788,7 @@
       </c>
       <c r="I2" s="17"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -5781,7 +5812,7 @@
       </c>
       <c r="I3" s="17"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -5803,7 +5834,7 @@
       <c r="G4" s="2"/>
       <c r="I4" s="17"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -5827,7 +5858,7 @@
       </c>
       <c r="I5" s="17"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -5851,7 +5882,7 @@
       </c>
       <c r="I6" s="17"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -5875,7 +5906,7 @@
       </c>
       <c r="I7" s="17"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
@@ -5899,7 +5930,7 @@
       </c>
       <c r="I8" s="17"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
@@ -5923,7 +5954,7 @@
       </c>
       <c r="I9" s="17"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
@@ -5945,7 +5976,7 @@
       <c r="G10" s="2"/>
       <c r="I10" s="17"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
@@ -5969,7 +6000,7 @@
       </c>
       <c r="I11" s="17"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>29</v>
       </c>
@@ -5993,7 +6024,7 @@
       </c>
       <c r="I12" s="17"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>32</v>
       </c>
@@ -6017,7 +6048,7 @@
       </c>
       <c r="I13" s="17"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>33</v>
       </c>
@@ -6041,7 +6072,7 @@
       </c>
       <c r="I14" s="17"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>36</v>
       </c>
@@ -6063,7 +6094,7 @@
       <c r="G15" s="2"/>
       <c r="I15" s="17"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>37</v>
       </c>
@@ -6085,7 +6116,7 @@
       <c r="G16" s="2"/>
       <c r="I16" s="17"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>40</v>
       </c>
@@ -6109,7 +6140,7 @@
       </c>
       <c r="I17" s="17"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>41</v>
       </c>
@@ -6123,15 +6154,17 @@
         <v>145</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>9</v>
+        <v>121</v>
       </c>
       <c r="F18" s="2">
         <v>8</v>
       </c>
-      <c r="G18" s="2"/>
+      <c r="G18" s="2">
+        <v>5</v>
+      </c>
       <c r="I18" s="17"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>44</v>
       </c>
@@ -6155,7 +6188,7 @@
       </c>
       <c r="I19" s="17"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>47</v>
       </c>
@@ -6179,7 +6212,7 @@
       </c>
       <c r="I20" s="17"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>50</v>
       </c>
@@ -6201,7 +6234,7 @@
       <c r="G21" s="2"/>
       <c r="I21" s="17"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>53</v>
       </c>
@@ -6223,7 +6256,7 @@
       <c r="G22" s="2"/>
       <c r="I22" s="17"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>56</v>
       </c>
@@ -6237,15 +6270,17 @@
         <v>49</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>9</v>
+        <v>121</v>
       </c>
       <c r="F23" s="2">
         <v>5</v>
       </c>
-      <c r="G23" s="2"/>
+      <c r="G23" s="2">
+        <v>5</v>
+      </c>
       <c r="I23" s="17"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>59</v>
       </c>
@@ -6267,7 +6302,7 @@
       <c r="G24" s="2"/>
       <c r="I24" s="17"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>62</v>
       </c>
@@ -6288,7 +6323,7 @@
       </c>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="4"/>
       <c r="B26" s="16"/>
       <c r="C26" s="4"/>

</xml_diff>

<commit_message>
feat: Implement dirt penalty system and improve hunger mechanics
- Add warning icon showing dirt level and penalty percentage
- Sync dirt penalty calculation with visible stains
- Balance cleaner fish effectiveness (radius 2.5x, strength 0.25)
- Invert hunger bar display (full green = satt, empty = hungry)
- Lower hunger threshold to 20, increase satiation to -60
- Slow hunger rate to 1 point per 5 seconds
- Add death after 2 minutes at hunger 100
- Implement 10-second despawn timer for dead fish
- Increase fish speeds to 9-14 range for better visibility
- Add satiation pause system (45s game time) that scales correctly with timeSpeed
- Fix: Satiation pause now adjusts dynamically when timeSpeed changes
</commit_message>
<xml_diff>
--- a/aquasphere/Excel_File/AquaSphare.xlsx
+++ b/aquasphere/Excel_File/AquaSphare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielhoheneder/Desktop/Schule/syp/AquaSphere/aquasphere/Excel_File/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\43680\Desktop\Schule\SYP\Aquarium\aquasphere\Excel_File\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D6C74E-D7C4-C34F-98B9-CD10B111C905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13D9FE3-A397-44FB-BAC5-B8AF8FC4DB0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="32480" windowHeight="20040" activeTab="6" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Dashboard" sheetId="2" r:id="rId1"/>
@@ -19,7 +19,8 @@
     <sheet name="Sprint3" sheetId="5" r:id="rId4"/>
     <sheet name="Sprint4" sheetId="6" r:id="rId5"/>
     <sheet name="Sprint5" sheetId="7" r:id="rId6"/>
-    <sheet name="Storys" sheetId="1" r:id="rId7"/>
+    <sheet name="Sprint6" sheetId="8" r:id="rId7"/>
+    <sheet name="Storys" sheetId="1" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="176">
   <si>
     <t>Story ID</t>
   </si>
@@ -562,6 +563,39 @@
     <t>* Es gibt eine Aquariumszeit, die von der realen Zeit unabhängig ist
 * Man kann den Zeitfortschritt verändern (2-fach bis x-fach??)
 * Wenn man ausloggt, geht die Zeit automatisch wieder auf 1-fach zurück</t>
+  </si>
+  <si>
+    <t>* Es gibt eine Aquariumszeit, die von der realen Zeit unabhängig ist</t>
+  </si>
+  <si>
+    <t>* Man kann den Zeitfortschritt verändern (2-fach bis x-fach??)</t>
+  </si>
+  <si>
+    <t>* Wenn man ausloggt, geht die Zeit automatisch wieder auf 1-fach zurück</t>
+  </si>
+  <si>
+    <t>Started</t>
+  </si>
+  <si>
+    <t>Reinigung</t>
+  </si>
+  <si>
+    <t>Als Nutzer möchte ich von meinen Pflanzen profitieren und auch Putzfische haben.</t>
+  </si>
+  <si>
+    <t>Pflanzen sollen sich passiv Positiv auf die Sauberkeit des Aquariums auswirken, Putzfische sollen ebenfalls passiv für Sauberkeit sorgen</t>
+  </si>
+  <si>
+    <t>Schmutzige Aquairen sollen weniger "Geld" produzieren</t>
+  </si>
+  <si>
+    <t>AQU25</t>
+  </si>
+  <si>
+    <t>Eco</t>
+  </si>
+  <si>
+    <t>Pflanzen sollen sich passiv Positiv auf die Sauberkeit des Aquariums auswirken, Putzfische sollen ebenfalls passiv für Sauberkeit sorgen. Schmutzige Aquairen sollen weniger "Geld" produzieren</t>
   </si>
 </sst>
 </file>
@@ -738,10 +772,401 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Prozent" xfId="1" builtinId="5"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="129">
+  <dxfs count="151">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -749,7 +1174,6 @@
           <bgColor theme="3" tint="0.89999084444715716"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -774,6 +1198,7 @@
           <bgColor theme="3" tint="0.89999084444715716"/>
         </patternFill>
       </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -3011,25 +3436,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AAF41172-5838-4CA9-A8A2-78B1E57ACF1F}" name="Tabelle1" displayName="Tabelle1" ref="A1:H8" totalsRowShown="0" headerRowDxfId="128" dataDxfId="127">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AAF41172-5838-4CA9-A8A2-78B1E57ACF1F}" name="Tabelle1" displayName="Tabelle1" ref="A1:H8" totalsRowShown="0" headerRowDxfId="150" dataDxfId="149">
   <autoFilter ref="A1:H8" xr:uid="{AAF41172-5838-4CA9-A8A2-78B1E57ACF1F}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{8BB8E342-544E-430C-A72A-9EBF9676D447}" name="Sprint" dataDxfId="126"/>
-    <tableColumn id="9" xr3:uid="{96A939A8-DA63-4E70-B123-D31A897D4192}" name="Story ID" dataDxfId="125"/>
-    <tableColumn id="2" xr3:uid="{CB307D23-EE39-436B-9E06-9E7789362DB6}" name="Estimated Hours" dataDxfId="124">
+    <tableColumn id="1" xr3:uid="{8BB8E342-544E-430C-A72A-9EBF9676D447}" name="Sprint" dataDxfId="148"/>
+    <tableColumn id="9" xr3:uid="{96A939A8-DA63-4E70-B123-D31A897D4192}" name="Story ID" dataDxfId="147"/>
+    <tableColumn id="2" xr3:uid="{CB307D23-EE39-436B-9E06-9E7789362DB6}" name="Estimated Hours" dataDxfId="146">
       <calculatedColumnFormula array="1">Tabelle3[Estimated time]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{5EFC7DEC-DFDE-454B-90FC-2713EB4181D8}" name="Actual Hours" dataDxfId="123">
+    <tableColumn id="3" xr3:uid="{5EFC7DEC-DFDE-454B-90FC-2713EB4181D8}" name="Actual Hours" dataDxfId="145">
       <calculatedColumnFormula array="1">Tabelle3[Actual time]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D6FF0659-1B35-4F09-B5A7-D22FEF5F7C3F}" name="Accomplished Story Points" dataDxfId="122">
+    <tableColumn id="4" xr3:uid="{D6FF0659-1B35-4F09-B5A7-D22FEF5F7C3F}" name="Accomplished Story Points" dataDxfId="144">
       <calculatedColumnFormula array="1">Tabelle4[[Total Storypoints ]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{9CD2DBE3-2E45-4440-8D7A-2A03A0291AAD}" name="Velocity" dataDxfId="121">
+    <tableColumn id="5" xr3:uid="{9CD2DBE3-2E45-4440-8D7A-2A03A0291AAD}" name="Velocity" dataDxfId="143">
       <calculatedColumnFormula>Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{1977DF7A-0A05-43B5-99D3-B72159480780}" name="Total Storypoints" dataDxfId="120"/>
-    <tableColumn id="7" xr3:uid="{D8A5F5FE-B9BC-448A-A9E7-3D00888AE639}" name="Storypoints Left" dataDxfId="119">
+    <tableColumn id="6" xr3:uid="{1977DF7A-0A05-43B5-99D3-B72159480780}" name="Total Storypoints" dataDxfId="142"/>
+    <tableColumn id="7" xr3:uid="{D8A5F5FE-B9BC-448A-A9E7-3D00888AE639}" name="Storypoints Left" dataDxfId="141">
       <calculatedColumnFormula>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3038,13 +3463,13 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0134C802-458D-4153-B0D4-D8B08E02E26A}" name="Tabelle4912" displayName="Tabelle4912" ref="E16:F17" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0134C802-458D-4153-B0D4-D8B08E02E26A}" name="Tabelle4912" displayName="Tabelle4912" ref="E16:F17" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
   <autoFilter ref="E16:F17" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C3438C75-AD69-46E0-B1BD-0445ED469483}" name="Total Storypoints " dataDxfId="55">
+    <tableColumn id="1" xr3:uid="{C3438C75-AD69-46E0-B1BD-0445ED469483}" name="Total Storypoints " dataDxfId="77">
       <calculatedColumnFormula>SUM(Tabelle2710[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0655740B-E1AB-4BD3-B7CA-852D4C79FC17}" name="Effort/Hour" dataDxfId="54">
+    <tableColumn id="2" xr3:uid="{0655740B-E1AB-4BD3-B7CA-852D4C79FC17}" name="Effort/Hour" dataDxfId="76">
       <calculatedColumnFormula>Tabelle4912[[#This Row],[Total Storypoints ]]/Tabelle3811[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3053,36 +3478,36 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}" name="Tabelle271013" displayName="Tabelle271013" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}" name="Tabelle271013" displayName="Tabelle271013" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
   <autoFilter ref="A1:K11" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{946A4B14-799A-49AD-8E3E-31E3F4BBE559}" name="Sprint Start" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{E61A962F-4EE4-4843-AF21-C647918EECAB}" name="Sprint End" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{4EC50B40-18BD-4D00-8BE2-5596A9347BB8}" name="User" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{2A1F175E-D14E-491C-B452-39567CF84CD6}" name="ID" dataDxfId="48"/>
-    <tableColumn id="6" xr3:uid="{DCE5121F-D243-470B-B0AF-D0EE5264DD5A}" name="Epic" dataDxfId="47"/>
-    <tableColumn id="12" xr3:uid="{45FDCCAE-F13D-47C1-B91E-2EF3CC9A5BA0}" name="User Story /Task" dataDxfId="46"/>
-    <tableColumn id="11" xr3:uid="{4057DF12-8977-4284-BF2B-9ED3AAE7221F}" name="Estimated time" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{08443A2E-5832-4299-8009-1F0D489DEE15}" name="COS (Criteria of Satisfaction)" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{8777A429-C11B-4CDC-BB2F-785D0BC89DAB}" name="Story points" dataDxfId="43"/>
-    <tableColumn id="10" xr3:uid="{0B18443F-D8D9-4015-8EAA-7050016E43C2}" name="Time in Hours" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{5C5B5C91-6376-4597-B69B-4D162307C569}" name="Status" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{946A4B14-799A-49AD-8E3E-31E3F4BBE559}" name="Sprint Start" dataDxfId="73"/>
+    <tableColumn id="2" xr3:uid="{E61A962F-4EE4-4843-AF21-C647918EECAB}" name="Sprint End" dataDxfId="72"/>
+    <tableColumn id="3" xr3:uid="{4EC50B40-18BD-4D00-8BE2-5596A9347BB8}" name="User" dataDxfId="71"/>
+    <tableColumn id="5" xr3:uid="{2A1F175E-D14E-491C-B452-39567CF84CD6}" name="ID" dataDxfId="70"/>
+    <tableColumn id="6" xr3:uid="{DCE5121F-D243-470B-B0AF-D0EE5264DD5A}" name="Epic" dataDxfId="69"/>
+    <tableColumn id="12" xr3:uid="{45FDCCAE-F13D-47C1-B91E-2EF3CC9A5BA0}" name="User Story /Task" dataDxfId="68"/>
+    <tableColumn id="11" xr3:uid="{4057DF12-8977-4284-BF2B-9ED3AAE7221F}" name="Estimated time" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{08443A2E-5832-4299-8009-1F0D489DEE15}" name="COS (Criteria of Satisfaction)" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{8777A429-C11B-4CDC-BB2F-785D0BC89DAB}" name="Story points" dataDxfId="65"/>
+    <tableColumn id="10" xr3:uid="{0B18443F-D8D9-4015-8EAA-7050016E43C2}" name="Time in Hours" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{5C5B5C91-6376-4597-B69B-4D162307C569}" name="Status" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}" name="Tabelle381114" displayName="Tabelle381114" ref="A15:C16" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}" name="Tabelle381114" displayName="Tabelle381114" ref="A15:C16" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
   <autoFilter ref="A15:C16" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{E71994D0-AB06-482B-8487-03AB7E3B1FF7}" name="Estimated time" dataDxfId="38">
+    <tableColumn id="1" xr3:uid="{E71994D0-AB06-482B-8487-03AB7E3B1FF7}" name="Estimated time" dataDxfId="60">
       <calculatedColumnFormula>SUM(Tabelle271013[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E607785B-5B58-4D1E-81ED-45AAAAF488F0}" name="Actual time" dataDxfId="37">
+    <tableColumn id="2" xr3:uid="{E607785B-5B58-4D1E-81ED-45AAAAF488F0}" name="Actual time" dataDxfId="59">
       <calculatedColumnFormula>SUM(Tabelle271013[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{0197CFBA-597E-49C6-88E5-ABAC17763EA4}" name="Delta" dataDxfId="36">
+    <tableColumn id="3" xr3:uid="{0197CFBA-597E-49C6-88E5-ABAC17763EA4}" name="Delta" dataDxfId="58">
       <calculatedColumnFormula>Tabelle381114[[#This Row],[Estimated time]]-Tabelle381114[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3091,13 +3516,13 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}" name="Tabelle491215" displayName="Tabelle491215" ref="E15:F16" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}" name="Tabelle491215" displayName="Tabelle491215" ref="E15:F16" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
   <autoFilter ref="E15:F16" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{E0381C51-E5FF-4087-9146-76E105FE701A}" name="Total Storypoints " dataDxfId="33">
+    <tableColumn id="1" xr3:uid="{E0381C51-E5FF-4087-9146-76E105FE701A}" name="Total Storypoints " dataDxfId="55">
       <calculatedColumnFormula>SUM(Tabelle271013[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0971B46C-CFAA-4F13-88AB-CDC5655C1F84}" name="Effort/Hour" dataDxfId="32">
+    <tableColumn id="2" xr3:uid="{0971B46C-CFAA-4F13-88AB-CDC5655C1F84}" name="Effort/Hour" dataDxfId="54">
       <calculatedColumnFormula>Tabelle491215[[#This Row],[Total Storypoints ]]/Tabelle381114[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3106,36 +3531,36 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{235F589F-8BC0-4A3D-A02E-03E630D61504}" name="Tabelle27101316" displayName="Tabelle27101316" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{235F589F-8BC0-4A3D-A02E-03E630D61504}" name="Tabelle27101316" displayName="Tabelle27101316" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
   <autoFilter ref="A1:K11" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{B7D16283-E8F5-4C03-BEC2-39D9F536B2DF}" name="Sprint Start" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{743B7730-744D-48F9-8435-134B358D299C}" name="Sprint End" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{6BB0BFF2-8337-4911-B853-52953695FFB8}" name="User" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{23B9485C-C756-4653-9A7E-4CBFBC4BDCC9}" name="ID" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{DA3B151D-2F3B-4817-810C-2B84F6D521DF}" name="Epic" dataDxfId="25"/>
-    <tableColumn id="12" xr3:uid="{0B21ADB3-F002-4AC8-8EFB-36998E0BA400}" name="User Story /Task" dataDxfId="24"/>
-    <tableColumn id="11" xr3:uid="{0AF7F7D2-16D8-4903-AFB0-E002FAFE9A7B}" name="Estimated time" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{2F945FB5-B8D6-4015-9863-4264314B3D66}" name="COS (Criteria of Satisfaction)" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{72841B6A-9C3A-4632-878E-ADBD76467B91}" name="Story points" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{99643A57-EC89-4FC7-B6E0-CEECFE14CE6B}" name="Time in Hours" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{D3F46A45-6C79-4B7E-9924-30DF1A278D97}" name="Status" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{B7D16283-E8F5-4C03-BEC2-39D9F536B2DF}" name="Sprint Start" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{743B7730-744D-48F9-8435-134B358D299C}" name="Sprint End" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{6BB0BFF2-8337-4911-B853-52953695FFB8}" name="User" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{23B9485C-C756-4653-9A7E-4CBFBC4BDCC9}" name="ID" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{DA3B151D-2F3B-4817-810C-2B84F6D521DF}" name="Epic" dataDxfId="47"/>
+    <tableColumn id="12" xr3:uid="{0B21ADB3-F002-4AC8-8EFB-36998E0BA400}" name="User Story /Task" dataDxfId="46"/>
+    <tableColumn id="11" xr3:uid="{0AF7F7D2-16D8-4903-AFB0-E002FAFE9A7B}" name="Estimated time" dataDxfId="45"/>
+    <tableColumn id="8" xr3:uid="{2F945FB5-B8D6-4015-9863-4264314B3D66}" name="COS (Criteria of Satisfaction)" dataDxfId="44"/>
+    <tableColumn id="9" xr3:uid="{72841B6A-9C3A-4632-878E-ADBD76467B91}" name="Story points" dataDxfId="43"/>
+    <tableColumn id="10" xr3:uid="{99643A57-EC89-4FC7-B6E0-CEECFE14CE6B}" name="Time in Hours" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{D3F46A45-6C79-4B7E-9924-30DF1A278D97}" name="Status" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{E0805314-F662-4E1D-85A9-F2EC30EC262D}" name="Tabelle38111417" displayName="Tabelle38111417" ref="A15:C16" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{E0805314-F662-4E1D-85A9-F2EC30EC262D}" name="Tabelle38111417" displayName="Tabelle38111417" ref="A15:C16" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
   <autoFilter ref="A15:C16" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{1993629C-98D2-4E46-B14A-696AAE563315}" name="Estimated time" dataDxfId="16">
+    <tableColumn id="1" xr3:uid="{1993629C-98D2-4E46-B14A-696AAE563315}" name="Estimated time" dataDxfId="38">
       <calculatedColumnFormula>SUM(Tabelle27101316[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C3F5A116-86A6-4D3A-9417-88FA122B0C81}" name="Actual time" dataDxfId="15">
+    <tableColumn id="2" xr3:uid="{C3F5A116-86A6-4D3A-9417-88FA122B0C81}" name="Actual time" dataDxfId="37">
       <calculatedColumnFormula>SUM(Tabelle27101316[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B86C31E6-5405-4B45-9B86-86A0C1DBF35C}" name="Delta" dataDxfId="14">
+    <tableColumn id="3" xr3:uid="{B86C31E6-5405-4B45-9B86-86A0C1DBF35C}" name="Delta" dataDxfId="36">
       <calculatedColumnFormula>Tabelle38111417[[#This Row],[Estimated time]]-Tabelle38111417[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3144,13 +3569,13 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{FE78B35D-B1A7-42FC-BB42-AF310800AF69}" name="Tabelle49121518" displayName="Tabelle49121518" ref="E15:F16" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{FE78B35D-B1A7-42FC-BB42-AF310800AF69}" name="Tabelle49121518" displayName="Tabelle49121518" ref="E15:F16" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="E15:F16" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{E7934959-5DF7-4D4C-858C-1FAD310B1F3B}" name="Total Storypoints " dataDxfId="11">
+    <tableColumn id="1" xr3:uid="{E7934959-5DF7-4D4C-858C-1FAD310B1F3B}" name="Total Storypoints " dataDxfId="33">
       <calculatedColumnFormula>SUM(Tabelle27101316[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D7E6F4E2-872C-4E38-9126-8A958E19087E}" name="Effort/Hour" dataDxfId="10">
+    <tableColumn id="2" xr3:uid="{D7E6F4E2-872C-4E38-9126-8A958E19087E}" name="Effort/Hour" dataDxfId="32">
       <calculatedColumnFormula>Tabelle49121518[[#This Row],[Total Storypoints ]]/Tabelle38111417[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3159,55 +3584,108 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:H26" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:H26" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H26">
-    <sortCondition ref="C9:C26"/>
-  </sortState>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Story" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{57E495A5-904B-1740-A858-653ACCE96658}" name="Acceptance Criteria" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{E37FAD70-20F3-4912-82B8-9AC496901DBE}" name="Tabelle2710131619" displayName="Tabelle2710131619" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+  <autoFilter ref="A1:K11" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{D532321B-43A9-4C7B-9711-0E9DB0F36080}" name="Sprint Start" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{F9445A15-FEA9-4142-9284-D23FEC81E85A}" name="Sprint End" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{98E29721-27A3-49D9-AB54-E3E822D61773}" name="User" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{A6CFA86C-B64A-4D7B-988B-D7EA90AE832B}" name="ID" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{2A363B76-0FF0-4E35-8B0D-D3DFE428B184}" name="Epic" dataDxfId="15"/>
+    <tableColumn id="12" xr3:uid="{58EF9BAF-7539-44AE-B4EA-ED1E3E2C43A2}" name="User Story /Task" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{5812FBDE-2CCF-4471-BA12-4B4E981FB0F8}" name="Estimated time" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{9D350C75-9112-414E-B33C-95BA4ED272B4}" name="COS (Criteria of Satisfaction)" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{79971A75-750E-427F-A5B6-5A61FA1008BB}" name="Story points" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{F15B638A-5756-448D-BFF1-F83357264427}" name="Time in Hours" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{5419A239-65A0-4210-A072-8D48A4908096}" name="Status" dataDxfId="9"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{1868505A-CACE-44B2-A7EA-9FE64E58BA8A}" name="Tabelle3811141720" displayName="Tabelle3811141720" ref="A15:C16" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A15:C16" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{3A312704-DAF9-41C4-9ED9-5DD84799E905}" name="Estimated time" dataDxfId="6">
+      <calculatedColumnFormula>SUM(Tabelle2710131619[Estimated time])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{72BDDA5F-E86A-4485-B7A7-C4A72345EFC4}" name="Actual time" dataDxfId="5">
+      <calculatedColumnFormula>SUM(Tabelle2710131619[Time in Hours])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{223E53E9-D637-4AC0-9A6C-5591B23BB953}" name="Delta" dataDxfId="4">
+      <calculatedColumnFormula>Tabelle3811141720[[#This Row],[Estimated time]]-Tabelle3811141720[[#This Row],[Actual time]]</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{F7C4B985-A6EE-4B5E-BF93-A6081AE08433}" name="Tabelle4912151821" displayName="Tabelle4912151821" ref="E15:F16" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
+  <autoFilter ref="E15:F16" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{DC2B1F8F-41E8-42FD-87FA-7DF04FEE86E6}" name="Total Storypoints " dataDxfId="1">
+      <calculatedColumnFormula>SUM(Tabelle2710131619[Story points])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{913BEBDF-DC3B-496C-982F-AE7F617915B6}" name="Effort/Hour" dataDxfId="0">
+      <calculatedColumnFormula>Tabelle4912151821[[#This Row],[Total Storypoints ]]/Tabelle3811141720[[#This Row],[Actual time]]</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}" name="Tabelle2" displayName="Tabelle2" ref="A1:J9" insertRowShift="1" totalsRowShown="0" headerRowDxfId="118" dataDxfId="117">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}" name="Tabelle2" displayName="Tabelle2" ref="A1:J9" insertRowShift="1" totalsRowShown="0" headerRowDxfId="140" dataDxfId="139">
   <autoFilter ref="A1:J9" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{0351E8C1-0BB8-4C19-A406-233CC12328E5}" name="Sprint Start" dataDxfId="116"/>
-    <tableColumn id="2" xr3:uid="{51BD2FE0-507A-4398-BD96-E186E78BB2C7}" name="Sprint End" dataDxfId="115"/>
-    <tableColumn id="3" xr3:uid="{A3B7E86B-E01A-4D78-82AD-BA81F6AC7ADF}" name="User" dataDxfId="114"/>
-    <tableColumn id="5" xr3:uid="{CE780601-F45C-4063-B216-98ACE5588903}" name="ID" dataDxfId="113"/>
-    <tableColumn id="6" xr3:uid="{A14D049D-AC5C-49A5-A7CC-A4D5ED8A8330}" name="Epic" dataDxfId="112"/>
-    <tableColumn id="12" xr3:uid="{770F10A6-830A-41AC-B069-6267CAE00BDF}" name="User Story /Task" dataDxfId="111"/>
-    <tableColumn id="11" xr3:uid="{0D9AB552-F7B4-4231-A35B-245B57383919}" name="Estimated time" dataDxfId="110"/>
-    <tableColumn id="8" xr3:uid="{3E2E3644-9002-4AB9-B3EC-96FFF84D8900}" name="COS (Criteria of Satisfaction)" dataDxfId="109"/>
-    <tableColumn id="9" xr3:uid="{14C8E3A9-BC37-48D9-A399-32A48A46993A}" name="Story points" dataDxfId="108"/>
-    <tableColumn id="10" xr3:uid="{151786D9-5F15-42D7-932B-664A024F4131}" name="Time in Hours" dataDxfId="107"/>
+    <tableColumn id="1" xr3:uid="{0351E8C1-0BB8-4C19-A406-233CC12328E5}" name="Sprint Start" dataDxfId="138"/>
+    <tableColumn id="2" xr3:uid="{51BD2FE0-507A-4398-BD96-E186E78BB2C7}" name="Sprint End" dataDxfId="137"/>
+    <tableColumn id="3" xr3:uid="{A3B7E86B-E01A-4D78-82AD-BA81F6AC7ADF}" name="User" dataDxfId="136"/>
+    <tableColumn id="5" xr3:uid="{CE780601-F45C-4063-B216-98ACE5588903}" name="ID" dataDxfId="135"/>
+    <tableColumn id="6" xr3:uid="{A14D049D-AC5C-49A5-A7CC-A4D5ED8A8330}" name="Epic" dataDxfId="134"/>
+    <tableColumn id="12" xr3:uid="{770F10A6-830A-41AC-B069-6267CAE00BDF}" name="User Story /Task" dataDxfId="133"/>
+    <tableColumn id="11" xr3:uid="{0D9AB552-F7B4-4231-A35B-245B57383919}" name="Estimated time" dataDxfId="132"/>
+    <tableColumn id="8" xr3:uid="{3E2E3644-9002-4AB9-B3EC-96FFF84D8900}" name="COS (Criteria of Satisfaction)" dataDxfId="131"/>
+    <tableColumn id="9" xr3:uid="{14C8E3A9-BC37-48D9-A399-32A48A46993A}" name="Story points" dataDxfId="130"/>
+    <tableColumn id="10" xr3:uid="{151786D9-5F15-42D7-932B-664A024F4131}" name="Time in Hours" dataDxfId="129"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:H27" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+  <autoFilter ref="A1:H27" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H27">
+    <sortCondition ref="C9:C27"/>
+  </sortState>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Story" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{57E495A5-904B-1740-A858-653ACCE96658}" name="Acceptance Criteria" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="23"/>
+    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}" name="Tabelle3" displayName="Tabelle3" ref="A15:C16" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}" name="Tabelle3" displayName="Tabelle3" ref="A15:C16" totalsRowShown="0" headerRowDxfId="128" dataDxfId="127">
   <autoFilter ref="A15:C16" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CD2D4D96-DD34-4EA3-92D7-B02BB9DE5647}" name="Estimated time" dataDxfId="104">
+    <tableColumn id="1" xr3:uid="{CD2D4D96-DD34-4EA3-92D7-B02BB9DE5647}" name="Estimated time" dataDxfId="126">
       <calculatedColumnFormula>SUM(Tabelle2[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0F14E190-6E0A-4AB8-8ADE-83875E98D4B5}" name="Actual time" dataDxfId="103">
+    <tableColumn id="2" xr3:uid="{0F14E190-6E0A-4AB8-8ADE-83875E98D4B5}" name="Actual time" dataDxfId="125">
       <calculatedColumnFormula>SUM(Tabelle2[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{5DE18543-F4D3-4732-9F2D-5B7F140CB974}" name="Delta" dataDxfId="102">
+    <tableColumn id="3" xr3:uid="{5DE18543-F4D3-4732-9F2D-5B7F140CB974}" name="Delta" dataDxfId="124">
       <calculatedColumnFormula>Tabelle3[[#This Row],[Estimated time]]-Tabelle3[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3216,13 +3694,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}" name="Tabelle4" displayName="Tabelle4" ref="E15:F16" totalsRowShown="0" headerRowDxfId="101" dataDxfId="100">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}" name="Tabelle4" displayName="Tabelle4" ref="E15:F16" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
   <autoFilter ref="E15:F16" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{2E187AEA-682F-4749-9FC8-ED3BA3DE1DA2}" name="Total Storypoints " dataDxfId="99">
+    <tableColumn id="1" xr3:uid="{2E187AEA-682F-4749-9FC8-ED3BA3DE1DA2}" name="Total Storypoints " dataDxfId="121">
       <calculatedColumnFormula>SUM(Tabelle2[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3C6DC8F5-724A-43AC-9128-7661A96380C1}" name="Efford/Hour" dataDxfId="98">
+    <tableColumn id="2" xr3:uid="{3C6DC8F5-724A-43AC-9128-7661A96380C1}" name="Efford/Hour" dataDxfId="120">
       <calculatedColumnFormula>Tabelle4[[#This Row],[Total Storypoints ]]/Tabelle3[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3231,36 +3709,36 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A211D33B-248F-4E66-AF7C-9632EAA38DAC}" name="Tabelle27" displayName="Tabelle27" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="97" dataDxfId="96">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A211D33B-248F-4E66-AF7C-9632EAA38DAC}" name="Tabelle27" displayName="Tabelle27" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="119" dataDxfId="118">
   <autoFilter ref="A1:K12" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{9C36A560-9153-4D8E-BA50-0044E74E1896}" name="Sprint Start" dataDxfId="95"/>
-    <tableColumn id="2" xr3:uid="{4FAB3106-8621-41F1-B866-EA5558F083D8}" name="Sprint End" dataDxfId="94"/>
-    <tableColumn id="3" xr3:uid="{2D2022CC-B165-4671-9773-4C7DCE737FC7}" name="User" dataDxfId="93"/>
-    <tableColumn id="5" xr3:uid="{6D49D607-DA69-4FF5-AC26-260E9F796217}" name="ID" dataDxfId="92"/>
-    <tableColumn id="6" xr3:uid="{95077F2F-115F-484E-A38C-A34A2BCBCB78}" name="Epic" dataDxfId="91"/>
-    <tableColumn id="12" xr3:uid="{2EAFDE91-2C58-4973-A684-28E2E964F629}" name="User Story /Task" dataDxfId="90"/>
-    <tableColumn id="11" xr3:uid="{D17AAC02-918A-4F08-B037-3622F37B62F0}" name="Estimated time" dataDxfId="89"/>
-    <tableColumn id="8" xr3:uid="{4D053EE2-698A-4191-ABEB-8F0701DA4D4E}" name="COS (Criteria of Satisfaction)" dataDxfId="88"/>
-    <tableColumn id="9" xr3:uid="{73BF0134-792D-4614-95FB-754C4A317665}" name="Story points" dataDxfId="87"/>
-    <tableColumn id="10" xr3:uid="{2620A9CC-A288-4874-BF27-2BBE69671B14}" name="Time in Hours" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="85"/>
+    <tableColumn id="1" xr3:uid="{9C36A560-9153-4D8E-BA50-0044E74E1896}" name="Sprint Start" dataDxfId="117"/>
+    <tableColumn id="2" xr3:uid="{4FAB3106-8621-41F1-B866-EA5558F083D8}" name="Sprint End" dataDxfId="116"/>
+    <tableColumn id="3" xr3:uid="{2D2022CC-B165-4671-9773-4C7DCE737FC7}" name="User" dataDxfId="115"/>
+    <tableColumn id="5" xr3:uid="{6D49D607-DA69-4FF5-AC26-260E9F796217}" name="ID" dataDxfId="114"/>
+    <tableColumn id="6" xr3:uid="{95077F2F-115F-484E-A38C-A34A2BCBCB78}" name="Epic" dataDxfId="113"/>
+    <tableColumn id="12" xr3:uid="{2EAFDE91-2C58-4973-A684-28E2E964F629}" name="User Story /Task" dataDxfId="112"/>
+    <tableColumn id="11" xr3:uid="{D17AAC02-918A-4F08-B037-3622F37B62F0}" name="Estimated time" dataDxfId="111"/>
+    <tableColumn id="8" xr3:uid="{4D053EE2-698A-4191-ABEB-8F0701DA4D4E}" name="COS (Criteria of Satisfaction)" dataDxfId="110"/>
+    <tableColumn id="9" xr3:uid="{73BF0134-792D-4614-95FB-754C4A317665}" name="Story points" dataDxfId="109"/>
+    <tableColumn id="10" xr3:uid="{2620A9CC-A288-4874-BF27-2BBE69671B14}" name="Time in Hours" dataDxfId="108"/>
+    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="107"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
   <autoFilter ref="A16:C17" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="82">
+    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="104">
       <calculatedColumnFormula>SUM(Tabelle27[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="81">
+    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="103">
       <calculatedColumnFormula>SUM(Tabelle27[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="80">
+    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="102">
       <calculatedColumnFormula>Tabelle38[[#This Row],[Estimated time]]-Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3269,13 +3747,13 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="101" dataDxfId="100">
   <autoFilter ref="E16:F17" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="77">
+    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="99">
       <calculatedColumnFormula>SUM(Tabelle27[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="76">
+    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="98">
       <calculatedColumnFormula>Tabelle49[[#This Row],[Total Storypoints ]]/Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3284,36 +3762,36 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6303AB7F-CDC2-408B-A450-96D692A68B43}" name="Tabelle2710" displayName="Tabelle2710" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6303AB7F-CDC2-408B-A450-96D692A68B43}" name="Tabelle2710" displayName="Tabelle2710" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="97" dataDxfId="96">
   <autoFilter ref="A1:K12" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{949CA967-02A0-4249-BB07-B02F4C4F69AE}" name="Sprint Start" dataDxfId="73"/>
-    <tableColumn id="2" xr3:uid="{A70AE104-D3DD-4C6E-8E50-E151404B19BD}" name="Sprint End" dataDxfId="72"/>
-    <tableColumn id="3" xr3:uid="{9168C6BE-6970-4420-9D5F-DBCF1E8E2BAE}" name="User" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{A7C4968E-9480-42FF-949B-9E41609C26A2}" name="ID" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{8564B7DD-8DB4-4E2B-BDDB-9791D9AAA0EA}" name="Epic" dataDxfId="69"/>
-    <tableColumn id="12" xr3:uid="{56FA47CB-3810-4B7F-A047-8358D5C73F6C}" name="User Story /Task" dataDxfId="68"/>
-    <tableColumn id="11" xr3:uid="{988CB3AF-F268-445B-887C-5163D9AE41DF}" name="Estimated time" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{14BDCFB4-F75D-4798-AFF3-3F8B177B78D6}" name="COS (Criteria of Satisfaction)" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{97C18CBF-2D3F-4A8A-B36D-6328E17F31C4}" name="Story points" dataDxfId="65"/>
-    <tableColumn id="10" xr3:uid="{D3E339CF-38BF-4AC1-8C80-41ECD30B6907}" name="Time in Hours" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{3BCBC0DA-7C9B-4D2B-9269-A319CBD925C5}" name="Status" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{949CA967-02A0-4249-BB07-B02F4C4F69AE}" name="Sprint Start" dataDxfId="95"/>
+    <tableColumn id="2" xr3:uid="{A70AE104-D3DD-4C6E-8E50-E151404B19BD}" name="Sprint End" dataDxfId="94"/>
+    <tableColumn id="3" xr3:uid="{9168C6BE-6970-4420-9D5F-DBCF1E8E2BAE}" name="User" dataDxfId="93"/>
+    <tableColumn id="5" xr3:uid="{A7C4968E-9480-42FF-949B-9E41609C26A2}" name="ID" dataDxfId="92"/>
+    <tableColumn id="6" xr3:uid="{8564B7DD-8DB4-4E2B-BDDB-9791D9AAA0EA}" name="Epic" dataDxfId="91"/>
+    <tableColumn id="12" xr3:uid="{56FA47CB-3810-4B7F-A047-8358D5C73F6C}" name="User Story /Task" dataDxfId="90"/>
+    <tableColumn id="11" xr3:uid="{988CB3AF-F268-445B-887C-5163D9AE41DF}" name="Estimated time" dataDxfId="89"/>
+    <tableColumn id="8" xr3:uid="{14BDCFB4-F75D-4798-AFF3-3F8B177B78D6}" name="COS (Criteria of Satisfaction)" dataDxfId="88"/>
+    <tableColumn id="9" xr3:uid="{97C18CBF-2D3F-4A8A-B36D-6328E17F31C4}" name="Story points" dataDxfId="87"/>
+    <tableColumn id="10" xr3:uid="{D3E339CF-38BF-4AC1-8C80-41ECD30B6907}" name="Time in Hours" dataDxfId="86"/>
+    <tableColumn id="4" xr3:uid="{3BCBC0DA-7C9B-4D2B-9269-A319CBD925C5}" name="Status" dataDxfId="85"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C1E761E2-D340-4C7F-A19A-AE84A76F5971}" name="Tabelle3811" displayName="Tabelle3811" ref="A16:C17" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C1E761E2-D340-4C7F-A19A-AE84A76F5971}" name="Tabelle3811" displayName="Tabelle3811" ref="A16:C17" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
   <autoFilter ref="A16:C17" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{F045D4AD-2D00-44A7-8EA7-B5C34869B26F}" name="Estimated time" dataDxfId="60">
+    <tableColumn id="1" xr3:uid="{F045D4AD-2D00-44A7-8EA7-B5C34869B26F}" name="Estimated time" dataDxfId="82">
       <calculatedColumnFormula>SUM(Tabelle2710[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DFDFE0A8-6207-4F3B-9D05-4D3AF083E31B}" name="Actual time" dataDxfId="59">
+    <tableColumn id="2" xr3:uid="{DFDFE0A8-6207-4F3B-9D05-4D3AF083E31B}" name="Actual time" dataDxfId="81">
       <calculatedColumnFormula>SUM(Tabelle2710[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{2529739A-9C5E-4AE4-80A6-DFC080EFE2D8}" name="Delta" dataDxfId="58">
+    <tableColumn id="3" xr3:uid="{2529739A-9C5E-4AE4-80A6-DFC080EFE2D8}" name="Delta" dataDxfId="80">
       <calculatedColumnFormula>Tabelle3811[[#This Row],[Estimated time]]-Tabelle3811[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3642,20 +4120,20 @@
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:H17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="6" t="s">
         <v>4</v>
       </c>
@@ -3681,7 +4159,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.5">
       <c r="A2" s="7" t="s">
         <v>69</v>
       </c>
@@ -3712,7 +4190,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.5">
       <c r="A3" s="7" t="s">
         <v>70</v>
       </c>
@@ -3743,7 +4221,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="21" x14ac:dyDescent="0.5">
       <c r="A4" s="7" t="s">
         <v>71</v>
       </c>
@@ -3775,7 +4253,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="21" x14ac:dyDescent="0.5">
       <c r="A5" s="7" t="s">
         <v>72</v>
       </c>
@@ -3807,7 +4285,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.5">
       <c r="A6" s="7" t="s">
         <v>73</v>
       </c>
@@ -3839,7 +4317,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="21" x14ac:dyDescent="0.5">
       <c r="A7" s="7" t="s">
         <v>74</v>
       </c>
@@ -3851,7 +4329,7 @@
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" ht="22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="21" x14ac:dyDescent="0.5">
       <c r="A8" s="7" t="s">
         <v>75</v>
       </c>
@@ -3863,7 +4341,7 @@
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
     </row>
-    <row r="12" spans="1:8" ht="24" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="1" t="s">
         <v>76</v>
       </c>
@@ -3871,7 +4349,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="24" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="B13" s="1" t="s">
         <v>117</v>
       </c>
@@ -3880,7 +4358,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="24" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="B14" s="1" t="s">
         <v>80</v>
       </c>
@@ -3889,7 +4367,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="24" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="1" t="s">
         <v>77</v>
       </c>
@@ -3898,7 +4376,7 @@
         <v>0.92867647058823533</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="24" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="B16" s="1" t="s">
         <v>78</v>
       </c>
@@ -3907,7 +4385,7 @@
         <v>0.64383561643835618</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="24" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="B17" s="1" t="s">
         <v>68</v>
       </c>
@@ -3935,21 +4413,21 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:J16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="95.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="95.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
@@ -3981,7 +4459,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="9">
         <v>45925</v>
       </c>
@@ -4011,7 +4489,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -4033,7 +4511,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -4053,7 +4531,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -4065,7 +4543,7 @@
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
     </row>
-    <row r="6" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -4093,7 +4571,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
@@ -4119,7 +4597,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
@@ -4143,7 +4621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -4155,7 +4633,7 @@
       <c r="I9" s="8"/>
       <c r="J9" s="8"/>
     </row>
-    <row r="10" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -4167,7 +4645,7 @@
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
     </row>
-    <row r="11" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -4179,7 +4657,7 @@
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
     </row>
-    <row r="12" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4191,7 +4669,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4203,7 +4681,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4215,7 +4693,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A15" s="13" t="s">
         <v>92</v>
       </c>
@@ -4237,7 +4715,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A16" s="12">
         <f>SUM(Tabelle2[Estimated time])</f>
         <v>13</v>
@@ -4280,22 +4758,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
@@ -4330,7 +4808,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="9">
         <v>45939</v>
       </c>
@@ -4365,7 +4843,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -4394,7 +4872,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -4407,7 +4885,7 @@
       <c r="J4" s="8"/>
       <c r="K4" s="19"/>
     </row>
-    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
@@ -4436,7 +4914,7 @@
       </c>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -4465,7 +4943,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -4478,7 +4956,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -4491,7 +4969,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
@@ -4522,7 +5000,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8" t="s">
@@ -4553,7 +5031,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8" t="s">
@@ -4580,7 +5058,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4593,7 +5071,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="19"/>
     </row>
-    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4605,7 +5083,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4617,7 +5095,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -4629,7 +5107,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A16" s="13" t="s">
         <v>92</v>
       </c>
@@ -4651,7 +5129,7 @@
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A17" s="12">
         <f>SUM(Tabelle27[Estimated time])</f>
         <v>42</v>
@@ -4695,22 +5173,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
@@ -4745,7 +5223,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="9">
         <v>45953</v>
       </c>
@@ -4762,7 +5240,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -4793,7 +5271,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -4824,7 +5302,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -4837,7 +5315,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -4850,7 +5328,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="19"/>
     </row>
-    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -4863,7 +5341,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -4876,7 +5354,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -4889,7 +5367,7 @@
       <c r="J9" s="8"/>
       <c r="K9" s="19"/>
     </row>
-    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -4902,7 +5380,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -4915,7 +5393,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4928,7 +5406,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="19"/>
     </row>
-    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4940,7 +5418,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4952,7 +5430,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -4964,7 +5442,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A16" s="13" t="s">
         <v>92</v>
       </c>
@@ -4986,7 +5464,7 @@
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A17" s="12">
         <f>SUM(Tabelle2710[Estimated time])</f>
         <v>9</v>
@@ -5030,22 +5508,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
@@ -5080,7 +5558,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="9">
         <v>45981</v>
       </c>
@@ -5097,7 +5575,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -5128,7 +5606,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -5157,7 +5635,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
@@ -5186,7 +5664,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -5217,7 +5695,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -5230,7 +5708,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
@@ -5261,7 +5739,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
@@ -5292,7 +5770,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -5305,7 +5783,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -5318,7 +5796,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -5330,7 +5808,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -5342,7 +5820,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -5354,7 +5832,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A15" s="13" t="s">
         <v>92</v>
       </c>
@@ -5376,7 +5854,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A16" s="12">
         <f>SUM(Tabelle271013[Estimated time])</f>
         <v>22</v>
@@ -5419,22 +5897,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
@@ -5469,7 +5947,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="9">
         <v>45623</v>
       </c>
@@ -5486,7 +5964,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -5517,7 +5995,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -5530,7 +6008,7 @@
       <c r="J4" s="8"/>
       <c r="K4" s="19"/>
     </row>
-    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -5543,7 +6021,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -5556,7 +6034,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="19"/>
     </row>
-    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
@@ -5587,7 +6065,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
@@ -5604,7 +6082,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
@@ -5635,7 +6113,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -5648,7 +6126,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -5661,7 +6139,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -5673,7 +6151,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -5685,7 +6163,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -5697,7 +6175,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A15" s="13" t="s">
         <v>92</v>
       </c>
@@ -5719,7 +6197,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A16" s="12">
         <f>SUM(Tabelle27101316[Estimated time])</f>
         <v>17</v>
@@ -5758,24 +6236,348 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD3B4F1C-3BF1-40C7-BF61-F9F2FD9C1FB4}">
+  <sheetPr>
+    <tabColor theme="0"/>
+  </sheetPr>
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="9">
+        <v>46002</v>
+      </c>
+      <c r="B2" s="9">
+        <v>46007</v>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="19"/>
+    </row>
+    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="19"/>
+    </row>
+    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A4" s="8"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="G4" s="8">
+        <v>4</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="I4" s="8">
+        <v>5</v>
+      </c>
+      <c r="J4" s="8">
+        <v>5</v>
+      </c>
+      <c r="K4" s="19"/>
+    </row>
+    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="19"/>
+    </row>
+    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="19"/>
+    </row>
+    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="19"/>
+    </row>
+    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="G8" s="8">
+        <v>3</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="19"/>
+    </row>
+    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="I9" s="8">
+        <v>5</v>
+      </c>
+      <c r="J9" s="8">
+        <v>6</v>
+      </c>
+      <c r="K9" s="19"/>
+    </row>
+    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="19"/>
+    </row>
+    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="19"/>
+    </row>
+    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+    </row>
+    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+    </row>
+    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A15" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="D15" s="8"/>
+      <c r="E15" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+    </row>
+    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A16" s="12">
+        <f>SUM(Tabelle2710131619[Estimated time])</f>
+        <v>7</v>
+      </c>
+      <c r="B16" s="12">
+        <f>SUM(Tabelle2710131619[Time in Hours])</f>
+        <v>11</v>
+      </c>
+      <c r="C16" s="12">
+        <f>Tabelle3811141720[[#This Row],[Estimated time]]-Tabelle3811141720[[#This Row],[Actual time]]</f>
+        <v>-4</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="12">
+        <f>SUM(Tabelle2710131619[Story points])</f>
+        <v>10</v>
+      </c>
+      <c r="F16" s="12">
+        <f>Tabelle4912151821[[#This Row],[Total Storypoints ]]/Tabelle3811141720[[#This Row],[Actual time]]</f>
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="3">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7C2A55-0520-4EB5-86E6-237FE14873A1}">
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:J27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="86.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="64.5" style="23" customWidth="1"/>
-    <col min="6" max="6" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="86.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.453125" style="23" customWidth="1"/>
+    <col min="6" max="6" width="10.1796875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -5802,7 +6604,7 @@
       </c>
       <c r="J1" s="17"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -5827,7 +6629,7 @@
       </c>
       <c r="J2" s="17"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -5852,7 +6654,7 @@
       </c>
       <c r="J3" s="17"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -5875,7 +6677,7 @@
       <c r="H4" s="2"/>
       <c r="J4" s="17"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -5900,7 +6702,7 @@
       </c>
       <c r="J5" s="17"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -5925,7 +6727,7 @@
       </c>
       <c r="J6" s="17"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -5950,7 +6752,7 @@
       </c>
       <c r="J7" s="17"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -5975,7 +6777,7 @@
       </c>
       <c r="J8" s="17"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -6000,7 +6802,7 @@
       </c>
       <c r="J9" s="17"/>
     </row>
-    <row r="10" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
@@ -6025,7 +6827,7 @@
       <c r="H10" s="2"/>
       <c r="J10" s="17"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
@@ -6050,7 +6852,7 @@
       </c>
       <c r="J11" s="17"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>28</v>
       </c>
@@ -6075,7 +6877,7 @@
       </c>
       <c r="J12" s="17"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>31</v>
       </c>
@@ -6100,7 +6902,7 @@
       </c>
       <c r="J13" s="17"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -6125,7 +6927,7 @@
       </c>
       <c r="J14" s="17"/>
     </row>
-    <row r="15" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>35</v>
       </c>
@@ -6142,15 +6944,17 @@
         <v>164</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>8</v>
+        <v>168</v>
       </c>
       <c r="G15" s="2">
         <v>5</v>
       </c>
-      <c r="H15" s="2"/>
+      <c r="H15" s="2">
+        <v>6</v>
+      </c>
       <c r="J15" s="17"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>36</v>
       </c>
@@ -6173,7 +6977,7 @@
       <c r="H16" s="2"/>
       <c r="J16" s="17"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>39</v>
       </c>
@@ -6198,7 +7002,7 @@
       </c>
       <c r="J17" s="17"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>40</v>
       </c>
@@ -6223,7 +7027,7 @@
       </c>
       <c r="J18" s="17"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>43</v>
       </c>
@@ -6248,7 +7052,7 @@
       </c>
       <c r="J19" s="17"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>46</v>
       </c>
@@ -6273,7 +7077,7 @@
       </c>
       <c r="J20" s="17"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>49</v>
       </c>
@@ -6296,7 +7100,7 @@
       <c r="H21" s="2"/>
       <c r="J21" s="17"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>52</v>
       </c>
@@ -6319,7 +7123,7 @@
       <c r="H22" s="2"/>
       <c r="J22" s="17"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>55</v>
       </c>
@@ -6344,7 +7148,7 @@
       </c>
       <c r="J23" s="17"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>58</v>
       </c>
@@ -6367,40 +7171,66 @@
       <c r="H24" s="2"/>
       <c r="J24" s="17"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="C25" s="2">
+        <v>6</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E25" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G25" s="2">
+        <v>3</v>
+      </c>
+      <c r="H25" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B26" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C26" s="2">
         <v>15</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E25" s="20"/>
-      <c r="F25" s="2" t="s">
+      <c r="E26" s="20"/>
+      <c r="F26" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G25" s="2">
+      <c r="G26" s="2">
         <v>5</v>
       </c>
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="4"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4">
+      <c r="H26" s="2"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" s="4"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4">
         <f>SUM(G2:G24)</f>
         <v>124</v>
       </c>
-      <c r="H26" s="4"/>
+      <c r="H27" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
added light function, changed light button beaviour
</commit_message>
<xml_diff>
--- a/aquasphere/Excel_File/AquaSphare.xlsx
+++ b/aquasphere/Excel_File/AquaSphare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\43680\Desktop\Schule\SYP\Aquarium\aquasphere\Excel_File\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielhoheneder/Desktop/Schule/syp/AquaSphere/aquasphere/Excel_File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13D9FE3-A397-44FB-BAC5-B8AF8FC4DB0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8EA61E-4E12-CB40-AB47-0558D1F2F0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Dashboard" sheetId="2" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="182">
   <si>
     <t>Story ID</t>
   </si>
@@ -596,6 +596,25 @@
   </si>
   <si>
     <t>Pflanzen sollen sich passiv Positiv auf die Sauberkeit des Aquariums auswirken, Putzfische sollen ebenfalls passiv für Sauberkeit sorgen. Schmutzige Aquairen sollen weniger "Geld" produzieren</t>
+  </si>
+  <si>
+    <t>AQU26</t>
+  </si>
+  <si>
+    <t>Schmutz</t>
+  </si>
+  <si>
+    <t>Als Nutzer möchte ich, dass sich der Schmutz realistisch verhält.</t>
+  </si>
+  <si>
+    <t>Schmutz muss die Sichtbarkeit der Fische beeinträchtigen und das Wasser verfärben</t>
+  </si>
+  <si>
+    <t>Onboarding</t>
+  </si>
+  <si>
+    <t>Wenn das Spiel das erste Mal gestartet wird, bekomme ich die wichtigsten Regeln in einem Splash Screen
+Es gibt einen Button, mit dem ich den Splashscreen herzeigen kann</t>
   </si>
 </sst>
 </file>
@@ -737,7 +756,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -770,403 +789,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Prozent" xfId="1" builtinId="5"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="151">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF0F9ED5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF0F9ED5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1275,6 +906,397 @@
           <bgColor theme="3" tint="0.499984740745262"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -3584,36 +3606,36 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{E37FAD70-20F3-4912-82B8-9AC496901DBE}" name="Tabelle2710131619" displayName="Tabelle2710131619" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
-  <autoFilter ref="A1:K11" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{E37FAD70-20F3-4912-82B8-9AC496901DBE}" name="Tabelle2710131619" displayName="Tabelle2710131619" ref="A1:K14" insertRowShift="1" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+  <autoFilter ref="A1:K14" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{D532321B-43A9-4C7B-9711-0E9DB0F36080}" name="Sprint Start" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{F9445A15-FEA9-4142-9284-D23FEC81E85A}" name="Sprint End" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{98E29721-27A3-49D9-AB54-E3E822D61773}" name="User" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{A6CFA86C-B64A-4D7B-988B-D7EA90AE832B}" name="ID" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{2A363B76-0FF0-4E35-8B0D-D3DFE428B184}" name="Epic" dataDxfId="15"/>
-    <tableColumn id="12" xr3:uid="{58EF9BAF-7539-44AE-B4EA-ED1E3E2C43A2}" name="User Story /Task" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{5812FBDE-2CCF-4471-BA12-4B4E981FB0F8}" name="Estimated time" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{9D350C75-9112-414E-B33C-95BA4ED272B4}" name="COS (Criteria of Satisfaction)" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{79971A75-750E-427F-A5B6-5A61FA1008BB}" name="Story points" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{F15B638A-5756-448D-BFF1-F83357264427}" name="Time in Hours" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{5419A239-65A0-4210-A072-8D48A4908096}" name="Status" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{D532321B-43A9-4C7B-9711-0E9DB0F36080}" name="Sprint Start" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{F9445A15-FEA9-4142-9284-D23FEC81E85A}" name="Sprint End" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{98E29721-27A3-49D9-AB54-E3E822D61773}" name="User" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{A6CFA86C-B64A-4D7B-988B-D7EA90AE832B}" name="ID" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{2A363B76-0FF0-4E35-8B0D-D3DFE428B184}" name="Epic" dataDxfId="25"/>
+    <tableColumn id="12" xr3:uid="{58EF9BAF-7539-44AE-B4EA-ED1E3E2C43A2}" name="User Story /Task" dataDxfId="24"/>
+    <tableColumn id="11" xr3:uid="{5812FBDE-2CCF-4471-BA12-4B4E981FB0F8}" name="Estimated time" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{9D350C75-9112-414E-B33C-95BA4ED272B4}" name="COS (Criteria of Satisfaction)" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{79971A75-750E-427F-A5B6-5A61FA1008BB}" name="Story points" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{F15B638A-5756-448D-BFF1-F83357264427}" name="Time in Hours" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{5419A239-65A0-4210-A072-8D48A4908096}" name="Status" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{1868505A-CACE-44B2-A7EA-9FE64E58BA8A}" name="Tabelle3811141720" displayName="Tabelle3811141720" ref="A15:C16" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A15:C16" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{1868505A-CACE-44B2-A7EA-9FE64E58BA8A}" name="Tabelle3811141720" displayName="Tabelle3811141720" ref="A18:C19" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+  <autoFilter ref="A18:C19" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{3A312704-DAF9-41C4-9ED9-5DD84799E905}" name="Estimated time" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{3A312704-DAF9-41C4-9ED9-5DD84799E905}" name="Estimated time" dataDxfId="16">
       <calculatedColumnFormula>SUM(Tabelle2710131619[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{72BDDA5F-E86A-4485-B7A7-C4A72345EFC4}" name="Actual time" dataDxfId="5">
+    <tableColumn id="2" xr3:uid="{72BDDA5F-E86A-4485-B7A7-C4A72345EFC4}" name="Actual time" dataDxfId="15">
       <calculatedColumnFormula>SUM(Tabelle2710131619[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{223E53E9-D637-4AC0-9A6C-5591B23BB953}" name="Delta" dataDxfId="4">
+    <tableColumn id="3" xr3:uid="{223E53E9-D637-4AC0-9A6C-5591B23BB953}" name="Delta" dataDxfId="14">
       <calculatedColumnFormula>Tabelle3811141720[[#This Row],[Estimated time]]-Tabelle3811141720[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3622,13 +3644,13 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{F7C4B985-A6EE-4B5E-BF93-A6081AE08433}" name="Tabelle4912151821" displayName="Tabelle4912151821" ref="E15:F16" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
-  <autoFilter ref="E15:F16" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{F7C4B985-A6EE-4B5E-BF93-A6081AE08433}" name="Tabelle4912151821" displayName="Tabelle4912151821" ref="E18:F19" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="E18:F19" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{DC2B1F8F-41E8-42FD-87FA-7DF04FEE86E6}" name="Total Storypoints " dataDxfId="1">
+    <tableColumn id="1" xr3:uid="{DC2B1F8F-41E8-42FD-87FA-7DF04FEE86E6}" name="Total Storypoints " dataDxfId="11">
       <calculatedColumnFormula>SUM(Tabelle2710131619[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{913BEBDF-DC3B-496C-982F-AE7F617915B6}" name="Effort/Hour" dataDxfId="0">
+    <tableColumn id="2" xr3:uid="{913BEBDF-DC3B-496C-982F-AE7F617915B6}" name="Effort/Hour" dataDxfId="10">
       <calculatedColumnFormula>Tabelle4912151821[[#This Row],[Total Storypoints ]]/Tabelle3811141720[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3656,20 +3678,20 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:H27" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
-  <autoFilter ref="A1:H27" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H27">
-    <sortCondition ref="C9:C27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:H28" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:H28" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H28">
+    <sortCondition ref="C9:C28"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Story" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{57E495A5-904B-1740-A858-653ACCE96658}" name="Acceptance Criteria" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="23"/>
-    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Story" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{57E495A5-904B-1740-A858-653ACCE96658}" name="Acceptance Criteria" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4120,20 +4142,20 @@
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:H17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>4</v>
       </c>
@@ -4159,7 +4181,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>69</v>
       </c>
@@ -4190,7 +4212,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>70</v>
       </c>
@@ -4221,7 +4243,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>71</v>
       </c>
@@ -4253,7 +4275,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>72</v>
       </c>
@@ -4285,7 +4307,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>73</v>
       </c>
@@ -4317,7 +4339,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>74</v>
       </c>
@@ -4329,7 +4351,7 @@
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>75</v>
       </c>
@@ -4341,7 +4363,7 @@
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
     </row>
-    <row r="12" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>76</v>
       </c>
@@ -4349,7 +4371,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>117</v>
       </c>
@@ -4358,7 +4380,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>80</v>
       </c>
@@ -4367,7 +4389,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>77</v>
       </c>
@@ -4376,7 +4398,7 @@
         <v>0.92867647058823533</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>78</v>
       </c>
@@ -4385,7 +4407,7 @@
         <v>0.64383561643835618</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:4" ht="24" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>68</v>
       </c>
@@ -4413,21 +4435,21 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:J16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="95.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="95.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
@@ -4459,7 +4481,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45925</v>
       </c>
@@ -4489,7 +4511,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -4511,7 +4533,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -4531,7 +4553,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -4543,7 +4565,7 @@
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
     </row>
-    <row r="6" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -4571,7 +4593,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
@@ -4597,7 +4619,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
@@ -4621,7 +4643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -4633,7 +4655,7 @@
       <c r="I9" s="8"/>
       <c r="J9" s="8"/>
     </row>
-    <row r="10" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -4645,7 +4667,7 @@
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
     </row>
-    <row r="11" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -4657,7 +4679,7 @@
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
     </row>
-    <row r="12" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -4669,7 +4691,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -4681,7 +4703,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -4693,7 +4715,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>92</v>
       </c>
@@ -4715,7 +4737,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <f>SUM(Tabelle2[Estimated time])</f>
         <v>13</v>
@@ -4758,22 +4780,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
@@ -4808,7 +4830,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45939</v>
       </c>
@@ -4843,7 +4865,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -4872,7 +4894,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -4885,7 +4907,7 @@
       <c r="J4" s="8"/>
       <c r="K4" s="19"/>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
@@ -4914,7 +4936,7 @@
       </c>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -4943,7 +4965,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -4956,7 +4978,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -4969,7 +4991,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
@@ -5000,7 +5022,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8" t="s">
@@ -5031,7 +5053,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8" t="s">
@@ -5058,7 +5080,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -5071,7 +5093,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="19"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -5083,7 +5105,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -5095,7 +5117,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -5107,7 +5129,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>92</v>
       </c>
@@ -5129,7 +5151,7 @@
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <f>SUM(Tabelle27[Estimated time])</f>
         <v>42</v>
@@ -5173,22 +5195,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
@@ -5223,7 +5245,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45953</v>
       </c>
@@ -5240,7 +5262,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -5271,7 +5293,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -5302,7 +5324,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -5315,7 +5337,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -5328,7 +5350,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="19"/>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -5341,7 +5363,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -5354,7 +5376,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -5367,7 +5389,7 @@
       <c r="J9" s="8"/>
       <c r="K9" s="19"/>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -5380,7 +5402,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -5393,7 +5415,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -5406,7 +5428,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="19"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -5418,7 +5440,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -5430,7 +5452,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -5442,7 +5464,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>92</v>
       </c>
@@ -5464,7 +5486,7 @@
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <f>SUM(Tabelle2710[Estimated time])</f>
         <v>9</v>
@@ -5508,22 +5530,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
@@ -5558,7 +5580,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45981</v>
       </c>
@@ -5575,7 +5597,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -5606,7 +5628,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -5635,7 +5657,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
@@ -5664,7 +5686,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
@@ -5695,7 +5717,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -5708,7 +5730,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
@@ -5739,7 +5761,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
@@ -5770,7 +5792,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -5783,7 +5805,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -5796,7 +5818,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -5808,7 +5830,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -5820,7 +5842,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -5832,7 +5854,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>92</v>
       </c>
@@ -5854,7 +5876,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <f>SUM(Tabelle271013[Estimated time])</f>
         <v>22</v>
@@ -5897,22 +5919,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
@@ -5947,7 +5969,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>45623</v>
       </c>
@@ -5964,7 +5986,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -5995,7 +6017,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -6008,7 +6030,7 @@
       <c r="J4" s="8"/>
       <c r="K4" s="19"/>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -6021,7 +6043,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -6034,7 +6056,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="19"/>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
@@ -6065,7 +6087,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
@@ -6082,7 +6104,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
@@ -6113,7 +6135,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -6126,7 +6148,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -6139,7 +6161,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -6151,7 +6173,7 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -6163,7 +6185,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -6175,7 +6197,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>92</v>
       </c>
@@ -6197,7 +6219,7 @@
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <f>SUM(Tabelle27101316[Estimated time])</f>
         <v>17</v>
@@ -6240,23 +6262,23 @@
   <sheetPr>
     <tabColor theme="0"/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="124.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="164.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
@@ -6291,7 +6313,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>46002</v>
       </c>
@@ -6308,7 +6330,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
@@ -6323,7 +6345,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="19"/>
     </row>
-    <row r="4" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -6350,7 +6372,7 @@
       </c>
       <c r="K4" s="19"/>
     </row>
-    <row r="5" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -6365,7 +6387,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="19"/>
     </row>
-    <row r="6" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -6380,7 +6402,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="19"/>
     </row>
-    <row r="7" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -6393,7 +6415,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
@@ -6418,11 +6440,11 @@
       <c r="J8" s="8"/>
       <c r="K8" s="19"/>
     </row>
-    <row r="9" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
+      <c r="D9" s="10"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
@@ -6437,11 +6459,11 @@
       </c>
       <c r="K9" s="19"/>
     </row>
-    <row r="10" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
+      <c r="D10" s="10"/>
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
@@ -6450,20 +6472,38 @@
       <c r="J10" s="8"/>
       <c r="K10" s="19"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="40" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="19"/>
-    </row>
-    <row r="12" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="C11" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="G11" s="8">
+        <v>4</v>
+      </c>
+      <c r="H11" s="24" t="s">
+        <v>181</v>
+      </c>
+      <c r="I11" s="8">
+        <v>5</v>
+      </c>
+      <c r="J11" s="8">
+        <v>3</v>
+      </c>
+      <c r="K11" s="19" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -6474,8 +6514,9 @@
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
-    </row>
-    <row r="13" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K12" s="19"/>
+    </row>
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -6486,8 +6527,9 @@
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
-    </row>
-    <row r="14" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="K13" s="19"/>
+    </row>
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -6498,55 +6540,92 @@
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
-    </row>
-    <row r="15" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A15" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>94</v>
-      </c>
+      <c r="K14" s="19"/>
+    </row>
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
       <c r="D15" s="8"/>
-      <c r="E15" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>123</v>
-      </c>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A16" s="12">
-        <f>SUM(Tabelle2710131619[Estimated time])</f>
-        <v>7</v>
-      </c>
-      <c r="B16" s="12">
-        <f>SUM(Tabelle2710131619[Time in Hours])</f>
-        <v>11</v>
-      </c>
-      <c r="C16" s="12">
-        <f>Tabelle3811141720[[#This Row],[Estimated time]]-Tabelle3811141720[[#This Row],[Actual time]]</f>
-        <v>-4</v>
-      </c>
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
       <c r="D16" s="8"/>
-      <c r="E16" s="12">
-        <f>SUM(Tabelle2710131619[Story points])</f>
-        <v>10</v>
-      </c>
-      <c r="F16" s="12">
-        <f>Tabelle4912151821[[#This Row],[Total Storypoints ]]/Tabelle3811141720[[#This Row],[Actual time]]</f>
-        <v>0.90909090909090906</v>
-      </c>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
+    </row>
+    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+    </row>
+    <row r="18" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+    </row>
+    <row r="19" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="A19" s="12">
+        <f>SUM(Tabelle2710131619[Estimated time])</f>
+        <v>11</v>
+      </c>
+      <c r="B19" s="12">
+        <f>SUM(Tabelle2710131619[Time in Hours])</f>
+        <v>14</v>
+      </c>
+      <c r="C19" s="12">
+        <f>Tabelle3811141720[[#This Row],[Estimated time]]-Tabelle3811141720[[#This Row],[Actual time]]</f>
+        <v>-3</v>
+      </c>
+      <c r="D19" s="8"/>
+      <c r="E19" s="12">
+        <f>SUM(Tabelle2710131619[Story points])</f>
+        <v>15</v>
+      </c>
+      <c r="F19" s="12">
+        <f>Tabelle4912151821[[#This Row],[Total Storypoints ]]/Tabelle3811141720[[#This Row],[Actual time]]</f>
+        <v>1.0714285714285714</v>
+      </c>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -6564,20 +6643,20 @@
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="86.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="64.453125" style="23" customWidth="1"/>
-    <col min="6" max="6" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="86.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.5" style="23" customWidth="1"/>
+    <col min="6" max="6" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -6604,7 +6683,7 @@
       </c>
       <c r="J1" s="17"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -6629,7 +6708,7 @@
       </c>
       <c r="J2" s="17"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -6654,7 +6733,7 @@
       </c>
       <c r="J3" s="17"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -6677,7 +6756,7 @@
       <c r="H4" s="2"/>
       <c r="J4" s="17"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -6702,7 +6781,7 @@
       </c>
       <c r="J5" s="17"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -6727,7 +6806,7 @@
       </c>
       <c r="J6" s="17"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -6752,7 +6831,7 @@
       </c>
       <c r="J7" s="17"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -6777,7 +6856,7 @@
       </c>
       <c r="J8" s="17"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -6802,7 +6881,7 @@
       </c>
       <c r="J9" s="17"/>
     </row>
-    <row r="10" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
@@ -6819,15 +6898,17 @@
         <v>163</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>8</v>
+        <v>168</v>
       </c>
       <c r="G10" s="2">
         <v>5</v>
       </c>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2">
+        <v>6</v>
+      </c>
       <c r="J10" s="17"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
@@ -6852,7 +6933,7 @@
       </c>
       <c r="J11" s="17"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>28</v>
       </c>
@@ -6877,7 +6958,7 @@
       </c>
       <c r="J12" s="17"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>31</v>
       </c>
@@ -6902,7 +6983,7 @@
       </c>
       <c r="J13" s="17"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -6927,7 +7008,7 @@
       </c>
       <c r="J14" s="17"/>
     </row>
-    <row r="15" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>35</v>
       </c>
@@ -6954,7 +7035,7 @@
       </c>
       <c r="J15" s="17"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>36</v>
       </c>
@@ -6977,7 +7058,7 @@
       <c r="H16" s="2"/>
       <c r="J16" s="17"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>39</v>
       </c>
@@ -7002,7 +7083,7 @@
       </c>
       <c r="J17" s="17"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>40</v>
       </c>
@@ -7027,7 +7108,7 @@
       </c>
       <c r="J18" s="17"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>43</v>
       </c>
@@ -7052,7 +7133,7 @@
       </c>
       <c r="J19" s="17"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>46</v>
       </c>
@@ -7077,7 +7158,7 @@
       </c>
       <c r="J20" s="17"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>49</v>
       </c>
@@ -7100,7 +7181,7 @@
       <c r="H21" s="2"/>
       <c r="J21" s="17"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>52</v>
       </c>
@@ -7123,7 +7204,7 @@
       <c r="H22" s="2"/>
       <c r="J22" s="17"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>55</v>
       </c>
@@ -7148,7 +7229,7 @@
       </c>
       <c r="J23" s="17"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>58</v>
       </c>
@@ -7171,7 +7252,7 @@
       <c r="H24" s="2"/>
       <c r="J24" s="17"/>
     </row>
-    <row r="25" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>173</v>
       </c>
@@ -7197,40 +7278,66 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="C26" s="2">
+        <v>13</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E26" s="20" t="s">
+        <v>179</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G26" s="2">
+        <v>3</v>
+      </c>
+      <c r="H26" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B27" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="2">
+      <c r="C27" s="2">
         <v>15</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E26" s="20"/>
-      <c r="F26" s="2" t="s">
+      <c r="E27" s="20"/>
+      <c r="F27" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G26" s="2">
+      <c r="G27" s="2">
         <v>5</v>
       </c>
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="4"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4">
+      <c r="H27" s="2"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28" s="4"/>
+      <c r="B28" s="16"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4">
         <f>SUM(G2:G24)</f>
         <v>124</v>
       </c>
-      <c r="H27" s="4"/>
+      <c r="H28" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
fixed lighting; updated excelFile
</commit_message>
<xml_diff>
--- a/aquasphere/Excel_File/AquaSphare.xlsx
+++ b/aquasphere/Excel_File/AquaSphare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielhoheneder/Desktop/Schule/syp/AquaSphere/aquasphere/Excel_File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8EA61E-4E12-CB40-AB47-0558D1F2F0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0256BA19-9CAF-5546-9038-384DFDD4516A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="25820" windowHeight="15500" xr2:uid="{3C511D28-10C8-4337-AED7-CFA66BBB7484}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Dashboard" sheetId="2" r:id="rId1"/>
@@ -20,7 +20,8 @@
     <sheet name="Sprint4" sheetId="6" r:id="rId5"/>
     <sheet name="Sprint5" sheetId="7" r:id="rId6"/>
     <sheet name="Sprint6" sheetId="8" r:id="rId7"/>
-    <sheet name="Storys" sheetId="1" r:id="rId8"/>
+    <sheet name="Sprint7" sheetId="10" r:id="rId8"/>
+    <sheet name="Storys" sheetId="1" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -65,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="181">
   <si>
     <t>Story ID</t>
   </si>
@@ -91,9 +92,6 @@
     <t>Als Nutzer möchte ich ein virtuelles Aquarium sehen.</t>
   </si>
   <si>
-    <t>Not Started</t>
-  </si>
-  <si>
     <t>AQU2</t>
   </si>
   <si>
@@ -145,12 +143,6 @@
     <t>AQU10</t>
   </si>
   <si>
-    <t>Anpassung</t>
-  </si>
-  <si>
-    <t>Als Nutzer möchte ich die Aquarium-Größe ändern.</t>
-  </si>
-  <si>
     <t>AQU11</t>
   </si>
   <si>
@@ -224,12 +216,6 @@
   </si>
   <si>
     <t>AQU21</t>
-  </si>
-  <si>
-    <t>Statistiken</t>
-  </si>
-  <si>
-    <t>Als Nutzer möchte ich Statistiken zu meinem Aquarium sehen.</t>
   </si>
   <si>
     <t>AQU22</t>
@@ -574,9 +560,6 @@
     <t>* Wenn man ausloggt, geht die Zeit automatisch wieder auf 1-fach zurück</t>
   </si>
   <si>
-    <t>Started</t>
-  </si>
-  <si>
     <t>Reinigung</t>
   </si>
   <si>
@@ -589,16 +572,10 @@
     <t>Schmutzige Aquairen sollen weniger "Geld" produzieren</t>
   </si>
   <si>
-    <t>AQU25</t>
-  </si>
-  <si>
     <t>Eco</t>
   </si>
   <si>
     <t>Pflanzen sollen sich passiv Positiv auf die Sauberkeit des Aquariums auswirken, Putzfische sollen ebenfalls passiv für Sauberkeit sorgen. Schmutzige Aquairen sollen weniger "Geld" produzieren</t>
-  </si>
-  <si>
-    <t>AQU26</t>
   </si>
   <si>
     <t>Schmutz</t>
@@ -615,13 +592,34 @@
   <si>
     <t>Wenn das Spiel das erste Mal gestartet wird, bekomme ich die wichtigsten Regeln in einem Splash Screen
 Es gibt einen Button, mit dem ich den Splashscreen herzeigen kann</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daten werden durch die Datenbank geschützt gespeichert. </t>
+  </si>
+  <si>
+    <t>Beleuchtung funktioniert und ist in verschiedenen Farben verfügbar.</t>
+  </si>
+  <si>
+    <t>Verschiedene Themes stehen zur Auswahl und können durch Punkte oder Erfolge freigeschaltete werden.</t>
+  </si>
+  <si>
+    <t>Erfolge setzen verschieden Bedignungen vorraus welche erüllt sein müssen um diese zu erreichen. Achievements schalten verschieden Dinge frei.</t>
+  </si>
+  <si>
+    <t>MR</t>
+  </si>
+  <si>
+    <t>UI/UX, Reinigung, Onboarding</t>
+  </si>
+  <si>
+    <t>Licht, Theme, Achiev, DataProt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -693,8 +691,15 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -731,8 +736,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAE9F8"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -751,12 +762,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF44B3E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF44B3E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF44B3E1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF44B3E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF44B3E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -792,12 +827,425 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="151">
+  <dxfs count="173">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF0F9ED5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3340,26 +3788,6 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="16"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.89999084444715716"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -3458,25 +3886,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AAF41172-5838-4CA9-A8A2-78B1E57ACF1F}" name="Tabelle1" displayName="Tabelle1" ref="A1:H8" totalsRowShown="0" headerRowDxfId="150" dataDxfId="149">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AAF41172-5838-4CA9-A8A2-78B1E57ACF1F}" name="Tabelle1" displayName="Tabelle1" ref="A1:H8" totalsRowShown="0" headerRowDxfId="172" dataDxfId="171">
   <autoFilter ref="A1:H8" xr:uid="{AAF41172-5838-4CA9-A8A2-78B1E57ACF1F}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{8BB8E342-544E-430C-A72A-9EBF9676D447}" name="Sprint" dataDxfId="148"/>
-    <tableColumn id="9" xr3:uid="{96A939A8-DA63-4E70-B123-D31A897D4192}" name="Story ID" dataDxfId="147"/>
-    <tableColumn id="2" xr3:uid="{CB307D23-EE39-436B-9E06-9E7789362DB6}" name="Estimated Hours" dataDxfId="146">
+    <tableColumn id="1" xr3:uid="{8BB8E342-544E-430C-A72A-9EBF9676D447}" name="Sprint" dataDxfId="170"/>
+    <tableColumn id="9" xr3:uid="{96A939A8-DA63-4E70-B123-D31A897D4192}" name="Story ID" dataDxfId="169"/>
+    <tableColumn id="2" xr3:uid="{CB307D23-EE39-436B-9E06-9E7789362DB6}" name="Estimated Hours" dataDxfId="168">
       <calculatedColumnFormula array="1">Tabelle3[Estimated time]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{5EFC7DEC-DFDE-454B-90FC-2713EB4181D8}" name="Actual Hours" dataDxfId="145">
+    <tableColumn id="3" xr3:uid="{5EFC7DEC-DFDE-454B-90FC-2713EB4181D8}" name="Actual Hours" dataDxfId="167">
       <calculatedColumnFormula array="1">Tabelle3[Actual time]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D6FF0659-1B35-4F09-B5A7-D22FEF5F7C3F}" name="Accomplished Story Points" dataDxfId="144">
+    <tableColumn id="4" xr3:uid="{D6FF0659-1B35-4F09-B5A7-D22FEF5F7C3F}" name="Accomplished Story Points" dataDxfId="166">
       <calculatedColumnFormula array="1">Tabelle4[[Total Storypoints ]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{9CD2DBE3-2E45-4440-8D7A-2A03A0291AAD}" name="Velocity" dataDxfId="143">
-      <calculatedColumnFormula>Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]]</calculatedColumnFormula>
+    <tableColumn id="5" xr3:uid="{9CD2DBE3-2E45-4440-8D7A-2A03A0291AAD}" name="Velocity" dataDxfId="0">
+      <calculatedColumnFormula>Tabelle1[[#This Row],[Estimated Hours]]/Tabelle1[[#This Row],[Actual Hours]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{1977DF7A-0A05-43B5-99D3-B72159480780}" name="Total Storypoints" dataDxfId="142"/>
-    <tableColumn id="7" xr3:uid="{D8A5F5FE-B9BC-448A-A9E7-3D00888AE639}" name="Storypoints Left" dataDxfId="141">
+    <tableColumn id="6" xr3:uid="{1977DF7A-0A05-43B5-99D3-B72159480780}" name="Total Storypoints" dataDxfId="165"/>
+    <tableColumn id="7" xr3:uid="{D8A5F5FE-B9BC-448A-A9E7-3D00888AE639}" name="Storypoints Left" dataDxfId="164">
       <calculatedColumnFormula>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3485,13 +3913,13 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0134C802-458D-4153-B0D4-D8B08E02E26A}" name="Tabelle4912" displayName="Tabelle4912" ref="E16:F17" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0134C802-458D-4153-B0D4-D8B08E02E26A}" name="Tabelle4912" displayName="Tabelle4912" ref="E16:F17" totalsRowShown="0" headerRowDxfId="102" dataDxfId="101">
   <autoFilter ref="E16:F17" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C3438C75-AD69-46E0-B1BD-0445ED469483}" name="Total Storypoints " dataDxfId="77">
+    <tableColumn id="1" xr3:uid="{C3438C75-AD69-46E0-B1BD-0445ED469483}" name="Total Storypoints " dataDxfId="100">
       <calculatedColumnFormula>SUM(Tabelle2710[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0655740B-E1AB-4BD3-B7CA-852D4C79FC17}" name="Effort/Hour" dataDxfId="76">
+    <tableColumn id="2" xr3:uid="{0655740B-E1AB-4BD3-B7CA-852D4C79FC17}" name="Effort/Hour" dataDxfId="99">
       <calculatedColumnFormula>Tabelle4912[[#This Row],[Total Storypoints ]]/Tabelle3811[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3500,36 +3928,36 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}" name="Tabelle271013" displayName="Tabelle271013" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}" name="Tabelle271013" displayName="Tabelle271013" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="98" dataDxfId="97">
   <autoFilter ref="A1:K11" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{946A4B14-799A-49AD-8E3E-31E3F4BBE559}" name="Sprint Start" dataDxfId="73"/>
-    <tableColumn id="2" xr3:uid="{E61A962F-4EE4-4843-AF21-C647918EECAB}" name="Sprint End" dataDxfId="72"/>
-    <tableColumn id="3" xr3:uid="{4EC50B40-18BD-4D00-8BE2-5596A9347BB8}" name="User" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{2A1F175E-D14E-491C-B452-39567CF84CD6}" name="ID" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{DCE5121F-D243-470B-B0AF-D0EE5264DD5A}" name="Epic" dataDxfId="69"/>
-    <tableColumn id="12" xr3:uid="{45FDCCAE-F13D-47C1-B91E-2EF3CC9A5BA0}" name="User Story /Task" dataDxfId="68"/>
-    <tableColumn id="11" xr3:uid="{4057DF12-8977-4284-BF2B-9ED3AAE7221F}" name="Estimated time" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{08443A2E-5832-4299-8009-1F0D489DEE15}" name="COS (Criteria of Satisfaction)" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{8777A429-C11B-4CDC-BB2F-785D0BC89DAB}" name="Story points" dataDxfId="65"/>
-    <tableColumn id="10" xr3:uid="{0B18443F-D8D9-4015-8EAA-7050016E43C2}" name="Time in Hours" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{5C5B5C91-6376-4597-B69B-4D162307C569}" name="Status" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{946A4B14-799A-49AD-8E3E-31E3F4BBE559}" name="Sprint Start" dataDxfId="96"/>
+    <tableColumn id="2" xr3:uid="{E61A962F-4EE4-4843-AF21-C647918EECAB}" name="Sprint End" dataDxfId="95"/>
+    <tableColumn id="3" xr3:uid="{4EC50B40-18BD-4D00-8BE2-5596A9347BB8}" name="User" dataDxfId="94"/>
+    <tableColumn id="5" xr3:uid="{2A1F175E-D14E-491C-B452-39567CF84CD6}" name="ID" dataDxfId="93"/>
+    <tableColumn id="6" xr3:uid="{DCE5121F-D243-470B-B0AF-D0EE5264DD5A}" name="Epic" dataDxfId="92"/>
+    <tableColumn id="12" xr3:uid="{45FDCCAE-F13D-47C1-B91E-2EF3CC9A5BA0}" name="User Story /Task" dataDxfId="91"/>
+    <tableColumn id="11" xr3:uid="{4057DF12-8977-4284-BF2B-9ED3AAE7221F}" name="Estimated time" dataDxfId="90"/>
+    <tableColumn id="8" xr3:uid="{08443A2E-5832-4299-8009-1F0D489DEE15}" name="COS (Criteria of Satisfaction)" dataDxfId="89"/>
+    <tableColumn id="9" xr3:uid="{8777A429-C11B-4CDC-BB2F-785D0BC89DAB}" name="Story points" dataDxfId="88"/>
+    <tableColumn id="10" xr3:uid="{0B18443F-D8D9-4015-8EAA-7050016E43C2}" name="Time in Hours" dataDxfId="87"/>
+    <tableColumn id="4" xr3:uid="{5C5B5C91-6376-4597-B69B-4D162307C569}" name="Status" dataDxfId="86"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}" name="Tabelle381114" displayName="Tabelle381114" ref="A15:C16" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}" name="Tabelle381114" displayName="Tabelle381114" ref="A15:C16" totalsRowShown="0" headerRowDxfId="85" dataDxfId="84">
   <autoFilter ref="A15:C16" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{E71994D0-AB06-482B-8487-03AB7E3B1FF7}" name="Estimated time" dataDxfId="60">
+    <tableColumn id="1" xr3:uid="{E71994D0-AB06-482B-8487-03AB7E3B1FF7}" name="Estimated time" dataDxfId="83">
       <calculatedColumnFormula>SUM(Tabelle271013[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E607785B-5B58-4D1E-81ED-45AAAAF488F0}" name="Actual time" dataDxfId="59">
+    <tableColumn id="2" xr3:uid="{E607785B-5B58-4D1E-81ED-45AAAAF488F0}" name="Actual time" dataDxfId="82">
       <calculatedColumnFormula>SUM(Tabelle271013[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{0197CFBA-597E-49C6-88E5-ABAC17763EA4}" name="Delta" dataDxfId="58">
+    <tableColumn id="3" xr3:uid="{0197CFBA-597E-49C6-88E5-ABAC17763EA4}" name="Delta" dataDxfId="81">
       <calculatedColumnFormula>Tabelle381114[[#This Row],[Estimated time]]-Tabelle381114[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3538,13 +3966,13 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}" name="Tabelle491215" displayName="Tabelle491215" ref="E15:F16" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}" name="Tabelle491215" displayName="Tabelle491215" ref="E15:F16" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79">
   <autoFilter ref="E15:F16" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{E0381C51-E5FF-4087-9146-76E105FE701A}" name="Total Storypoints " dataDxfId="55">
+    <tableColumn id="1" xr3:uid="{E0381C51-E5FF-4087-9146-76E105FE701A}" name="Total Storypoints " dataDxfId="78">
       <calculatedColumnFormula>SUM(Tabelle271013[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0971B46C-CFAA-4F13-88AB-CDC5655C1F84}" name="Effort/Hour" dataDxfId="54">
+    <tableColumn id="2" xr3:uid="{0971B46C-CFAA-4F13-88AB-CDC5655C1F84}" name="Effort/Hour" dataDxfId="77">
       <calculatedColumnFormula>Tabelle491215[[#This Row],[Total Storypoints ]]/Tabelle381114[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3553,36 +3981,36 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{235F589F-8BC0-4A3D-A02E-03E630D61504}" name="Tabelle27101316" displayName="Tabelle27101316" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{235F589F-8BC0-4A3D-A02E-03E630D61504}" name="Tabelle27101316" displayName="Tabelle27101316" ref="A1:K11" insertRowShift="1" totalsRowShown="0" headerRowDxfId="76" dataDxfId="75">
   <autoFilter ref="A1:K11" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{B7D16283-E8F5-4C03-BEC2-39D9F536B2DF}" name="Sprint Start" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{743B7730-744D-48F9-8435-134B358D299C}" name="Sprint End" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{6BB0BFF2-8337-4911-B853-52953695FFB8}" name="User" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{23B9485C-C756-4653-9A7E-4CBFBC4BDCC9}" name="ID" dataDxfId="48"/>
-    <tableColumn id="6" xr3:uid="{DA3B151D-2F3B-4817-810C-2B84F6D521DF}" name="Epic" dataDxfId="47"/>
-    <tableColumn id="12" xr3:uid="{0B21ADB3-F002-4AC8-8EFB-36998E0BA400}" name="User Story /Task" dataDxfId="46"/>
-    <tableColumn id="11" xr3:uid="{0AF7F7D2-16D8-4903-AFB0-E002FAFE9A7B}" name="Estimated time" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{2F945FB5-B8D6-4015-9863-4264314B3D66}" name="COS (Criteria of Satisfaction)" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{72841B6A-9C3A-4632-878E-ADBD76467B91}" name="Story points" dataDxfId="43"/>
-    <tableColumn id="10" xr3:uid="{99643A57-EC89-4FC7-B6E0-CEECFE14CE6B}" name="Time in Hours" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{D3F46A45-6C79-4B7E-9924-30DF1A278D97}" name="Status" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{B7D16283-E8F5-4C03-BEC2-39D9F536B2DF}" name="Sprint Start" dataDxfId="74"/>
+    <tableColumn id="2" xr3:uid="{743B7730-744D-48F9-8435-134B358D299C}" name="Sprint End" dataDxfId="73"/>
+    <tableColumn id="3" xr3:uid="{6BB0BFF2-8337-4911-B853-52953695FFB8}" name="User" dataDxfId="72"/>
+    <tableColumn id="5" xr3:uid="{23B9485C-C756-4653-9A7E-4CBFBC4BDCC9}" name="ID" dataDxfId="71"/>
+    <tableColumn id="6" xr3:uid="{DA3B151D-2F3B-4817-810C-2B84F6D521DF}" name="Epic" dataDxfId="70"/>
+    <tableColumn id="12" xr3:uid="{0B21ADB3-F002-4AC8-8EFB-36998E0BA400}" name="User Story /Task" dataDxfId="69"/>
+    <tableColumn id="11" xr3:uid="{0AF7F7D2-16D8-4903-AFB0-E002FAFE9A7B}" name="Estimated time" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{2F945FB5-B8D6-4015-9863-4264314B3D66}" name="COS (Criteria of Satisfaction)" dataDxfId="67"/>
+    <tableColumn id="9" xr3:uid="{72841B6A-9C3A-4632-878E-ADBD76467B91}" name="Story points" dataDxfId="66"/>
+    <tableColumn id="10" xr3:uid="{99643A57-EC89-4FC7-B6E0-CEECFE14CE6B}" name="Time in Hours" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{D3F46A45-6C79-4B7E-9924-30DF1A278D97}" name="Status" dataDxfId="64"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{E0805314-F662-4E1D-85A9-F2EC30EC262D}" name="Tabelle38111417" displayName="Tabelle38111417" ref="A15:C16" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{E0805314-F662-4E1D-85A9-F2EC30EC262D}" name="Tabelle38111417" displayName="Tabelle38111417" ref="A15:C16" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
   <autoFilter ref="A15:C16" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{1993629C-98D2-4E46-B14A-696AAE563315}" name="Estimated time" dataDxfId="38">
+    <tableColumn id="1" xr3:uid="{1993629C-98D2-4E46-B14A-696AAE563315}" name="Estimated time" dataDxfId="61">
       <calculatedColumnFormula>SUM(Tabelle27101316[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C3F5A116-86A6-4D3A-9417-88FA122B0C81}" name="Actual time" dataDxfId="37">
+    <tableColumn id="2" xr3:uid="{C3F5A116-86A6-4D3A-9417-88FA122B0C81}" name="Actual time" dataDxfId="60">
       <calculatedColumnFormula>SUM(Tabelle27101316[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B86C31E6-5405-4B45-9B86-86A0C1DBF35C}" name="Delta" dataDxfId="36">
+    <tableColumn id="3" xr3:uid="{B86C31E6-5405-4B45-9B86-86A0C1DBF35C}" name="Delta" dataDxfId="59">
       <calculatedColumnFormula>Tabelle38111417[[#This Row],[Estimated time]]-Tabelle38111417[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3591,13 +4019,13 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{FE78B35D-B1A7-42FC-BB42-AF310800AF69}" name="Tabelle49121518" displayName="Tabelle49121518" ref="E15:F16" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{FE78B35D-B1A7-42FC-BB42-AF310800AF69}" name="Tabelle49121518" displayName="Tabelle49121518" ref="E15:F16" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
   <autoFilter ref="E15:F16" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{E7934959-5DF7-4D4C-858C-1FAD310B1F3B}" name="Total Storypoints " dataDxfId="33">
+    <tableColumn id="1" xr3:uid="{E7934959-5DF7-4D4C-858C-1FAD310B1F3B}" name="Total Storypoints " dataDxfId="56">
       <calculatedColumnFormula>SUM(Tabelle27101316[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D7E6F4E2-872C-4E38-9126-8A958E19087E}" name="Effort/Hour" dataDxfId="32">
+    <tableColumn id="2" xr3:uid="{D7E6F4E2-872C-4E38-9126-8A958E19087E}" name="Effort/Hour" dataDxfId="55">
       <calculatedColumnFormula>Tabelle49121518[[#This Row],[Total Storypoints ]]/Tabelle38111417[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3606,36 +4034,36 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{E37FAD70-20F3-4912-82B8-9AC496901DBE}" name="Tabelle2710131619" displayName="Tabelle2710131619" ref="A1:K14" insertRowShift="1" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{E37FAD70-20F3-4912-82B8-9AC496901DBE}" name="Tabelle2710131619" displayName="Tabelle2710131619" ref="A1:K14" insertRowShift="1" totalsRowShown="0" headerRowDxfId="54" dataDxfId="53">
   <autoFilter ref="A1:K14" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{D532321B-43A9-4C7B-9711-0E9DB0F36080}" name="Sprint Start" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{F9445A15-FEA9-4142-9284-D23FEC81E85A}" name="Sprint End" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{98E29721-27A3-49D9-AB54-E3E822D61773}" name="User" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{A6CFA86C-B64A-4D7B-988B-D7EA90AE832B}" name="ID" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{2A363B76-0FF0-4E35-8B0D-D3DFE428B184}" name="Epic" dataDxfId="25"/>
-    <tableColumn id="12" xr3:uid="{58EF9BAF-7539-44AE-B4EA-ED1E3E2C43A2}" name="User Story /Task" dataDxfId="24"/>
-    <tableColumn id="11" xr3:uid="{5812FBDE-2CCF-4471-BA12-4B4E981FB0F8}" name="Estimated time" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{9D350C75-9112-414E-B33C-95BA4ED272B4}" name="COS (Criteria of Satisfaction)" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{79971A75-750E-427F-A5B6-5A61FA1008BB}" name="Story points" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{F15B638A-5756-448D-BFF1-F83357264427}" name="Time in Hours" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{5419A239-65A0-4210-A072-8D48A4908096}" name="Status" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{D532321B-43A9-4C7B-9711-0E9DB0F36080}" name="Sprint Start" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{F9445A15-FEA9-4142-9284-D23FEC81E85A}" name="Sprint End" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{98E29721-27A3-49D9-AB54-E3E822D61773}" name="User" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{A6CFA86C-B64A-4D7B-988B-D7EA90AE832B}" name="ID" dataDxfId="49"/>
+    <tableColumn id="6" xr3:uid="{2A363B76-0FF0-4E35-8B0D-D3DFE428B184}" name="Epic" dataDxfId="48"/>
+    <tableColumn id="12" xr3:uid="{58EF9BAF-7539-44AE-B4EA-ED1E3E2C43A2}" name="User Story /Task" dataDxfId="47"/>
+    <tableColumn id="11" xr3:uid="{5812FBDE-2CCF-4471-BA12-4B4E981FB0F8}" name="Estimated time" dataDxfId="46"/>
+    <tableColumn id="8" xr3:uid="{9D350C75-9112-414E-B33C-95BA4ED272B4}" name="COS (Criteria of Satisfaction)" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{79971A75-750E-427F-A5B6-5A61FA1008BB}" name="Story points" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{F15B638A-5756-448D-BFF1-F83357264427}" name="Time in Hours" dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{5419A239-65A0-4210-A072-8D48A4908096}" name="Status" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{1868505A-CACE-44B2-A7EA-9FE64E58BA8A}" name="Tabelle3811141720" displayName="Tabelle3811141720" ref="A18:C19" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{1868505A-CACE-44B2-A7EA-9FE64E58BA8A}" name="Tabelle3811141720" displayName="Tabelle3811141720" ref="A18:C19" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
   <autoFilter ref="A18:C19" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{3A312704-DAF9-41C4-9ED9-5DD84799E905}" name="Estimated time" dataDxfId="16">
+    <tableColumn id="1" xr3:uid="{3A312704-DAF9-41C4-9ED9-5DD84799E905}" name="Estimated time" dataDxfId="39">
       <calculatedColumnFormula>SUM(Tabelle2710131619[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{72BDDA5F-E86A-4485-B7A7-C4A72345EFC4}" name="Actual time" dataDxfId="15">
+    <tableColumn id="2" xr3:uid="{72BDDA5F-E86A-4485-B7A7-C4A72345EFC4}" name="Actual time" dataDxfId="38">
       <calculatedColumnFormula>SUM(Tabelle2710131619[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{223E53E9-D637-4AC0-9A6C-5591B23BB953}" name="Delta" dataDxfId="14">
+    <tableColumn id="3" xr3:uid="{223E53E9-D637-4AC0-9A6C-5591B23BB953}" name="Delta" dataDxfId="37">
       <calculatedColumnFormula>Tabelle3811141720[[#This Row],[Estimated time]]-Tabelle3811141720[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3644,13 +4072,13 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{F7C4B985-A6EE-4B5E-BF93-A6081AE08433}" name="Tabelle4912151821" displayName="Tabelle4912151821" ref="E18:F19" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{F7C4B985-A6EE-4B5E-BF93-A6081AE08433}" name="Tabelle4912151821" displayName="Tabelle4912151821" ref="E18:F19" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
   <autoFilter ref="E18:F19" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{DC2B1F8F-41E8-42FD-87FA-7DF04FEE86E6}" name="Total Storypoints " dataDxfId="11">
+    <tableColumn id="1" xr3:uid="{DC2B1F8F-41E8-42FD-87FA-7DF04FEE86E6}" name="Total Storypoints " dataDxfId="34">
       <calculatedColumnFormula>SUM(Tabelle2710131619[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{913BEBDF-DC3B-496C-982F-AE7F617915B6}" name="Effort/Hour" dataDxfId="10">
+    <tableColumn id="2" xr3:uid="{913BEBDF-DC3B-496C-982F-AE7F617915B6}" name="Effort/Hour" dataDxfId="33">
       <calculatedColumnFormula>Tabelle4912151821[[#This Row],[Total Storypoints ]]/Tabelle3811141720[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3659,55 +4087,108 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}" name="Tabelle2" displayName="Tabelle2" ref="A1:J9" insertRowShift="1" totalsRowShown="0" headerRowDxfId="140" dataDxfId="139">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}" name="Tabelle2" displayName="Tabelle2" ref="A1:J9" insertRowShift="1" totalsRowShown="0" headerRowDxfId="163" dataDxfId="162">
   <autoFilter ref="A1:J9" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{0351E8C1-0BB8-4C19-A406-233CC12328E5}" name="Sprint Start" dataDxfId="138"/>
-    <tableColumn id="2" xr3:uid="{51BD2FE0-507A-4398-BD96-E186E78BB2C7}" name="Sprint End" dataDxfId="137"/>
-    <tableColumn id="3" xr3:uid="{A3B7E86B-E01A-4D78-82AD-BA81F6AC7ADF}" name="User" dataDxfId="136"/>
-    <tableColumn id="5" xr3:uid="{CE780601-F45C-4063-B216-98ACE5588903}" name="ID" dataDxfId="135"/>
-    <tableColumn id="6" xr3:uid="{A14D049D-AC5C-49A5-A7CC-A4D5ED8A8330}" name="Epic" dataDxfId="134"/>
-    <tableColumn id="12" xr3:uid="{770F10A6-830A-41AC-B069-6267CAE00BDF}" name="User Story /Task" dataDxfId="133"/>
-    <tableColumn id="11" xr3:uid="{0D9AB552-F7B4-4231-A35B-245B57383919}" name="Estimated time" dataDxfId="132"/>
-    <tableColumn id="8" xr3:uid="{3E2E3644-9002-4AB9-B3EC-96FFF84D8900}" name="COS (Criteria of Satisfaction)" dataDxfId="131"/>
-    <tableColumn id="9" xr3:uid="{14C8E3A9-BC37-48D9-A399-32A48A46993A}" name="Story points" dataDxfId="130"/>
-    <tableColumn id="10" xr3:uid="{151786D9-5F15-42D7-932B-664A024F4131}" name="Time in Hours" dataDxfId="129"/>
+    <tableColumn id="1" xr3:uid="{0351E8C1-0BB8-4C19-A406-233CC12328E5}" name="Sprint Start" dataDxfId="161"/>
+    <tableColumn id="2" xr3:uid="{51BD2FE0-507A-4398-BD96-E186E78BB2C7}" name="Sprint End" dataDxfId="160"/>
+    <tableColumn id="3" xr3:uid="{A3B7E86B-E01A-4D78-82AD-BA81F6AC7ADF}" name="User" dataDxfId="159"/>
+    <tableColumn id="5" xr3:uid="{CE780601-F45C-4063-B216-98ACE5588903}" name="ID" dataDxfId="158"/>
+    <tableColumn id="6" xr3:uid="{A14D049D-AC5C-49A5-A7CC-A4D5ED8A8330}" name="Epic" dataDxfId="157"/>
+    <tableColumn id="12" xr3:uid="{770F10A6-830A-41AC-B069-6267CAE00BDF}" name="User Story /Task" dataDxfId="156"/>
+    <tableColumn id="11" xr3:uid="{0D9AB552-F7B4-4231-A35B-245B57383919}" name="Estimated time" dataDxfId="155"/>
+    <tableColumn id="8" xr3:uid="{3E2E3644-9002-4AB9-B3EC-96FFF84D8900}" name="COS (Criteria of Satisfaction)" dataDxfId="154"/>
+    <tableColumn id="9" xr3:uid="{14C8E3A9-BC37-48D9-A399-32A48A46993A}" name="Story points" dataDxfId="153"/>
+    <tableColumn id="10" xr3:uid="{151786D9-5F15-42D7-932B-664A024F4131}" name="Time in Hours" dataDxfId="152"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:H28" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:H28" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H28">
-    <sortCondition ref="C9:C28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{98C1BB39-A2E9-0E45-AC8B-15B77F0EF61D}" name="Tabelle271013161922" displayName="Tabelle271013161922" ref="A1:K14" insertRowShift="1" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+  <autoFilter ref="A1:K14" xr:uid="{D3B682F1-6F73-4656-A177-C3533051D55F}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{04332918-0CB8-8C4A-8A46-BF72B0B731C8}" name="Sprint Start" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{E398574F-DF91-7542-B4C1-883C0529B26F}" name="Sprint End" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{DFEC897C-9674-AB47-8D3F-43A5742FD343}" name="User" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{FF870139-F7B0-3146-A447-320C7996DFEF}" name="ID" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{94CC98F1-00B8-2D4B-BE4A-A22464CF5704}" name="Epic" dataDxfId="16"/>
+    <tableColumn id="12" xr3:uid="{DAB3489B-9371-D944-82BB-D87BBB34B3E7}" name="User Story /Task" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{851C6BD5-3FF8-E74A-9C96-F111B229BC11}" name="Estimated time" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{DD283687-4ECB-3B43-B95B-DF6761DE6889}" name="COS (Criteria of Satisfaction)" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{7AE176F9-D6D9-9446-8443-894F6415A70E}" name="Story points" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{D468B082-F4E7-D24B-8BFE-41EA21742D10}" name="Time in Hours" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{2CC0CF29-93A0-6645-9328-8FD2C834881C}" name="Status" dataDxfId="10"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{D649AC79-C1A8-4F47-A4EA-9B33E4654536}" name="Tabelle381114172023" displayName="Tabelle381114172023" ref="A18:C19" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A18:C19" xr:uid="{64CE46E8-9109-463E-9929-B04F65880A6E}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{D88E3592-B2C1-DC43-903C-3A61A8C3E650}" name="Estimated time" dataDxfId="7">
+      <calculatedColumnFormula>SUM(Tabelle271013161922[Estimated time])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{A85C0AC7-7E35-D140-A9D1-DC5F2E46EF5E}" name="Actual time" dataDxfId="6">
+      <calculatedColumnFormula>SUM(Tabelle271013161922[Time in Hours])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{6501830E-BDFF-EF4D-847F-CD50B63E2201}" name="Delta" dataDxfId="5">
+      <calculatedColumnFormula>Tabelle381114172023[[#This Row],[Estimated time]]-Tabelle381114172023[[#This Row],[Actual time]]</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{6579DE2E-4664-1348-88BB-D035B9CA9A3F}" name="Tabelle491215182124" displayName="Tabelle491215182124" ref="E18:F19" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="E18:F19" xr:uid="{76B5E61D-16B7-49D5-8782-AA9FAFD44E36}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{F3D80279-C6C5-CD48-8B24-87E47D7C3A02}" name="Total Storypoints " dataDxfId="2">
+      <calculatedColumnFormula>SUM(Tabelle271013161922[Story points])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{E1EC842A-1920-FB40-A838-FD8D30319D54}" name="Effort/Hour" dataDxfId="1">
+      <calculatedColumnFormula>Tabelle491215182124[[#This Row],[Total Storypoints ]]/Tabelle381114172023[[#This Row],[Actual time]]</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}" name="Tabelle5" displayName="Tabelle5" ref="A1:H26" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
+  <autoFilter ref="A1:H26" xr:uid="{9C26F5F1-3CA5-4498-8D9F-A792FBE4E032}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H26">
+    <sortCondition ref="C9:C26"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Story" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{57E495A5-904B-1740-A858-653ACCE96658}" name="Acceptance Criteria" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{BC6E6F54-B9E2-4D1B-BB78-E6F30265832D}" name="Story ID" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{5BD6C059-22C9-4C4A-90A3-74736AC1F83D}" name="Title" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{F3A7207B-9229-4096-9A5B-C4FB1EDD5455}" name="Priority" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{E38B598E-699A-460C-AB30-1E65BB7404BF}" name="Story" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{57E495A5-904B-1740-A858-653ACCE96658}" name="Acceptance Criteria" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{5087B805-D2DF-49C7-9936-ECACDF516D64}" name="Status" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{05DFD049-144E-4717-9B70-2B02AA12CC20}" name="Story Points" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{98F7F45D-928E-4B6F-868A-18B3899C12B6}" name="Sprint" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}" name="Tabelle3" displayName="Tabelle3" ref="A15:C16" totalsRowShown="0" headerRowDxfId="128" dataDxfId="127">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}" name="Tabelle3" displayName="Tabelle3" ref="A15:C16" totalsRowShown="0" headerRowDxfId="151" dataDxfId="150">
   <autoFilter ref="A15:C16" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CD2D4D96-DD34-4EA3-92D7-B02BB9DE5647}" name="Estimated time" dataDxfId="126">
+    <tableColumn id="1" xr3:uid="{CD2D4D96-DD34-4EA3-92D7-B02BB9DE5647}" name="Estimated time" dataDxfId="149">
       <calculatedColumnFormula>SUM(Tabelle2[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0F14E190-6E0A-4AB8-8ADE-83875E98D4B5}" name="Actual time" dataDxfId="125">
+    <tableColumn id="2" xr3:uid="{0F14E190-6E0A-4AB8-8ADE-83875E98D4B5}" name="Actual time" dataDxfId="148">
       <calculatedColumnFormula>SUM(Tabelle2[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{5DE18543-F4D3-4732-9F2D-5B7F140CB974}" name="Delta" dataDxfId="124">
+    <tableColumn id="3" xr3:uid="{5DE18543-F4D3-4732-9F2D-5B7F140CB974}" name="Delta" dataDxfId="147">
       <calculatedColumnFormula>Tabelle3[[#This Row],[Estimated time]]-Tabelle3[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3716,13 +4197,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}" name="Tabelle4" displayName="Tabelle4" ref="E15:F16" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}" name="Tabelle4" displayName="Tabelle4" ref="E15:F16" totalsRowShown="0" headerRowDxfId="146" dataDxfId="145">
   <autoFilter ref="E15:F16" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{2E187AEA-682F-4749-9FC8-ED3BA3DE1DA2}" name="Total Storypoints " dataDxfId="121">
+    <tableColumn id="1" xr3:uid="{2E187AEA-682F-4749-9FC8-ED3BA3DE1DA2}" name="Total Storypoints " dataDxfId="144">
       <calculatedColumnFormula>SUM(Tabelle2[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3C6DC8F5-724A-43AC-9128-7661A96380C1}" name="Efford/Hour" dataDxfId="120">
+    <tableColumn id="2" xr3:uid="{3C6DC8F5-724A-43AC-9128-7661A96380C1}" name="Efford/Hour" dataDxfId="143">
       <calculatedColumnFormula>Tabelle4[[#This Row],[Total Storypoints ]]/Tabelle3[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3731,36 +4212,36 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A211D33B-248F-4E66-AF7C-9632EAA38DAC}" name="Tabelle27" displayName="Tabelle27" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="119" dataDxfId="118">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A211D33B-248F-4E66-AF7C-9632EAA38DAC}" name="Tabelle27" displayName="Tabelle27" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="142" dataDxfId="141">
   <autoFilter ref="A1:K12" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{9C36A560-9153-4D8E-BA50-0044E74E1896}" name="Sprint Start" dataDxfId="117"/>
-    <tableColumn id="2" xr3:uid="{4FAB3106-8621-41F1-B866-EA5558F083D8}" name="Sprint End" dataDxfId="116"/>
-    <tableColumn id="3" xr3:uid="{2D2022CC-B165-4671-9773-4C7DCE737FC7}" name="User" dataDxfId="115"/>
-    <tableColumn id="5" xr3:uid="{6D49D607-DA69-4FF5-AC26-260E9F796217}" name="ID" dataDxfId="114"/>
-    <tableColumn id="6" xr3:uid="{95077F2F-115F-484E-A38C-A34A2BCBCB78}" name="Epic" dataDxfId="113"/>
-    <tableColumn id="12" xr3:uid="{2EAFDE91-2C58-4973-A684-28E2E964F629}" name="User Story /Task" dataDxfId="112"/>
-    <tableColumn id="11" xr3:uid="{D17AAC02-918A-4F08-B037-3622F37B62F0}" name="Estimated time" dataDxfId="111"/>
-    <tableColumn id="8" xr3:uid="{4D053EE2-698A-4191-ABEB-8F0701DA4D4E}" name="COS (Criteria of Satisfaction)" dataDxfId="110"/>
-    <tableColumn id="9" xr3:uid="{73BF0134-792D-4614-95FB-754C4A317665}" name="Story points" dataDxfId="109"/>
-    <tableColumn id="10" xr3:uid="{2620A9CC-A288-4874-BF27-2BBE69671B14}" name="Time in Hours" dataDxfId="108"/>
-    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="107"/>
+    <tableColumn id="1" xr3:uid="{9C36A560-9153-4D8E-BA50-0044E74E1896}" name="Sprint Start" dataDxfId="140"/>
+    <tableColumn id="2" xr3:uid="{4FAB3106-8621-41F1-B866-EA5558F083D8}" name="Sprint End" dataDxfId="139"/>
+    <tableColumn id="3" xr3:uid="{2D2022CC-B165-4671-9773-4C7DCE737FC7}" name="User" dataDxfId="138"/>
+    <tableColumn id="5" xr3:uid="{6D49D607-DA69-4FF5-AC26-260E9F796217}" name="ID" dataDxfId="137"/>
+    <tableColumn id="6" xr3:uid="{95077F2F-115F-484E-A38C-A34A2BCBCB78}" name="Epic" dataDxfId="136"/>
+    <tableColumn id="12" xr3:uid="{2EAFDE91-2C58-4973-A684-28E2E964F629}" name="User Story /Task" dataDxfId="135"/>
+    <tableColumn id="11" xr3:uid="{D17AAC02-918A-4F08-B037-3622F37B62F0}" name="Estimated time" dataDxfId="134"/>
+    <tableColumn id="8" xr3:uid="{4D053EE2-698A-4191-ABEB-8F0701DA4D4E}" name="COS (Criteria of Satisfaction)" dataDxfId="133"/>
+    <tableColumn id="9" xr3:uid="{73BF0134-792D-4614-95FB-754C4A317665}" name="Story points" dataDxfId="132"/>
+    <tableColumn id="10" xr3:uid="{2620A9CC-A288-4874-BF27-2BBE69671B14}" name="Time in Hours" dataDxfId="131"/>
+    <tableColumn id="4" xr3:uid="{EEDB864F-4BEC-E84C-8BC3-11680213E110}" name="Status" dataDxfId="130"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7635EDC6-25C8-4AEE-8477-EE4C813DEB0C}" name="Tabelle38" displayName="Tabelle38" ref="A16:C17" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
   <autoFilter ref="A16:C17" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="104">
+    <tableColumn id="1" xr3:uid="{608DD481-0706-4498-AF85-EB4AD6D17A03}" name="Estimated time" dataDxfId="127">
       <calculatedColumnFormula>SUM(Tabelle27[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="103">
+    <tableColumn id="2" xr3:uid="{727CC20C-885F-49B6-A31D-85E6D39BFD35}" name="Actual time" dataDxfId="126">
       <calculatedColumnFormula>SUM(Tabelle27[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="102">
+    <tableColumn id="3" xr3:uid="{DB626F11-D2AA-4B08-BE29-BA7526E2BE88}" name="Delta" dataDxfId="125">
       <calculatedColumnFormula>Tabelle38[[#This Row],[Estimated time]]-Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3769,13 +4250,13 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="101" dataDxfId="100">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{96D8EE75-69AD-457A-99FC-A0696238BDE6}" name="Tabelle49" displayName="Tabelle49" ref="E16:F17" totalsRowShown="0" headerRowDxfId="124" dataDxfId="123">
   <autoFilter ref="E16:F17" xr:uid="{F5FF718A-3E4E-40DD-BD72-E3ACE1B58735}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="99">
+    <tableColumn id="1" xr3:uid="{1F43F730-E2EB-4487-8A5C-6B0E3F4CC598}" name="Total Storypoints " dataDxfId="122">
       <calculatedColumnFormula>SUM(Tabelle27[Story points])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="98">
+    <tableColumn id="2" xr3:uid="{95E1605C-A4E2-4173-B0AE-218EC74BDEA1}" name="Effort/Hour" dataDxfId="121">
       <calculatedColumnFormula>Tabelle49[[#This Row],[Total Storypoints ]]/Tabelle38[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3784,36 +4265,36 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6303AB7F-CDC2-408B-A450-96D692A68B43}" name="Tabelle2710" displayName="Tabelle2710" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="97" dataDxfId="96">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{6303AB7F-CDC2-408B-A450-96D692A68B43}" name="Tabelle2710" displayName="Tabelle2710" ref="A1:K12" insertRowShift="1" totalsRowShown="0" headerRowDxfId="120" dataDxfId="119">
   <autoFilter ref="A1:K12" xr:uid="{739F99A6-83FF-4FC0-82EE-54F2B8B8AE5A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{949CA967-02A0-4249-BB07-B02F4C4F69AE}" name="Sprint Start" dataDxfId="95"/>
-    <tableColumn id="2" xr3:uid="{A70AE104-D3DD-4C6E-8E50-E151404B19BD}" name="Sprint End" dataDxfId="94"/>
-    <tableColumn id="3" xr3:uid="{9168C6BE-6970-4420-9D5F-DBCF1E8E2BAE}" name="User" dataDxfId="93"/>
-    <tableColumn id="5" xr3:uid="{A7C4968E-9480-42FF-949B-9E41609C26A2}" name="ID" dataDxfId="92"/>
-    <tableColumn id="6" xr3:uid="{8564B7DD-8DB4-4E2B-BDDB-9791D9AAA0EA}" name="Epic" dataDxfId="91"/>
-    <tableColumn id="12" xr3:uid="{56FA47CB-3810-4B7F-A047-8358D5C73F6C}" name="User Story /Task" dataDxfId="90"/>
-    <tableColumn id="11" xr3:uid="{988CB3AF-F268-445B-887C-5163D9AE41DF}" name="Estimated time" dataDxfId="89"/>
-    <tableColumn id="8" xr3:uid="{14BDCFB4-F75D-4798-AFF3-3F8B177B78D6}" name="COS (Criteria of Satisfaction)" dataDxfId="88"/>
-    <tableColumn id="9" xr3:uid="{97C18CBF-2D3F-4A8A-B36D-6328E17F31C4}" name="Story points" dataDxfId="87"/>
-    <tableColumn id="10" xr3:uid="{D3E339CF-38BF-4AC1-8C80-41ECD30B6907}" name="Time in Hours" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{3BCBC0DA-7C9B-4D2B-9269-A319CBD925C5}" name="Status" dataDxfId="85"/>
+    <tableColumn id="1" xr3:uid="{949CA967-02A0-4249-BB07-B02F4C4F69AE}" name="Sprint Start" dataDxfId="118"/>
+    <tableColumn id="2" xr3:uid="{A70AE104-D3DD-4C6E-8E50-E151404B19BD}" name="Sprint End" dataDxfId="117"/>
+    <tableColumn id="3" xr3:uid="{9168C6BE-6970-4420-9D5F-DBCF1E8E2BAE}" name="User" dataDxfId="116"/>
+    <tableColumn id="5" xr3:uid="{A7C4968E-9480-42FF-949B-9E41609C26A2}" name="ID" dataDxfId="115"/>
+    <tableColumn id="6" xr3:uid="{8564B7DD-8DB4-4E2B-BDDB-9791D9AAA0EA}" name="Epic" dataDxfId="114"/>
+    <tableColumn id="12" xr3:uid="{56FA47CB-3810-4B7F-A047-8358D5C73F6C}" name="User Story /Task" dataDxfId="113"/>
+    <tableColumn id="11" xr3:uid="{988CB3AF-F268-445B-887C-5163D9AE41DF}" name="Estimated time" dataDxfId="112"/>
+    <tableColumn id="8" xr3:uid="{14BDCFB4-F75D-4798-AFF3-3F8B177B78D6}" name="COS (Criteria of Satisfaction)" dataDxfId="111"/>
+    <tableColumn id="9" xr3:uid="{97C18CBF-2D3F-4A8A-B36D-6328E17F31C4}" name="Story points" dataDxfId="110"/>
+    <tableColumn id="10" xr3:uid="{D3E339CF-38BF-4AC1-8C80-41ECD30B6907}" name="Time in Hours" dataDxfId="109"/>
+    <tableColumn id="4" xr3:uid="{3BCBC0DA-7C9B-4D2B-9269-A319CBD925C5}" name="Status" dataDxfId="108"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C1E761E2-D340-4C7F-A19A-AE84A76F5971}" name="Tabelle3811" displayName="Tabelle3811" ref="A16:C17" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C1E761E2-D340-4C7F-A19A-AE84A76F5971}" name="Tabelle3811" displayName="Tabelle3811" ref="A16:C17" totalsRowShown="0" headerRowDxfId="107" dataDxfId="106">
   <autoFilter ref="A16:C17" xr:uid="{F79F1E8C-9DFD-4482-95C6-9C23936D055B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{F045D4AD-2D00-44A7-8EA7-B5C34869B26F}" name="Estimated time" dataDxfId="82">
+    <tableColumn id="1" xr3:uid="{F045D4AD-2D00-44A7-8EA7-B5C34869B26F}" name="Estimated time" dataDxfId="105">
       <calculatedColumnFormula>SUM(Tabelle2710[Estimated time])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DFDFE0A8-6207-4F3B-9D05-4D3AF083E31B}" name="Actual time" dataDxfId="81">
+    <tableColumn id="2" xr3:uid="{DFDFE0A8-6207-4F3B-9D05-4D3AF083E31B}" name="Actual time" dataDxfId="104">
       <calculatedColumnFormula>SUM(Tabelle2710[Time in Hours])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{2529739A-9C5E-4AE4-80A6-DFC080EFE2D8}" name="Delta" dataDxfId="80">
+    <tableColumn id="3" xr3:uid="{2529739A-9C5E-4AE4-80A6-DFC080EFE2D8}" name="Delta" dataDxfId="103">
       <calculatedColumnFormula>Tabelle3811[[#This Row],[Estimated time]]-Tabelle3811[[#This Row],[Actual time]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4163,30 +4644,30 @@
         <v>0</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C2" s="7" cm="1">
         <f t="array" ref="C2">Tabelle3[Estimated time]</f>
@@ -4201,23 +4682,24 @@
         <v>0</v>
       </c>
       <c r="F2" s="7">
-        <f>Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]]</f>
-        <v>0</v>
+        <f>Tabelle1[[#This Row],[Estimated Hours]]/Tabelle1[[#This Row],[Actual Hours]]</f>
+        <v>0.76470588235294112</v>
       </c>
       <c r="G2" s="7">
-        <v>146</v>
+        <f>C12</f>
+        <v>116</v>
       </c>
       <c r="H2" s="7">
         <f>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</f>
-        <v>146</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C3" s="7" cm="1">
         <f t="array" ref="C3">Tabelle38[Estimated time]</f>
@@ -4232,23 +4714,24 @@
         <v>24</v>
       </c>
       <c r="F3" s="7">
-        <f>Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]]</f>
-        <v>0.70588235294117652</v>
+        <f>Tabelle1[[#This Row],[Estimated Hours]]/Tabelle1[[#This Row],[Actual Hours]]</f>
+        <v>1.2352941176470589</v>
       </c>
       <c r="G3" s="7">
-        <v>146</v>
+        <f>H2</f>
+        <v>116</v>
       </c>
       <c r="H3" s="7">
         <f>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</f>
-        <v>122</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="7" cm="1">
         <f t="array" ref="C4">Tabelle3811[Estimated time]</f>
@@ -4263,24 +4746,24 @@
         <v>10</v>
       </c>
       <c r="F4" s="7">
-        <f>Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]]</f>
-        <v>1</v>
+        <f>Tabelle1[[#This Row],[Estimated Hours]]/Tabelle1[[#This Row],[Actual Hours]]</f>
+        <v>0.9</v>
       </c>
       <c r="G4" s="7">
         <f>H3</f>
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="H4" s="7">
         <f>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</f>
-        <v>112</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C5" s="7" cm="1">
         <f t="array" ref="C5">Tabelle381114[Estimated time]</f>
@@ -4295,24 +4778,24 @@
         <v>39</v>
       </c>
       <c r="F5" s="7">
-        <f>Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]]</f>
-        <v>1.625</v>
+        <f>Tabelle1[[#This Row],[Estimated Hours]]/Tabelle1[[#This Row],[Actual Hours]]</f>
+        <v>0.91666666666666663</v>
       </c>
       <c r="G5" s="7">
         <f>H4</f>
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="H5" s="7">
         <f>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</f>
-        <v>73</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C6" s="7" cm="1">
         <f t="array" ref="C6">Tabelle38111417[Estimated time]</f>
@@ -4327,62 +4810,101 @@
         <v>21</v>
       </c>
       <c r="F6" s="7">
-        <f>Tabelle1[[#This Row],[Accomplished Story Points]]/Tabelle1[[#This Row],[Actual Hours]]</f>
-        <v>1.3125</v>
+        <f>Tabelle1[[#This Row],[Estimated Hours]]/Tabelle1[[#This Row],[Actual Hours]]</f>
+        <v>1.0625</v>
       </c>
       <c r="G6" s="7">
         <f>H5</f>
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="H6" s="7">
-        <f>C13</f>
-        <v>52</v>
+        <f>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</f>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
+        <v>69</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C7" s="7" cm="1">
+        <f t="array" ref="C7">Tabelle3811141720[Estimated time]</f>
+        <v>11</v>
+      </c>
+      <c r="D7" s="7" cm="1">
+        <f t="array" ref="D7">Tabelle3811141720[Actual time]</f>
+        <v>14</v>
+      </c>
+      <c r="E7" s="7" cm="1">
+        <f t="array" ref="E7">Tabelle4912151821[[Total Storypoints ]]</f>
+        <v>15</v>
+      </c>
+      <c r="F7" s="7">
+        <f>Tabelle1[[#This Row],[Estimated Hours]]/Tabelle1[[#This Row],[Actual Hours]]</f>
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="G7" s="7">
+        <f>H6</f>
+        <v>22</v>
+      </c>
+      <c r="H7" s="7">
+        <f>Tabelle1[[#This Row],[Total Storypoints]]-Tabelle1[[#This Row],[Accomplished Story Points]]</f>
+        <v>7</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="22" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
+        <v>70</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C8" s="7" cm="1">
+        <f t="array" ref="C8">Tabelle381114172023[Estimated time]</f>
+        <v>16</v>
+      </c>
+      <c r="D8" s="7" cm="1">
+        <f t="array" ref="D8">Tabelle381114172023[Actual time]</f>
+        <v>14</v>
+      </c>
+      <c r="E8" s="7">
+        <v>15</v>
+      </c>
+      <c r="F8" s="7">
+        <f>Tabelle1[[#This Row],[Estimated Hours]]/Tabelle1[[#This Row],[Actual Hours]]</f>
+        <v>1.1428571428571428</v>
+      </c>
+      <c r="G8" s="7">
+        <f>G7-H7</f>
+        <v>15</v>
+      </c>
+      <c r="H8" s="7">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C12" s="5">
-        <v>146</v>
+        <f>Storys!G26</f>
+        <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C13" s="5">
-        <f>C12-SUM(Tabelle1[Accomplished Story Points])</f>
-        <v>52</v>
+        <f>H8</f>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C14" s="5">
         <f>COUNTIF(Tabelle1[Sprint],"*Sprint*")</f>
@@ -4391,33 +4913,32 @@
     </row>
     <row r="15" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C15" s="5">
         <f>AVERAGE(Tabelle1[Velocity])</f>
-        <v>0.92867647058823533</v>
+        <v>0.97253401360544223</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C16" s="14">
-        <f>(SUM(Tabelle1[Accomplished Story Points],)/G2)</f>
-        <v>0.64383561643835618</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="24" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C17" s="18">
         <f>C13/C15</f>
-        <v>55.993665874901026</v>
+        <v>0</v>
       </c>
       <c r="D17">
         <f>C17/4</f>
-        <v>13.998416468725257</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4451,34 +4972,34 @@
   <sheetData>
     <row r="1" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="19" x14ac:dyDescent="0.25">
@@ -4489,23 +5010,23 @@
         <v>45932</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D2" s="10"/>
       <c r="E2" s="8" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="G2" s="8">
         <v>2</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J2" s="8">
         <v>2</v>
@@ -4515,18 +5036,18 @@
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
       <c r="F3" s="8" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="G3" s="8">
         <v>4</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="I3" s="8"/>
       <c r="J3" s="8">
@@ -4537,12 +5058,12 @@
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
       <c r="F4" s="8" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G4" s="8">
         <v>1</v>
@@ -4569,22 +5090,22 @@
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>5</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G6" s="8">
         <v>2</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="I6" s="8">
         <v>0</v>
@@ -4597,22 +5118,22 @@
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>5</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G7" s="8">
         <v>3</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="I7" s="8"/>
       <c r="J7" s="8">
@@ -4623,16 +5144,16 @@
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>5</v>
       </c>
       <c r="E8" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>103</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>108</v>
       </c>
       <c r="G8" s="8">
         <v>1</v>
@@ -4717,20 +5238,20 @@
     </row>
     <row r="15" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
@@ -4797,34 +5318,34 @@
   <sheetData>
     <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>87</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>3</v>
@@ -4838,22 +5359,22 @@
         <v>45953</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>5</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G2" s="8">
         <v>2</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="I2" s="10">
         <v>5</v>
@@ -4862,36 +5383,36 @@
         <v>2</v>
       </c>
       <c r="K2" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G3" s="8">
         <v>1</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="I3" s="8"/>
       <c r="J3" s="8">
         <v>1</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -4911,22 +5432,22 @@
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D5" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="8" t="s">
-        <v>11</v>
-      </c>
       <c r="F5" s="8" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="G5" s="8">
         <v>5</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="I5" s="8">
         <v>8</v>
@@ -4940,29 +5461,29 @@
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D6" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>13</v>
-      </c>
       <c r="F6" s="8" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="G6" s="8">
         <v>4</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="I6" s="8">
         <v>5</v>
       </c>
       <c r="J6" s="8"/>
       <c r="K6" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -4995,22 +5516,22 @@
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="G9" s="8">
         <v>10</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="I9" s="8">
         <v>3</v>
@@ -5019,29 +5540,29 @@
         <v>15</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="G10" s="8">
         <v>15</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I10" s="8">
         <v>3</v>
@@ -5050,34 +5571,34 @@
         <v>10</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="G11" s="8">
         <v>5</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
       <c r="K11" s="19" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -5131,20 +5652,20 @@
     </row>
     <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
@@ -5212,34 +5733,34 @@
   <sheetData>
     <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>87</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>3</v>
@@ -5266,22 +5787,22 @@
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G3" s="8">
         <v>5</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="I3" s="8">
         <v>3</v>
@@ -5290,29 +5811,29 @@
         <v>6</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G4" s="8">
         <v>4</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="I4" s="8">
         <v>7</v>
@@ -5321,7 +5842,7 @@
         <v>4</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -5466,20 +5987,20 @@
     </row>
     <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
@@ -5547,34 +6068,34 @@
   <sheetData>
     <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>87</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>3</v>
@@ -5601,22 +6122,22 @@
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G3" s="8">
         <v>10</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="I3" s="8">
         <v>8</v>
@@ -5625,23 +6146,23 @@
         <v>10</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="F4" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="G4" s="8">
         <v>1</v>
@@ -5654,23 +6175,23 @@
         <v>1</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="15" t="s">
-        <v>11</v>
-      </c>
       <c r="F5" s="8" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="G5" s="8">
         <v>1</v>
@@ -5683,29 +6204,29 @@
         <v>1</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G6" s="8">
         <v>1</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="I6" s="8">
         <v>6</v>
@@ -5714,7 +6235,7 @@
         <v>2</v>
       </c>
       <c r="K6" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -5734,22 +6255,22 @@
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G8" s="8">
         <v>4</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="I8" s="8">
         <v>9</v>
@@ -5758,29 +6279,29 @@
         <v>6</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="G9" s="8">
         <v>5</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="I9" s="8">
         <v>4</v>
@@ -5789,7 +6310,7 @@
         <v>4</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -5856,20 +6377,20 @@
     </row>
     <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
@@ -5936,34 +6457,34 @@
   <sheetData>
     <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>87</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>3</v>
@@ -5990,22 +6511,22 @@
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="G3" s="8">
         <v>8</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="I3" s="8">
         <v>8</v>
@@ -6014,7 +6535,7 @@
         <v>8</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -6060,22 +6581,22 @@
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G7" s="8">
         <v>6</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="I7" s="8">
         <v>5</v>
@@ -6084,21 +6605,21 @@
         <v>5</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
@@ -6108,22 +6629,22 @@
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="G9" s="8">
         <v>3</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="I9" s="8">
         <v>8</v>
@@ -6132,7 +6653,7 @@
         <v>3</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -6199,20 +6720,20 @@
     </row>
     <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
@@ -6280,34 +6801,34 @@
   <sheetData>
     <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>87</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>3</v>
@@ -6334,7 +6855,7 @@
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
@@ -6350,19 +6871,19 @@
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
       <c r="D4" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="G4" s="8">
         <v>4</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="I4" s="8">
         <v>5</v>
@@ -6381,7 +6902,7 @@
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
       <c r="H5" s="8" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
@@ -6396,7 +6917,7 @@
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
@@ -6419,22 +6940,22 @@
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="G8" s="8">
         <v>3</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
@@ -6449,7 +6970,7 @@
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="I9" s="8">
         <v>5</v>
@@ -6476,22 +6997,22 @@
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="G11" s="8">
         <v>4</v>
       </c>
       <c r="H11" s="24" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="I11" s="8">
         <v>5</v>
@@ -6500,7 +7021,7 @@
         <v>3</v>
       </c>
       <c r="K11" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -6580,20 +7101,20 @@
     </row>
     <row r="18" spans="1:10" ht="19" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
@@ -6639,11 +7160,408 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34DF71FA-E7FA-0C46-9251-968C0E7F6625}">
+  <sheetPr>
+    <tabColor theme="0"/>
+  </sheetPr>
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="124.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="164.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A2" s="9">
+        <v>46007</v>
+      </c>
+      <c r="B2" s="9">
+        <v>46044</v>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="19"/>
+    </row>
+    <row r="3" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" s="8">
+        <v>5</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="I3" s="8">
+        <v>3</v>
+      </c>
+      <c r="J3" s="8">
+        <v>5</v>
+      </c>
+      <c r="K3" s="19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A4" s="8"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" s="8">
+        <v>2</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="I4" s="2">
+        <v>3</v>
+      </c>
+      <c r="J4" s="8">
+        <v>2</v>
+      </c>
+      <c r="K4" s="19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="8">
+        <v>5</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="I5" s="8">
+        <v>5</v>
+      </c>
+      <c r="J5" s="8">
+        <v>4</v>
+      </c>
+      <c r="K5" s="19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G6" s="8">
+        <v>4</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="I6" s="8">
+        <v>5</v>
+      </c>
+      <c r="J6" s="8">
+        <v>3</v>
+      </c>
+      <c r="K6" s="19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="19"/>
+    </row>
+    <row r="8" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="19"/>
+    </row>
+    <row r="9" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="19"/>
+    </row>
+    <row r="10" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="19"/>
+    </row>
+    <row r="11" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="19"/>
+    </row>
+    <row r="12" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="19"/>
+    </row>
+    <row r="13" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="19"/>
+    </row>
+    <row r="14" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="19"/>
+    </row>
+    <row r="15" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+    </row>
+    <row r="16" spans="1:11" ht="19" x14ac:dyDescent="0.25">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+    </row>
+    <row r="17" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+    </row>
+    <row r="18" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+    </row>
+    <row r="19" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="A19" s="12">
+        <f>SUM(Tabelle271013161922[Estimated time])</f>
+        <v>16</v>
+      </c>
+      <c r="B19" s="12">
+        <f>SUM(Tabelle271013161922[Time in Hours])</f>
+        <v>14</v>
+      </c>
+      <c r="C19" s="12">
+        <f>Tabelle381114172023[[#This Row],[Estimated time]]-Tabelle381114172023[[#This Row],[Actual time]]</f>
+        <v>2</v>
+      </c>
+      <c r="D19" s="8"/>
+      <c r="E19" s="12">
+        <f>SUM(Tabelle271013161922[Story points])</f>
+        <v>16</v>
+      </c>
+      <c r="F19" s="12">
+        <f>Tabelle491215182124[[#This Row],[Total Storypoints ]]/Tabelle381114172023[[#This Row],[Actual time]]</f>
+        <v>1.1428571428571428</v>
+      </c>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="3">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7C2A55-0520-4EB5-86E6-237FE14873A1}">
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
@@ -6667,16 +7585,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>4</v>
@@ -6698,7 +7616,7 @@
       </c>
       <c r="E2" s="20"/>
       <c r="F2" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G2" s="2">
         <v>5</v>
@@ -6710,20 +7628,20 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="E3" s="20"/>
       <c r="F3" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G3" s="2">
         <v>8</v>
@@ -6735,43 +7653,45 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C4" s="2">
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E4" s="20"/>
       <c r="F4" s="2" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
       <c r="G4" s="2">
         <v>3</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2">
+        <v>7</v>
+      </c>
       <c r="J4" s="17"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C5" s="2">
         <v>2</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="E5" s="20"/>
       <c r="F5" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G5" s="2">
         <v>8</v>
@@ -6783,20 +7703,20 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" s="2">
         <v>2</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6" s="20"/>
       <c r="F6" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G6" s="2">
         <v>5</v>
@@ -6808,20 +7728,20 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C7" s="2">
         <v>2</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="E7" s="20"/>
       <c r="F7" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G7" s="2">
         <v>8</v>
@@ -6833,20 +7753,20 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C8" s="2">
         <v>3</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E8" s="20"/>
       <c r="F8" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G8" s="2">
         <v>5</v>
@@ -6858,20 +7778,20 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C9" s="2">
         <v>3</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E9" s="20"/>
       <c r="F9" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G9" s="2">
         <v>5</v>
@@ -6883,22 +7803,22 @@
     </row>
     <row r="10" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C10" s="2">
         <v>3</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>163</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>168</v>
+        <v>158</v>
+      </c>
+      <c r="F10" s="25" t="s">
+        <v>115</v>
       </c>
       <c r="G10" s="2">
         <v>5</v>
@@ -6910,20 +7830,20 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C11" s="2">
         <v>4</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E11" s="20"/>
       <c r="F11" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G11" s="2">
         <v>3</v>
@@ -6935,20 +7855,20 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C12" s="2">
         <v>4</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E12" s="20"/>
       <c r="F12" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G12" s="2">
         <v>8</v>
@@ -6960,20 +7880,20 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13" s="2">
         <v>5</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E13" s="20"/>
       <c r="F13" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G13" s="2">
         <v>3</v>
@@ -6985,20 +7905,20 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C14" s="2">
         <v>5</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="E14" s="20"/>
       <c r="F14" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G14" s="2">
         <v>8</v>
@@ -7010,22 +7930,22 @@
     </row>
     <row r="15" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C15" s="2">
         <v>6</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>164</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>168</v>
+        <v>159</v>
+      </c>
+      <c r="F15" s="25" t="s">
+        <v>115</v>
       </c>
       <c r="G15" s="2">
         <v>5</v>
@@ -7037,96 +7957,98 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>26</v>
+        <v>135</v>
       </c>
       <c r="C16" s="2">
         <v>7</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>27</v>
+        <v>136</v>
       </c>
       <c r="E16" s="20"/>
       <c r="F16" s="2" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
       <c r="G16" s="2">
-        <v>5</v>
-      </c>
-      <c r="H16" s="2"/>
+        <v>3</v>
+      </c>
+      <c r="H16" s="2">
+        <v>4</v>
+      </c>
       <c r="J16" s="17"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C17" s="2">
         <v>7</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E17" s="20"/>
       <c r="F17" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G17" s="2">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H17" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J17" s="17"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C18" s="2">
         <v>7</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E18" s="20"/>
       <c r="F18" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G18" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H18" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J18" s="17"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>142</v>
+        <v>47</v>
       </c>
       <c r="C19" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>145</v>
+        <v>48</v>
       </c>
       <c r="E19" s="20"/>
       <c r="F19" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G19" s="2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H19" s="2">
         <v>4</v>
@@ -7135,209 +8057,167 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="C20" s="2">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="E20" s="20"/>
-      <c r="F20" s="2" t="s">
-        <v>120</v>
+      <c r="F20" s="25" t="s">
+        <v>115</v>
       </c>
       <c r="G20" s="2">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H20" s="2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J20" s="17"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C21" s="2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E21" s="20"/>
-      <c r="F21" s="2" t="s">
-        <v>8</v>
+      <c r="F21" s="25" t="s">
+        <v>115</v>
       </c>
       <c r="G21" s="2">
-        <v>3</v>
-      </c>
-      <c r="H21" s="2"/>
+        <v>5</v>
+      </c>
+      <c r="H21" s="2">
+        <v>7</v>
+      </c>
       <c r="J21" s="17"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C22" s="2">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E22" s="20"/>
       <c r="F22" s="2" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
       <c r="G22" s="2">
         <v>5</v>
       </c>
-      <c r="H22" s="2"/>
+      <c r="H22" s="2">
+        <v>5</v>
+      </c>
       <c r="J22" s="17"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>47</v>
+        <v>167</v>
       </c>
       <c r="C23" s="2">
+        <v>6</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E23" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="F23" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="G23" s="2">
+        <v>3</v>
+      </c>
+      <c r="H23" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="C24" s="2">
         <v>13</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E23" s="20"/>
-      <c r="F23" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G23" s="2">
-        <v>5</v>
-      </c>
-      <c r="H23" s="2">
-        <v>5</v>
-      </c>
-      <c r="J23" s="17"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="C24" s="2">
-        <v>14</v>
-      </c>
       <c r="D24" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E24" s="20"/>
+        <v>170</v>
+      </c>
+      <c r="E24" s="20" t="s">
+        <v>171</v>
+      </c>
       <c r="F24" s="2" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
       <c r="G24" s="2">
         <v>3</v>
       </c>
-      <c r="H24" s="2"/>
-      <c r="J24" s="17"/>
-    </row>
-    <row r="25" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+      <c r="H24" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>173</v>
+        <v>56</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>174</v>
+        <v>54</v>
       </c>
       <c r="C25" s="2">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E25" s="20" t="s">
-        <v>175</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="E25" s="20"/>
       <c r="F25" s="2" t="s">
-        <v>168</v>
+        <v>115</v>
       </c>
       <c r="G25" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H25" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>177</v>
-      </c>
-      <c r="C26" s="2">
-        <v>13</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="E26" s="20" t="s">
-        <v>179</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="G26" s="2">
-        <v>3</v>
-      </c>
-      <c r="H26" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="2">
-        <v>15</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E27" s="20"/>
-      <c r="F27" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G27" s="2">
-        <v>5</v>
-      </c>
-      <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="4"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4">
-        <f>SUM(G2:G24)</f>
-        <v>124</v>
-      </c>
-      <c r="H28" s="4"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" s="4"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4">
+        <f>SUM(G2:G22)</f>
+        <v>116</v>
+      </c>
+      <c r="H26" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>